<commit_message>
Repas: fenêtres 11h30-14h et 18h30-21h, au moins 3 personnes en pause ensemble
</commit_message>
<xml_diff>
--- a/Planning_Stunfest2026_Indie.xlsx
+++ b/Planning_Stunfest2026_Indie.xlsx
@@ -989,9 +989,9 @@
           <t>12h00</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="C9" s="8" t="inlineStr">
@@ -999,24 +999,24 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="E9" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="F9" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="G9" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
@@ -1190,19 +1190,19 @@
           <t>Run</t>
         </is>
       </c>
-      <c r="H12" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="I12" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="J12" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="H12" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="J12" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="K12" s="4" t="inlineStr">
@@ -1755,19 +1755,19 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="G22" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="H22" s="10" t="inlineStr">
+      <c r="G22" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="H22" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="I22" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="I22" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
@@ -1787,9 +1787,9 @@
           <t>19h00</t>
         </is>
       </c>
-      <c r="B23" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="B23" s="10" t="inlineStr">
+        <is>
+          <t>Stand IC</t>
         </is>
       </c>
       <c r="C23" s="8" t="inlineStr">
@@ -1797,9 +1797,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="D23" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="E23" s="8" t="inlineStr">
@@ -1812,24 +1812,24 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="G23" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="H23" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="I23" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="J23" s="10" t="inlineStr">
-        <is>
-          <t>Stand IC</t>
+      <c r="G23" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="H23" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="I23" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="J23" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="K23" s="4" t="inlineStr">
@@ -2233,7 +2233,7 @@
     <row r="46">
       <c r="A46" s="23" t="inlineStr">
         <is>
-          <t>Règles : max 2h consécutives sur un même poste (hors Run de préparation du vendredi matin et Standiers fixes pendant les Awards, demandés explicitement) · 30 min de pause déjeuner (12h00 ou 13h30) + 30 min de pause dîner (19h00 ou 20h30) pour chacun·e, à effectif égal (affichées en Off).</t>
+          <t>Règles : max 2h consécutives sur un même poste (hors Run de préparation du vendredi matin et Standiers fixes pendant les Awards, demandés explicitement) · 30 min de pause déjeuner (fenêtre 11h30-14h) + 30 min de pause dîner (fenêtre 18h30-21h) pour chacun·e, au moins 3 personnes en pause en même temps (affichées en Off). Exceptions : Jeff (Run continu) et, le samedi, les 2 Standiers fixes des Awards.</t>
         </is>
       </c>
     </row>
@@ -2673,29 +2673,29 @@
           <t>Standiers</t>
         </is>
       </c>
-      <c r="F8" s="10" t="inlineStr">
+      <c r="F8" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="G8" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="I8" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="J8" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="G8" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="H8" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="I8" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="J8" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
         </is>
       </c>
       <c r="K8" s="4" t="inlineStr">
@@ -2750,14 +2750,14 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="I9" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="J9" s="10" t="inlineStr">
+      <c r="I9" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
+        </is>
+      </c>
+      <c r="J9" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
       <c r="K9" s="4" t="inlineStr">
@@ -2792,14 +2792,14 @@
           <t>Standiers</t>
         </is>
       </c>
-      <c r="E10" s="10" t="inlineStr">
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="F10" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="F10" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
@@ -2849,39 +2849,39 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="E11" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="F11" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="G11" s="10" t="inlineStr">
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="E11" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="H11" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="I11" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="J11" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="J11" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="K11" s="8" t="inlineStr">
@@ -2921,19 +2921,19 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="F12" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="G12" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="H12" s="10" t="inlineStr">
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="G12" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
+        </is>
+      </c>
+      <c r="H12" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
       <c r="I12" s="8" t="inlineStr">
@@ -2973,19 +2973,19 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D13" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="E13" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="F13" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="G13" s="8" t="inlineStr">
@@ -2998,9 +2998,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="I13" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="I13" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="J13" s="9" t="inlineStr">
@@ -3035,9 +3035,9 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D14" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="E14" s="8" t="inlineStr">
@@ -3045,19 +3045,19 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="F14" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="G14" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="H14" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="G14" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="H14" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="I14" s="10" t="inlineStr">
@@ -3087,9 +3087,9 @@
           <t>15h00</t>
         </is>
       </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>Stand IC</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
@@ -3097,24 +3097,24 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D15" s="11" t="inlineStr">
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="F15" s="11" t="inlineStr">
         <is>
           <t>Vote public</t>
         </is>
       </c>
-      <c r="E15" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="F15" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="G15" s="10" t="inlineStr">
-        <is>
-          <t>Stand IC</t>
+      <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="H15" s="8" t="inlineStr">
@@ -3132,9 +3132,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="K15" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="K15" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
       <c r="L15" s="4" t="inlineStr">
@@ -3159,34 +3159,34 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D16" s="10" t="inlineStr">
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="F16" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="E16" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="F16" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="G16" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="H16" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="I16" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="I16" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
       <c r="J16" s="8" t="inlineStr">
@@ -3211,9 +3211,9 @@
           <t>16h00</t>
         </is>
       </c>
-      <c r="B17" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
@@ -3231,9 +3231,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="F17" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="G17" s="8" t="inlineStr">
@@ -3241,19 +3241,19 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="H17" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="I17" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="J17" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="H17" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="I17" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="J17" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
       <c r="K17" s="10" t="inlineStr">
@@ -3273,34 +3273,34 @@
           <t>16h30</t>
         </is>
       </c>
-      <c r="B18" s="10" t="inlineStr">
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="E18" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="D18" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="E18" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
       <c r="F18" s="8" t="inlineStr">
         <is>
           <t>Off</t>
         </is>
       </c>
-      <c r="G18" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="G18" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="H18" s="8" t="inlineStr">
@@ -3308,19 +3308,19 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="I18" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="J18" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="K18" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="I18" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="J18" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="K18" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="L18" s="4" t="inlineStr">
@@ -3335,9 +3335,9 @@
           <t>17h00</t>
         </is>
       </c>
-      <c r="B19" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
@@ -3350,29 +3350,29 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="E19" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="F19" s="10" t="inlineStr">
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="F19" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="G19" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="H19" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="G19" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="H19" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="I19" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="I19" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="J19" s="8" t="inlineStr">
@@ -3380,9 +3380,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="K19" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="K19" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="L19" s="4" t="inlineStr">
@@ -3397,9 +3397,9 @@
           <t>17h30</t>
         </is>
       </c>
-      <c r="B20" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="B20" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
@@ -3407,24 +3407,24 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D20" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="E20" s="10" t="inlineStr">
+      <c r="D20" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="F20" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="G20" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="E20" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="H20" s="8" t="inlineStr">
@@ -3437,9 +3437,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="J20" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="J20" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="K20" s="8" t="inlineStr">
@@ -3479,34 +3479,34 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="F21" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="G21" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="H21" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="I21" s="10" t="inlineStr">
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="G21" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="H21" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="I21" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="J21" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="J21" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="K21" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="K21" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="L21" s="4" t="inlineStr">
@@ -3521,54 +3521,54 @@
           <t>18h30</t>
         </is>
       </c>
-      <c r="B22" s="24" t="inlineStr">
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="E22" s="24" t="inlineStr">
         <is>
           <t>Awards</t>
         </is>
       </c>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="D22" s="24" t="inlineStr">
+      <c r="F22" s="24" t="inlineStr">
         <is>
           <t>Awards</t>
         </is>
       </c>
-      <c r="E22" s="24" t="inlineStr">
+      <c r="G22" s="24" t="inlineStr">
         <is>
           <t>Awards</t>
         </is>
       </c>
-      <c r="F22" s="24" t="inlineStr">
+      <c r="H22" s="24" t="inlineStr">
         <is>
           <t>Awards</t>
         </is>
       </c>
-      <c r="G22" s="24" t="inlineStr">
+      <c r="I22" s="24" t="inlineStr">
         <is>
           <t>Awards</t>
         </is>
       </c>
-      <c r="H22" s="24" t="inlineStr">
+      <c r="J22" s="24" t="inlineStr">
         <is>
           <t>Awards</t>
         </is>
       </c>
-      <c r="I22" s="24" t="inlineStr">
+      <c r="K22" s="24" t="inlineStr">
         <is>
           <t>Awards</t>
-        </is>
-      </c>
-      <c r="J22" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="K22" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
         </is>
       </c>
       <c r="L22" s="24" t="inlineStr">
@@ -3583,54 +3583,54 @@
           <t>19h00</t>
         </is>
       </c>
-      <c r="B23" s="24" t="inlineStr">
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="D23" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="F23" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="G23" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="H23" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="I23" s="24" t="inlineStr">
         <is>
           <t>Awards</t>
         </is>
       </c>
-      <c r="C23" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="D23" s="24" t="inlineStr">
+      <c r="J23" s="24" t="inlineStr">
         <is>
           <t>Awards</t>
         </is>
       </c>
-      <c r="E23" s="24" t="inlineStr">
+      <c r="K23" s="24" t="inlineStr">
         <is>
           <t>Awards</t>
-        </is>
-      </c>
-      <c r="F23" s="24" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="G23" s="24" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="H23" s="24" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="I23" s="24" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="J23" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="K23" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
         </is>
       </c>
       <c r="L23" s="24" t="inlineStr">
@@ -3645,54 +3645,54 @@
           <t>19h30</t>
         </is>
       </c>
-      <c r="B24" s="24" t="inlineStr">
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="D24" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="E24" s="24" t="inlineStr">
         <is>
           <t>Awards</t>
         </is>
       </c>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="D24" s="24" t="inlineStr">
+      <c r="F24" s="24" t="inlineStr">
         <is>
           <t>Awards</t>
         </is>
       </c>
-      <c r="E24" s="24" t="inlineStr">
+      <c r="G24" s="24" t="inlineStr">
         <is>
           <t>Awards</t>
         </is>
       </c>
-      <c r="F24" s="24" t="inlineStr">
+      <c r="H24" s="24" t="inlineStr">
         <is>
           <t>Awards</t>
         </is>
       </c>
-      <c r="G24" s="24" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="H24" s="24" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="I24" s="24" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="J24" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="K24" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="I24" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="J24" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="K24" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="L24" s="24" t="inlineStr">
@@ -3707,54 +3707,54 @@
           <t>20h00</t>
         </is>
       </c>
-      <c r="B25" s="24" t="inlineStr">
+      <c r="B25" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="D25" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="E25" s="24" t="inlineStr">
         <is>
           <t>Awards</t>
         </is>
       </c>
-      <c r="C25" s="5" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="D25" s="24" t="inlineStr">
+      <c r="F25" s="24" t="inlineStr">
         <is>
           <t>Awards</t>
         </is>
       </c>
-      <c r="E25" s="24" t="inlineStr">
+      <c r="G25" s="24" t="inlineStr">
         <is>
           <t>Awards</t>
         </is>
       </c>
-      <c r="F25" s="24" t="inlineStr">
+      <c r="H25" s="24" t="inlineStr">
         <is>
           <t>Awards</t>
         </is>
       </c>
-      <c r="G25" s="24" t="inlineStr">
+      <c r="I25" s="24" t="inlineStr">
         <is>
           <t>Awards</t>
         </is>
       </c>
-      <c r="H25" s="24" t="inlineStr">
+      <c r="J25" s="24" t="inlineStr">
         <is>
           <t>Awards</t>
         </is>
       </c>
-      <c r="I25" s="24" t="inlineStr">
+      <c r="K25" s="24" t="inlineStr">
         <is>
           <t>Awards</t>
-        </is>
-      </c>
-      <c r="J25" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="K25" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
         </is>
       </c>
       <c r="L25" s="24" t="inlineStr">
@@ -3769,54 +3769,54 @@
           <t>20h30</t>
         </is>
       </c>
-      <c r="B26" s="24" t="inlineStr">
+      <c r="B26" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="D26" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="E26" s="24" t="inlineStr">
         <is>
           <t>Awards</t>
         </is>
       </c>
-      <c r="C26" s="5" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="D26" s="24" t="inlineStr">
+      <c r="F26" s="24" t="inlineStr">
         <is>
           <t>Awards</t>
         </is>
       </c>
-      <c r="E26" s="24" t="inlineStr">
+      <c r="G26" s="24" t="inlineStr">
         <is>
           <t>Awards</t>
         </is>
       </c>
-      <c r="F26" s="24" t="inlineStr">
+      <c r="H26" s="24" t="inlineStr">
         <is>
           <t>Awards</t>
         </is>
       </c>
-      <c r="G26" s="24" t="inlineStr">
+      <c r="I26" s="24" t="inlineStr">
         <is>
           <t>Awards</t>
         </is>
       </c>
-      <c r="H26" s="24" t="inlineStr">
+      <c r="J26" s="24" t="inlineStr">
         <is>
           <t>Awards</t>
         </is>
       </c>
-      <c r="I26" s="24" t="inlineStr">
+      <c r="K26" s="24" t="inlineStr">
         <is>
           <t>Awards</t>
-        </is>
-      </c>
-      <c r="J26" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="K26" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
         </is>
       </c>
       <c r="L26" s="24" t="inlineStr">
@@ -4059,7 +4059,7 @@
     <row r="46">
       <c r="A46" s="23" t="inlineStr">
         <is>
-          <t>Règles : max 2h consécutives sur un même poste (hors Run de préparation du vendredi matin et Standiers fixes pendant les Awards, demandés explicitement) · 30 min de pause déjeuner (12h00 ou 13h30) + 30 min de pause dîner (19h00 ou 20h30) pour chacun·e, à effectif égal (affichées en Off).</t>
+          <t>Règles : max 2h consécutives sur un même poste (hors Run de préparation du vendredi matin et Standiers fixes pendant les Awards, demandés explicitement) · 30 min de pause déjeuner (fenêtre 11h30-14h) + 30 min de pause dîner (fenêtre 18h30-21h) pour chacun·e, au moins 3 personnes en pause en même temps (affichées en Off). Exceptions : Jeff (Run continu) et, le samedi, les 2 Standiers fixes des Awards.</t>
         </is>
       </c>
     </row>
@@ -4499,29 +4499,29 @@
           <t>Standiers</t>
         </is>
       </c>
-      <c r="F8" s="10" t="inlineStr">
+      <c r="F8" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="G8" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="I8" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="J8" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="G8" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="H8" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="I8" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="J8" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
         </is>
       </c>
       <c r="K8" s="4" t="inlineStr">
@@ -4576,14 +4576,14 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="I9" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="J9" s="10" t="inlineStr">
+      <c r="I9" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
+        </is>
+      </c>
+      <c r="J9" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
       <c r="K9" s="4" t="inlineStr">
@@ -4618,14 +4618,14 @@
           <t>Standiers</t>
         </is>
       </c>
-      <c r="E10" s="10" t="inlineStr">
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="F10" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="F10" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
@@ -4675,39 +4675,39 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="E11" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="F11" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="G11" s="10" t="inlineStr">
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="E11" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="H11" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="I11" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="J11" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="J11" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="K11" s="8" t="inlineStr">
@@ -4747,19 +4747,19 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="F12" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="G12" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="H12" s="10" t="inlineStr">
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="G12" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
+        </is>
+      </c>
+      <c r="H12" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
       <c r="I12" s="8" t="inlineStr">
@@ -4799,19 +4799,19 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D13" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="E13" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="F13" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="G13" s="8" t="inlineStr">
@@ -4824,9 +4824,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="I13" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="I13" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="J13" s="9" t="inlineStr">
@@ -4861,9 +4861,9 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D14" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="E14" s="8" t="inlineStr">
@@ -4871,19 +4871,19 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="F14" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="G14" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="H14" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="G14" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="H14" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="I14" s="10" t="inlineStr">
@@ -4913,9 +4913,9 @@
           <t>15h00</t>
         </is>
       </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>Stand IC</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
@@ -4923,24 +4923,24 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D15" s="11" t="inlineStr">
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="F15" s="11" t="inlineStr">
         <is>
           <t>Vote public</t>
         </is>
       </c>
-      <c r="E15" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="F15" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="G15" s="10" t="inlineStr">
-        <is>
-          <t>Stand IC</t>
+      <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="H15" s="8" t="inlineStr">
@@ -4958,9 +4958,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="K15" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="K15" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
       <c r="L15" s="4" t="inlineStr">
@@ -4985,34 +4985,34 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D16" s="10" t="inlineStr">
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="F16" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="E16" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="F16" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="G16" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="H16" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="I16" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="I16" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
       <c r="J16" s="8" t="inlineStr">
@@ -5037,9 +5037,9 @@
           <t>16h00</t>
         </is>
       </c>
-      <c r="B17" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
@@ -5057,9 +5057,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="F17" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="G17" s="8" t="inlineStr">
@@ -5067,19 +5067,19 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="H17" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="I17" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="J17" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="H17" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="I17" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="J17" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
       <c r="K17" s="10" t="inlineStr">
@@ -5099,34 +5099,34 @@
           <t>16h30</t>
         </is>
       </c>
-      <c r="B18" s="10" t="inlineStr">
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="E18" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="D18" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="E18" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
       <c r="F18" s="8" t="inlineStr">
         <is>
           <t>Off</t>
         </is>
       </c>
-      <c r="G18" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="G18" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="H18" s="8" t="inlineStr">
@@ -5134,19 +5134,19 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="I18" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="J18" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="K18" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="I18" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="J18" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="K18" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="L18" s="4" t="inlineStr">
@@ -5161,9 +5161,9 @@
           <t>17h00</t>
         </is>
       </c>
-      <c r="B19" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
@@ -5176,29 +5176,29 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="E19" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="F19" s="10" t="inlineStr">
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="F19" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="G19" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="H19" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="G19" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="H19" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="I19" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="I19" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="J19" s="8" t="inlineStr">
@@ -5206,9 +5206,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="K19" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="K19" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="L19" s="4" t="inlineStr">
@@ -5223,9 +5223,9 @@
           <t>17h30</t>
         </is>
       </c>
-      <c r="B20" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="B20" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
@@ -5233,24 +5233,24 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D20" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="E20" s="10" t="inlineStr">
+      <c r="D20" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="F20" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="G20" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="E20" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="H20" s="8" t="inlineStr">
@@ -5263,9 +5263,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="J20" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="J20" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="K20" s="8" t="inlineStr">
@@ -5305,34 +5305,34 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="F21" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="G21" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="H21" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="I21" s="10" t="inlineStr">
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="G21" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="H21" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="I21" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="J21" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="J21" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="K21" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="K21" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="L21" s="4" t="inlineStr">
@@ -5362,14 +5362,14 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="E22" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="F22" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="E22" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="F22" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="G22" s="8" t="inlineStr">
@@ -5382,19 +5382,19 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="I22" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="J22" s="10" t="inlineStr">
+      <c r="I22" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="J22" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="K22" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="K22" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
         </is>
       </c>
       <c r="L22" s="4" t="inlineStr">
@@ -5409,9 +5409,9 @@
           <t>19h00</t>
         </is>
       </c>
-      <c r="B23" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
       <c r="C23" s="8" t="inlineStr">
@@ -5419,9 +5419,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="D23" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="E23" s="8" t="inlineStr">
@@ -5434,9 +5434,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="G23" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="G23" s="10" t="inlineStr">
+        <is>
+          <t>Stand IC</t>
         </is>
       </c>
       <c r="H23" s="8" t="inlineStr">
@@ -5444,19 +5444,19 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="I23" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="J23" s="10" t="inlineStr">
-        <is>
-          <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="K23" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="I23" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="J23" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="K23" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="L23" s="4" t="inlineStr">
@@ -5878,7 +5878,7 @@
     <row r="45">
       <c r="A45" s="23" t="inlineStr">
         <is>
-          <t>Règles : max 2h consécutives sur un même poste (hors Run de préparation du vendredi matin et Standiers fixes pendant les Awards, demandés explicitement) · 30 min de pause déjeuner (12h00 ou 13h30) + 30 min de pause dîner (19h00 ou 20h30) pour chacun·e, à effectif égal (affichées en Off).</t>
+          <t>Règles : max 2h consécutives sur un même poste (hors Run de préparation du vendredi matin et Standiers fixes pendant les Awards, demandés explicitement) · 30 min de pause déjeuner (fenêtre 11h30-14h) + 30 min de pause dîner (fenêtre 18h30-21h) pour chacun·e, au moins 3 personnes en pause en même temps (affichées en Off). Exceptions : Jeff (Run continu) et, le samedi, les 2 Standiers fixes des Awards.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Suppression du rôle Vote public (intégré au Run)
</commit_message>
<xml_diff>
--- a/Planning_Stunfest2026_Indie.xlsx
+++ b/Planning_Stunfest2026_Indie.xlsx
@@ -64,7 +64,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="12">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -111,11 +111,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="006A1B9A"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00B71C1C"/>
       </patternFill>
     </fill>
@@ -146,7 +141,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -178,22 +173,18 @@
     <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -561,7 +552,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K46"/>
+  <dimension ref="A1:K45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1346,9 +1337,9 @@
           <t>Standiers</t>
         </is>
       </c>
-      <c r="E15" s="11" t="inlineStr">
-        <is>
-          <t>Vote public</t>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="F15" s="8" t="inlineStr">
@@ -2124,114 +2115,106 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="12" t="inlineStr">
+      <c r="A31" s="11" t="inlineStr">
         <is>
           <t>Légende</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="13" t="inlineStr"/>
-      <c r="B32" s="14" t="inlineStr">
+      <c r="A32" s="12" t="inlineStr"/>
+      <c r="B32" s="13" t="inlineStr">
         <is>
           <t>Standiers = Back-up standiers Indie</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="15" t="inlineStr"/>
-      <c r="B33" s="14" t="inlineStr">
-        <is>
-          <t>Run = IC volant / Run</t>
+      <c r="A33" s="14" t="inlineStr"/>
+      <c r="B33" s="13" t="inlineStr">
+        <is>
+          <t>Run = IC volant / Run (inclut le vote du public et le check des stands)</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="16" t="inlineStr"/>
-      <c r="B34" s="14" t="inlineStr">
+      <c r="A34" s="15" t="inlineStr"/>
+      <c r="B34" s="13" t="inlineStr">
         <is>
           <t>Stand IC = Stand IC / Stunjam</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="17" t="inlineStr"/>
-      <c r="B35" s="14" t="inlineStr">
-        <is>
-          <t>Vote public = Vote du public</t>
+      <c r="A35" s="16" t="inlineStr"/>
+      <c r="B35" s="13" t="inlineStr">
+        <is>
+          <t>Awards = Indie Awards (18h30-20h30, samedi) ; 2 personnes fixes restent en Standiers</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="18" t="inlineStr"/>
-      <c r="B36" s="14" t="inlineStr">
-        <is>
-          <t>Awards = Indie Awards (18h30-20h30, samedi) ; 2 personnes fixes restent en Standiers</t>
+      <c r="A36" s="17" t="inlineStr"/>
+      <c r="B36" s="13" t="inlineStr">
+        <is>
+          <t>Média = Captation média (Chris, en continu les 3 jours)</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="19" t="inlineStr"/>
-      <c r="B37" s="14" t="inlineStr">
-        <is>
-          <t>Média = Captation média (Chris, en continu les 3 jours)</t>
+      <c r="A37" s="18" t="inlineStr"/>
+      <c r="B37" s="13" t="inlineStr">
+        <is>
+          <t>Briefing = Briefing d'équipe (vendredi 10h00-10h30)</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="20" t="inlineStr"/>
-      <c r="B38" s="14" t="inlineStr">
-        <is>
-          <t>Briefing = Briefing d'équipe (vendredi 10h00-10h30)</t>
+      <c r="A38" s="19" t="inlineStr"/>
+      <c r="B38" s="13" t="inlineStr">
+        <is>
+          <t>Off (inclut les 30 min de pause déjeuner + 30 min de pause dîner)</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="21" t="inlineStr"/>
-      <c r="B39" s="14" t="inlineStr">
-        <is>
-          <t>Off (inclut les 30 min de pause déjeuner + 30 min de pause dîner)</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="22" t="inlineStr"/>
-      <c r="B40" s="14" t="inlineStr">
+      <c r="A39" s="20" t="inlineStr"/>
+      <c r="B39" s="13" t="inlineStr">
         <is>
           <t>— = pas encore arrivé / absent ce jour-là</t>
         </is>
       </c>
     </row>
+    <row r="41">
+      <c r="A41" s="21" t="inlineStr">
+        <is>
+          <t>FERMETURE DE LA ZONE INDÉ À 19h30 TOUS LES SOIRS.</t>
+        </is>
+      </c>
+    </row>
     <row r="42">
-      <c r="A42" s="23" t="inlineStr">
-        <is>
-          <t>FERMETURE DE LA ZONE INDÉ À 19h30 TOUS LES SOIRS.</t>
+      <c r="A42" s="21" t="inlineStr">
+        <is>
+          <t>Ouverture au public à 14h. Bénévoles présents dès 9h pour la préparation : tout le monde en Run de 9h à 14h.</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="23" t="inlineStr">
-        <is>
-          <t>Ouverture au public à 14h. Bénévoles présents dès 9h pour la préparation : tout le monde en Run de 9h à 14h.</t>
+      <c r="A43" s="21" t="inlineStr">
+        <is>
+          <t>Briefing d'équipe 10h00-10h30 (Jeff arrive à 11h).</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="23" t="inlineStr">
-        <is>
-          <t>Briefing d'équipe 10h00-10h30 (Jeff arrive à 11h).</t>
+      <c r="A44" s="21" t="inlineStr">
+        <is>
+          <t>Robin : présent uniquement samedi et dimanche. Jeff : présent les 3 jours de 11h à 22h, en Run continu. Chris : captation Média en continu.</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="23" t="inlineStr">
-        <is>
-          <t>Robin : présent uniquement samedi et dimanche. Jeff : présent les 3 jours de 11h à 22h, en Run continu. Chris : captation Média en continu.</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="23" t="inlineStr">
+      <c r="A45" s="21" t="inlineStr">
         <is>
           <t>Règles : max 2h consécutives sur un même poste (hors Run de préparation du vendredi matin et Standiers fixes pendant les Awards, demandés explicitement) · 30 min de pause déjeuner (fenêtre 11h30-14h) + 30 min de pause dîner (fenêtre 18h30-21h) pour chacun·e, au moins 3 personnes en pause en même temps (affichées en Off). Exceptions : Jeff (Run continu) et, le samedi, les 2 Standiers fixes des Awards.</t>
         </is>
@@ -2246,1832 +2229,6 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:L46"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
-    <col width="11" customWidth="1" min="10" max="10"/>
-    <col width="11" customWidth="1" min="11" max="11"/>
-    <col width="11" customWidth="1" min="12" max="12"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>STUNFEST 2026 — Planning bénévolat Indé — Samedi 24 octobre</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Horaire</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>François</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Chris</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Étienne</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Florent</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Arthur</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>Mael</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>Gabriel</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>Lylou</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>Suliac</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>Robin</t>
-        </is>
-      </c>
-      <c r="L2" s="2" t="inlineStr">
-        <is>
-          <t>Jeff</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="14" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>9h00</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="G3" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="H3" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="I3" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="J3" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="K3" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="L3" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="14" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>9h30</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="G4" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="H4" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="I4" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="J4" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="K4" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="L4" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="14" customHeight="1">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>10h00</t>
-        </is>
-      </c>
-      <c r="B5" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="D5" s="10" t="inlineStr">
-        <is>
-          <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="G5" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="H5" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="I5" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="J5" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="K5" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="L5" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="14" customHeight="1">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>10h30</t>
-        </is>
-      </c>
-      <c r="B6" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="D6" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="E6" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="F6" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="G6" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="H6" s="10" t="inlineStr">
-        <is>
-          <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="I6" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="J6" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="K6" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="L6" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="14" customHeight="1">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>11h00</t>
-        </is>
-      </c>
-      <c r="B7" s="10" t="inlineStr">
-        <is>
-          <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="E7" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="F7" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="G7" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="H7" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="I7" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="J7" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="K7" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="L7" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="14" customHeight="1">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>11h30</t>
-        </is>
-      </c>
-      <c r="B8" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="D8" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="E8" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="F8" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="G8" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="H8" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="I8" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="J8" s="10" t="inlineStr">
-        <is>
-          <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="K8" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="L8" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="14" customHeight="1">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>12h00</t>
-        </is>
-      </c>
-      <c r="B9" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="C9" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="D9" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="E9" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="F9" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="G9" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="H9" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="I9" s="10" t="inlineStr">
-        <is>
-          <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="J9" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="K9" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="L9" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="14" customHeight="1">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>12h30</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="D10" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="E10" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="F10" s="10" t="inlineStr">
-        <is>
-          <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="G10" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="H10" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="I10" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="J10" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="K10" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="L10" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="14" customHeight="1">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>13h00</t>
-        </is>
-      </c>
-      <c r="B11" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="D11" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="E11" s="10" t="inlineStr">
-        <is>
-          <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="F11" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="G11" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="H11" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="I11" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="J11" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="K11" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="L11" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="14" customHeight="1">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>13h30</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="D12" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="E12" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="F12" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="G12" s="10" t="inlineStr">
-        <is>
-          <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="H12" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="I12" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="J12" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="K12" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="L12" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="14" customHeight="1">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>14h00</t>
-        </is>
-      </c>
-      <c r="B13" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="D13" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="E13" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="F13" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="G13" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="H13" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="I13" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="J13" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="K13" s="10" t="inlineStr">
-        <is>
-          <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="L13" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="14" customHeight="1">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>14h30</t>
-        </is>
-      </c>
-      <c r="B14" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="D14" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="E14" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="F14" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="G14" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="H14" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="I14" s="10" t="inlineStr">
-        <is>
-          <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="J14" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="K14" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="L14" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="14" customHeight="1">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>15h00</t>
-        </is>
-      </c>
-      <c r="B15" s="10" t="inlineStr">
-        <is>
-          <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="D15" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="E15" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="F15" s="11" t="inlineStr">
-        <is>
-          <t>Vote public</t>
-        </is>
-      </c>
-      <c r="G15" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="H15" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="I15" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="J15" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="K15" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="L15" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="14" customHeight="1">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>15h30</t>
-        </is>
-      </c>
-      <c r="B16" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="D16" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="E16" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="F16" s="10" t="inlineStr">
-        <is>
-          <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="G16" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="H16" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="I16" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="J16" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="K16" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="L16" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="14" customHeight="1">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>16h00</t>
-        </is>
-      </c>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="D17" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="E17" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="F17" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="G17" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="H17" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="I17" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="J17" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="K17" s="10" t="inlineStr">
-        <is>
-          <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="L17" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="14" customHeight="1">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>16h30</t>
-        </is>
-      </c>
-      <c r="B18" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="D18" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="E18" s="10" t="inlineStr">
-        <is>
-          <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="F18" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="G18" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="H18" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="I18" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="J18" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="K18" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="L18" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="14" customHeight="1">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>17h00</t>
-        </is>
-      </c>
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="D19" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="E19" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="F19" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="G19" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="H19" s="10" t="inlineStr">
-        <is>
-          <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="I19" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="J19" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="K19" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="L19" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="14" customHeight="1">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t>17h30</t>
-        </is>
-      </c>
-      <c r="B20" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="C20" s="5" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="D20" s="10" t="inlineStr">
-        <is>
-          <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="E20" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="F20" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="G20" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="H20" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="I20" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="J20" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="K20" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="L20" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="14" customHeight="1">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>18h00</t>
-        </is>
-      </c>
-      <c r="B21" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="C21" s="5" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="D21" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="E21" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="F21" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="G21" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="H21" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="I21" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="J21" s="10" t="inlineStr">
-        <is>
-          <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="K21" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="L21" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="14" customHeight="1">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t>18h30</t>
-        </is>
-      </c>
-      <c r="B22" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="D22" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="E22" s="24" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="F22" s="24" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="G22" s="24" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="H22" s="24" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="I22" s="24" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="J22" s="24" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="K22" s="24" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="L22" s="24" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="14" customHeight="1">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t>19h00</t>
-        </is>
-      </c>
-      <c r="B23" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="C23" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="D23" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="E23" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="F23" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="G23" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="H23" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="I23" s="24" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="J23" s="24" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="K23" s="24" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="L23" s="24" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="14" customHeight="1">
-      <c r="A24" s="3" t="inlineStr">
-        <is>
-          <t>19h30</t>
-        </is>
-      </c>
-      <c r="B24" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="D24" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="E24" s="24" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="F24" s="24" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="G24" s="24" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="H24" s="24" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="I24" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="J24" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="K24" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="L24" s="24" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="14" customHeight="1">
-      <c r="A25" s="3" t="inlineStr">
-        <is>
-          <t>20h00</t>
-        </is>
-      </c>
-      <c r="B25" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="C25" s="5" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="D25" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="E25" s="24" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="F25" s="24" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="G25" s="24" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="H25" s="24" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="I25" s="24" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="J25" s="24" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="K25" s="24" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="L25" s="24" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="14" customHeight="1">
-      <c r="A26" s="3" t="inlineStr">
-        <is>
-          <t>20h30</t>
-        </is>
-      </c>
-      <c r="B26" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="C26" s="5" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="D26" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="E26" s="24" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="F26" s="24" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="G26" s="24" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="H26" s="24" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="I26" s="24" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="J26" s="24" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="K26" s="24" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="L26" s="24" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="14" customHeight="1">
-      <c r="A27" s="3" t="inlineStr">
-        <is>
-          <t>21h00</t>
-        </is>
-      </c>
-      <c r="B27" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C27" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D27" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E27" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F27" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G27" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H27" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I27" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J27" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K27" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L27" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="14" customHeight="1">
-      <c r="A28" s="3" t="inlineStr">
-        <is>
-          <t>21h30</t>
-        </is>
-      </c>
-      <c r="B28" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C28" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D28" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E28" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F28" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G28" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H28" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I28" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J28" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K28" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L28" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="12" t="inlineStr">
-        <is>
-          <t>Légende</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="13" t="inlineStr"/>
-      <c r="B32" s="14" t="inlineStr">
-        <is>
-          <t>Standiers = Back-up standiers Indie</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="15" t="inlineStr"/>
-      <c r="B33" s="14" t="inlineStr">
-        <is>
-          <t>Run = IC volant / Run</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="16" t="inlineStr"/>
-      <c r="B34" s="14" t="inlineStr">
-        <is>
-          <t>Stand IC = Stand IC / Stunjam</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="17" t="inlineStr"/>
-      <c r="B35" s="14" t="inlineStr">
-        <is>
-          <t>Vote public = Vote du public</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="18" t="inlineStr"/>
-      <c r="B36" s="14" t="inlineStr">
-        <is>
-          <t>Awards = Indie Awards (18h30-20h30, samedi) ; 2 personnes fixes restent en Standiers</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="19" t="inlineStr"/>
-      <c r="B37" s="14" t="inlineStr">
-        <is>
-          <t>Média = Captation média (Chris, en continu les 3 jours)</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="20" t="inlineStr"/>
-      <c r="B38" s="14" t="inlineStr">
-        <is>
-          <t>Briefing = Briefing d'équipe (vendredi 10h00-10h30)</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="21" t="inlineStr"/>
-      <c r="B39" s="14" t="inlineStr">
-        <is>
-          <t>Off (inclut les 30 min de pause déjeuner + 30 min de pause dîner)</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="22" t="inlineStr"/>
-      <c r="B40" s="14" t="inlineStr">
-        <is>
-          <t>— = pas encore arrivé / absent ce jour-là</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="23" t="inlineStr">
-        <is>
-          <t>FERMETURE DE LA ZONE INDÉ À 19h30 TOUS LES SOIRS.</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="23" t="inlineStr">
-        <is>
-          <t>Ouverture au public à 10h. Bénévoles présents dès 9h pour la préparation : tout le monde en Run de 9h à 10h.</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="23" t="inlineStr">
-        <is>
-          <t>Robin : présent uniquement samedi et dimanche. Jeff : présent les 3 jours de 11h à 22h, en Run continu. Chris : captation Média en continu.</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="23" t="inlineStr">
-        <is>
-          <t>Indie Awards 18h30-20h30 : 2 personnes restent fixes sur l'accueil Standiers (sans rotation), le reste de l'équipe (y compris Jeff dès 18h30) est sur Awards ; Chris reste en Média. Le planning de l'équipe va jusqu'à 21h le samedi pour afficher les Awards en entier (Jeff jusqu'à 22h).</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="23" t="inlineStr">
-        <is>
-          <t>Règles : max 2h consécutives sur un même poste (hors Run de préparation du vendredi matin et Standiers fixes pendant les Awards, demandés explicitement) · 30 min de pause déjeuner (fenêtre 11h30-14h) + 30 min de pause dîner (fenêtre 18h30-21h) pour chacun·e, au moins 3 personnes en pause en même temps (affichées en Off). Exceptions : Jeff (Run continu) et, le samedi, les 2 Standiers fixes des Awards.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:L1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4097,7 +2254,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>STUNFEST 2026 — Planning bénévolat Indé — Dimanche 25 octobre</t>
+          <t>STUNFEST 2026 — Planning bénévolat Indé — Samedi 24 octobre</t>
         </is>
       </c>
     </row>
@@ -4933,9 +3090,9 @@
           <t>Run</t>
         </is>
       </c>
-      <c r="F15" s="11" t="inlineStr">
-        <is>
-          <t>Vote public</t>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="G15" s="8" t="inlineStr">
@@ -5347,9 +3504,9 @@
           <t>18h30</t>
         </is>
       </c>
-      <c r="B22" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
@@ -5357,49 +3514,49 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D22" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="E22" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="F22" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="G22" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="H22" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="I22" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="J22" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="K22" s="10" t="inlineStr">
-        <is>
-          <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="L22" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="E22" s="22" t="inlineStr">
+        <is>
+          <t>Awards</t>
+        </is>
+      </c>
+      <c r="F22" s="22" t="inlineStr">
+        <is>
+          <t>Awards</t>
+        </is>
+      </c>
+      <c r="G22" s="22" t="inlineStr">
+        <is>
+          <t>Awards</t>
+        </is>
+      </c>
+      <c r="H22" s="22" t="inlineStr">
+        <is>
+          <t>Awards</t>
+        </is>
+      </c>
+      <c r="I22" s="22" t="inlineStr">
+        <is>
+          <t>Awards</t>
+        </is>
+      </c>
+      <c r="J22" s="22" t="inlineStr">
+        <is>
+          <t>Awards</t>
+        </is>
+      </c>
+      <c r="K22" s="22" t="inlineStr">
+        <is>
+          <t>Awards</t>
+        </is>
+      </c>
+      <c r="L22" s="22" t="inlineStr">
+        <is>
+          <t>Awards</t>
         </is>
       </c>
     </row>
@@ -5419,9 +3576,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="D23" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="D23" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
       <c r="E23" s="8" t="inlineStr">
@@ -5434,9 +3591,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="G23" s="10" t="inlineStr">
-        <is>
-          <t>Stand IC</t>
+      <c r="G23" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="H23" s="8" t="inlineStr">
@@ -5444,24 +3601,24 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="I23" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="J23" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="K23" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="L23" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="I23" s="22" t="inlineStr">
+        <is>
+          <t>Awards</t>
+        </is>
+      </c>
+      <c r="J23" s="22" t="inlineStr">
+        <is>
+          <t>Awards</t>
+        </is>
+      </c>
+      <c r="K23" s="22" t="inlineStr">
+        <is>
+          <t>Awards</t>
+        </is>
+      </c>
+      <c r="L23" s="22" t="inlineStr">
+        <is>
+          <t>Awards</t>
         </is>
       </c>
     </row>
@@ -5471,59 +3628,59 @@
           <t>19h30</t>
         </is>
       </c>
-      <c r="B24" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C24" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D24" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E24" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F24" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G24" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H24" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I24" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J24" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K24" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L24" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="D24" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="E24" s="22" t="inlineStr">
+        <is>
+          <t>Awards</t>
+        </is>
+      </c>
+      <c r="F24" s="22" t="inlineStr">
+        <is>
+          <t>Awards</t>
+        </is>
+      </c>
+      <c r="G24" s="22" t="inlineStr">
+        <is>
+          <t>Awards</t>
+        </is>
+      </c>
+      <c r="H24" s="22" t="inlineStr">
+        <is>
+          <t>Awards</t>
+        </is>
+      </c>
+      <c r="I24" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="J24" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="K24" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="L24" s="22" t="inlineStr">
+        <is>
+          <t>Awards</t>
         </is>
       </c>
     </row>
@@ -5533,59 +3690,59 @@
           <t>20h00</t>
         </is>
       </c>
-      <c r="B25" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C25" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D25" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E25" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F25" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G25" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H25" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I25" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J25" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K25" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L25" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="B25" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="D25" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="E25" s="22" t="inlineStr">
+        <is>
+          <t>Awards</t>
+        </is>
+      </c>
+      <c r="F25" s="22" t="inlineStr">
+        <is>
+          <t>Awards</t>
+        </is>
+      </c>
+      <c r="G25" s="22" t="inlineStr">
+        <is>
+          <t>Awards</t>
+        </is>
+      </c>
+      <c r="H25" s="22" t="inlineStr">
+        <is>
+          <t>Awards</t>
+        </is>
+      </c>
+      <c r="I25" s="22" t="inlineStr">
+        <is>
+          <t>Awards</t>
+        </is>
+      </c>
+      <c r="J25" s="22" t="inlineStr">
+        <is>
+          <t>Awards</t>
+        </is>
+      </c>
+      <c r="K25" s="22" t="inlineStr">
+        <is>
+          <t>Awards</t>
+        </is>
+      </c>
+      <c r="L25" s="22" t="inlineStr">
+        <is>
+          <t>Awards</t>
         </is>
       </c>
     </row>
@@ -5595,59 +3752,59 @@
           <t>20h30</t>
         </is>
       </c>
-      <c r="B26" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C26" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D26" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E26" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F26" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G26" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H26" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I26" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J26" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K26" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L26" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="B26" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="D26" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="E26" s="22" t="inlineStr">
+        <is>
+          <t>Awards</t>
+        </is>
+      </c>
+      <c r="F26" s="22" t="inlineStr">
+        <is>
+          <t>Awards</t>
+        </is>
+      </c>
+      <c r="G26" s="22" t="inlineStr">
+        <is>
+          <t>Awards</t>
+        </is>
+      </c>
+      <c r="H26" s="22" t="inlineStr">
+        <is>
+          <t>Awards</t>
+        </is>
+      </c>
+      <c r="I26" s="22" t="inlineStr">
+        <is>
+          <t>Awards</t>
+        </is>
+      </c>
+      <c r="J26" s="22" t="inlineStr">
+        <is>
+          <t>Awards</t>
+        </is>
+      </c>
+      <c r="K26" s="22" t="inlineStr">
+        <is>
+          <t>Awards</t>
+        </is>
+      </c>
+      <c r="L26" s="22" t="inlineStr">
+        <is>
+          <t>Awards</t>
         </is>
       </c>
     </row>
@@ -5776,107 +3933,1917 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="12" t="inlineStr">
+      <c r="A31" s="11" t="inlineStr">
         <is>
           <t>Légende</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="13" t="inlineStr"/>
-      <c r="B32" s="14" t="inlineStr">
+      <c r="A32" s="12" t="inlineStr"/>
+      <c r="B32" s="13" t="inlineStr">
         <is>
           <t>Standiers = Back-up standiers Indie</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="15" t="inlineStr"/>
-      <c r="B33" s="14" t="inlineStr">
-        <is>
-          <t>Run = IC volant / Run</t>
+      <c r="A33" s="14" t="inlineStr"/>
+      <c r="B33" s="13" t="inlineStr">
+        <is>
+          <t>Run = IC volant / Run (inclut le vote du public et le check des stands)</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="16" t="inlineStr"/>
-      <c r="B34" s="14" t="inlineStr">
+      <c r="A34" s="15" t="inlineStr"/>
+      <c r="B34" s="13" t="inlineStr">
         <is>
           <t>Stand IC = Stand IC / Stunjam</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="17" t="inlineStr"/>
-      <c r="B35" s="14" t="inlineStr">
-        <is>
-          <t>Vote public = Vote du public</t>
+      <c r="A35" s="16" t="inlineStr"/>
+      <c r="B35" s="13" t="inlineStr">
+        <is>
+          <t>Awards = Indie Awards (18h30-20h30, samedi) ; 2 personnes fixes restent en Standiers</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="18" t="inlineStr"/>
-      <c r="B36" s="14" t="inlineStr">
+      <c r="A36" s="17" t="inlineStr"/>
+      <c r="B36" s="13" t="inlineStr">
+        <is>
+          <t>Média = Captation média (Chris, en continu les 3 jours)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="18" t="inlineStr"/>
+      <c r="B37" s="13" t="inlineStr">
+        <is>
+          <t>Briefing = Briefing d'équipe (vendredi 10h00-10h30)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="19" t="inlineStr"/>
+      <c r="B38" s="13" t="inlineStr">
+        <is>
+          <t>Off (inclut les 30 min de pause déjeuner + 30 min de pause dîner)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="20" t="inlineStr"/>
+      <c r="B39" s="13" t="inlineStr">
+        <is>
+          <t>— = pas encore arrivé / absent ce jour-là</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="21" t="inlineStr">
+        <is>
+          <t>FERMETURE DE LA ZONE INDÉ À 19h30 TOUS LES SOIRS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="21" t="inlineStr">
+        <is>
+          <t>Ouverture au public à 10h. Bénévoles présents dès 9h pour la préparation : tout le monde en Run de 9h à 10h.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="21" t="inlineStr">
+        <is>
+          <t>Robin : présent uniquement samedi et dimanche. Jeff : présent les 3 jours de 11h à 22h, en Run continu. Chris : captation Média en continu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="21" t="inlineStr">
+        <is>
+          <t>Indie Awards 18h30-20h30 : 2 personnes restent fixes sur l'accueil Standiers (sans rotation), le reste de l'équipe (y compris Jeff dès 18h30) est sur Awards ; Chris reste en Média. Le planning de l'équipe va jusqu'à 21h le samedi pour afficher les Awards en entier (Jeff jusqu'à 22h).</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="21" t="inlineStr">
+        <is>
+          <t>Règles : max 2h consécutives sur un même poste (hors Run de préparation du vendredi matin et Standiers fixes pendant les Awards, demandés explicitement) · 30 min de pause déjeuner (fenêtre 11h30-14h) + 30 min de pause dîner (fenêtre 18h30-21h) pour chacun·e, au moins 3 personnes en pause en même temps (affichées en Off). Exceptions : Jeff (Run continu) et, le samedi, les 2 Standiers fixes des Awards.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:L1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L44"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>STUNFEST 2026 — Planning bénévolat Indé — Dimanche 25 octobre</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Horaire</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>François</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Chris</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Étienne</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Florent</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Arthur</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Mael</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Gabriel</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Lylou</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Suliac</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Robin</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>Jeff</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="14" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>9h00</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="I3" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="J3" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="K3" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="L3" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="14" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>9h30</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="K4" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="L4" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="14" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>10h00</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>Stand IC</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="G5" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="H5" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="I5" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="J5" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="K5" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="L5" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="14" customHeight="1">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>10h30</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="G6" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="H6" s="10" t="inlineStr">
+        <is>
+          <t>Stand IC</t>
+        </is>
+      </c>
+      <c r="I6" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="J6" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="K6" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="L6" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="14" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>11h00</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>Stand IC</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="H7" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="I7" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="J7" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="K7" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="L7" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="14" customHeight="1">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>11h30</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="F8" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="G8" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="I8" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="J8" s="10" t="inlineStr">
+        <is>
+          <t>Stand IC</t>
+        </is>
+      </c>
+      <c r="K8" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="L8" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="14" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>12h00</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="H9" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="I9" s="10" t="inlineStr">
+        <is>
+          <t>Stand IC</t>
+        </is>
+      </c>
+      <c r="J9" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="K9" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="L9" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="14" customHeight="1">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>12h30</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="F10" s="10" t="inlineStr">
+        <is>
+          <t>Stand IC</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="H10" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="J10" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="K10" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="L10" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="14" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>13h00</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="E11" s="10" t="inlineStr">
+        <is>
+          <t>Stand IC</t>
+        </is>
+      </c>
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="J11" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="K11" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="L11" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="14" customHeight="1">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>13h30</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="G12" s="10" t="inlineStr">
+        <is>
+          <t>Stand IC</t>
+        </is>
+      </c>
+      <c r="H12" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="J12" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="K12" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="L12" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="14" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>14h00</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="G13" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="H13" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="I13" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="J13" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="K13" s="10" t="inlineStr">
+        <is>
+          <t>Stand IC</t>
+        </is>
+      </c>
+      <c r="L13" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="14" customHeight="1">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>14h30</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="G14" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="H14" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="I14" s="10" t="inlineStr">
+        <is>
+          <t>Stand IC</t>
+        </is>
+      </c>
+      <c r="J14" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="K14" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="L14" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="14" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>15h00</t>
+        </is>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>Stand IC</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="H15" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="I15" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="J15" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="K15" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="L15" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="14" customHeight="1">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>15h30</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="F16" s="10" t="inlineStr">
+        <is>
+          <t>Stand IC</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="I16" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="J16" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="K16" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="L16" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="14" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>16h00</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="G17" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="H17" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="I17" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="J17" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="K17" s="10" t="inlineStr">
+        <is>
+          <t>Stand IC</t>
+        </is>
+      </c>
+      <c r="L17" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="14" customHeight="1">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>16h30</t>
+        </is>
+      </c>
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="E18" s="10" t="inlineStr">
+        <is>
+          <t>Stand IC</t>
+        </is>
+      </c>
+      <c r="F18" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="G18" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="H18" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="I18" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="J18" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="K18" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="L18" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="14" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>17h00</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="F19" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="G19" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="H19" s="10" t="inlineStr">
+        <is>
+          <t>Stand IC</t>
+        </is>
+      </c>
+      <c r="I19" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="J19" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="K19" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="L19" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="14" customHeight="1">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>17h30</t>
+        </is>
+      </c>
+      <c r="B20" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="D20" s="10" t="inlineStr">
+        <is>
+          <t>Stand IC</t>
+        </is>
+      </c>
+      <c r="E20" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="H20" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="I20" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="J20" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="K20" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="L20" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="14" customHeight="1">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>18h00</t>
+        </is>
+      </c>
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="G21" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="H21" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="I21" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="J21" s="10" t="inlineStr">
+        <is>
+          <t>Stand IC</t>
+        </is>
+      </c>
+      <c r="K21" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="L21" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="14" customHeight="1">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>18h30</t>
+        </is>
+      </c>
+      <c r="B22" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="F22" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="G22" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="H22" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="I22" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="J22" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="K22" s="10" t="inlineStr">
+        <is>
+          <t>Stand IC</t>
+        </is>
+      </c>
+      <c r="L22" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="14" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>19h00</t>
+        </is>
+      </c>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="F23" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="G23" s="10" t="inlineStr">
+        <is>
+          <t>Stand IC</t>
+        </is>
+      </c>
+      <c r="H23" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="I23" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="J23" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="K23" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="L23" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="14" customHeight="1">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>19h30</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E24" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G24" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H24" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I24" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J24" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K24" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L24" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="14" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>20h00</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E25" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G25" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H25" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I25" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J25" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K25" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L25" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="14" customHeight="1">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>20h30</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E26" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G26" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H26" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I26" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J26" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K26" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L26" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="14" customHeight="1">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>21h00</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E27" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G27" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H27" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I27" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J27" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K27" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L27" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="14" customHeight="1">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>21h30</t>
+        </is>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E28" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G28" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H28" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I28" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J28" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K28" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L28" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="11" t="inlineStr">
+        <is>
+          <t>Légende</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="12" t="inlineStr"/>
+      <c r="B32" s="13" t="inlineStr">
+        <is>
+          <t>Standiers = Back-up standiers Indie</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="14" t="inlineStr"/>
+      <c r="B33" s="13" t="inlineStr">
+        <is>
+          <t>Run = IC volant / Run (inclut le vote du public et le check des stands)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="15" t="inlineStr"/>
+      <c r="B34" s="13" t="inlineStr">
+        <is>
+          <t>Stand IC = Stand IC / Stunjam</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="16" t="inlineStr"/>
+      <c r="B35" s="13" t="inlineStr">
         <is>
           <t>Awards = Indie Awards (18h30-20h30, samedi) ; 2 personnes fixes restent en Standiers</t>
         </is>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" s="17" t="inlineStr"/>
+      <c r="B36" s="13" t="inlineStr">
+        <is>
+          <t>Média = Captation média (Chris, en continu les 3 jours)</t>
+        </is>
+      </c>
+    </row>
     <row r="37">
-      <c r="A37" s="19" t="inlineStr"/>
-      <c r="B37" s="14" t="inlineStr">
-        <is>
-          <t>Média = Captation média (Chris, en continu les 3 jours)</t>
+      <c r="A37" s="18" t="inlineStr"/>
+      <c r="B37" s="13" t="inlineStr">
+        <is>
+          <t>Briefing = Briefing d'équipe (vendredi 10h00-10h30)</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="20" t="inlineStr"/>
-      <c r="B38" s="14" t="inlineStr">
-        <is>
-          <t>Briefing = Briefing d'équipe (vendredi 10h00-10h30)</t>
+      <c r="A38" s="19" t="inlineStr"/>
+      <c r="B38" s="13" t="inlineStr">
+        <is>
+          <t>Off (inclut les 30 min de pause déjeuner + 30 min de pause dîner)</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="21" t="inlineStr"/>
-      <c r="B39" s="14" t="inlineStr">
-        <is>
-          <t>Off (inclut les 30 min de pause déjeuner + 30 min de pause dîner)</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="22" t="inlineStr"/>
-      <c r="B40" s="14" t="inlineStr">
+      <c r="A39" s="20" t="inlineStr"/>
+      <c r="B39" s="13" t="inlineStr">
         <is>
           <t>— = pas encore arrivé / absent ce jour-là</t>
         </is>
       </c>
     </row>
+    <row r="41">
+      <c r="A41" s="21" t="inlineStr">
+        <is>
+          <t>FERMETURE DE LA ZONE INDÉ À 19h30 TOUS LES SOIRS.</t>
+        </is>
+      </c>
+    </row>
     <row r="42">
-      <c r="A42" s="23" t="inlineStr">
-        <is>
-          <t>FERMETURE DE LA ZONE INDÉ À 19h30 TOUS LES SOIRS.</t>
+      <c r="A42" s="21" t="inlineStr">
+        <is>
+          <t>Ouverture au public à 10h. Bénévoles présents dès 9h pour la préparation : tout le monde en Run de 9h à 10h.</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="23" t="inlineStr">
-        <is>
-          <t>Ouverture au public à 10h. Bénévoles présents dès 9h pour la préparation : tout le monde en Run de 9h à 10h.</t>
+      <c r="A43" s="21" t="inlineStr">
+        <is>
+          <t>Robin : présent uniquement samedi et dimanche. Jeff : présent les 3 jours de 11h à 22h, en Run continu. Chris : captation Média en continu.</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="23" t="inlineStr">
-        <is>
-          <t>Robin : présent uniquement samedi et dimanche. Jeff : présent les 3 jours de 11h à 22h, en Run continu. Chris : captation Média en continu.</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="23" t="inlineStr">
+      <c r="A44" s="21" t="inlineStr">
         <is>
           <t>Règles : max 2h consécutives sur un même poste (hors Run de préparation du vendredi matin et Standiers fixes pendant les Awards, demandés explicitement) · 30 min de pause déjeuner (fenêtre 11h30-14h) + 30 min de pause dîner (fenêtre 18h30-21h) pour chacun·e, au moins 3 personnes en pause en même temps (affichées en Off). Exceptions : Jeff (Run continu) et, le samedi, les 2 Standiers fixes des Awards.</t>
         </is>

</xml_diff>

<commit_message>
Jeff dans la rotation (Standiers / Run / Stand IC, pauses repas)
</commit_message>
<xml_diff>
--- a/Planning_Stunfest2026_Indie.xlsx
+++ b/Planning_Stunfest2026_Indie.xlsx
@@ -1010,9 +1010,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="H9" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="H9" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -1181,9 +1181,9 @@
           <t>Run</t>
         </is>
       </c>
-      <c r="H12" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="I12" s="8" t="inlineStr">
@@ -1196,9 +1196,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="K12" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="K12" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
     </row>
@@ -1253,9 +1253,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="K13" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="K13" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
     </row>
@@ -1310,9 +1310,9 @@
           <t>Run</t>
         </is>
       </c>
-      <c r="K14" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="K14" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
     </row>
@@ -1332,9 +1332,9 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D15" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="E15" s="8" t="inlineStr">
@@ -1352,9 +1352,9 @@
           <t>Run</t>
         </is>
       </c>
-      <c r="H15" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="H15" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="I15" s="8" t="inlineStr">
@@ -1367,9 +1367,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="K15" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="K15" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
     </row>
@@ -1379,9 +1379,9 @@
           <t>15h30</t>
         </is>
       </c>
-      <c r="B16" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
@@ -1389,9 +1389,9 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -1409,9 +1409,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="H16" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="I16" s="8" t="inlineStr">
@@ -1436,9 +1436,9 @@
           <t>16h00</t>
         </is>
       </c>
-      <c r="B17" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
@@ -1446,19 +1446,19 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D17" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="E17" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="F17" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="G17" s="8" t="inlineStr">
@@ -1481,9 +1481,9 @@
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="K17" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="K17" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
     </row>
@@ -1508,39 +1508,39 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="E18" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="F18" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="G18" s="10" t="inlineStr">
+      <c r="E18" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="H18" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="I18" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="J18" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="K18" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="F18" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="H18" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="J18" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="K18" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
     </row>
@@ -1560,39 +1560,39 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="E19" s="10" t="inlineStr">
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="F19" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="G19" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="H19" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="I19" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="F19" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="G19" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="H19" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="I19" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="J19" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="J19" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
       <c r="K19" s="4" t="inlineStr">
@@ -1617,44 +1617,44 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D20" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="E20" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="F20" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="G20" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="H20" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="I20" s="10" t="inlineStr">
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="G20" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="J20" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="K20" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="H20" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="I20" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="J20" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="K20" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
     </row>
@@ -1664,9 +1664,9 @@
           <t>18h00</t>
         </is>
       </c>
-      <c r="B21" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
@@ -1674,44 +1674,44 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D21" s="10" t="inlineStr">
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="G21" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="H21" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="I21" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="J21" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="K21" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="E21" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="F21" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="G21" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="H21" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="I21" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="J21" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="K21" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
         </is>
       </c>
     </row>
@@ -1751,19 +1751,19 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="H22" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="I22" s="10" t="inlineStr">
+      <c r="H22" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="I22" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="J22" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="J22" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
         </is>
       </c>
       <c r="K22" s="4" t="inlineStr">
@@ -1778,24 +1778,24 @@
           <t>19h00</t>
         </is>
       </c>
-      <c r="B23" s="10" t="inlineStr">
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="D23" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="C23" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="D23" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="E23" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="F23" s="8" t="inlineStr">
@@ -1803,9 +1803,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="G23" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="G23" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="H23" s="8" t="inlineStr">
@@ -1823,9 +1823,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="K23" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="K23" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
     </row>
@@ -2209,14 +2209,14 @@
     <row r="44">
       <c r="A44" s="21" t="inlineStr">
         <is>
-          <t>Robin : présent uniquement samedi et dimanche. Jeff : présent les 3 jours de 11h à 22h, en Run continu. Chris : captation Média en continu.</t>
+          <t>Robin : présent uniquement samedi et dimanche. Jeff : présent les 3 jours de 11h à 22h, dans la rotation (seul en Run après 19h30). Chris : captation Média en continu.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="21" t="inlineStr">
         <is>
-          <t>Règles : max 2h consécutives sur un même poste (hors Run de préparation du vendredi matin et Standiers fixes pendant les Awards, demandés explicitement) · 30 min de pause déjeuner (fenêtre 11h30-14h) + 30 min de pause dîner (fenêtre 18h30-21h) pour chacun·e, au moins 3 personnes en pause en même temps (affichées en Off). Exceptions : Jeff (Run continu) et, le samedi, les 2 Standiers fixes des Awards.</t>
+          <t>Règles : max 2h consécutives sur un même poste (hors Run de préparation du vendredi matin et Standiers fixes pendant les Awards, demandés explicitement) · 30 min de pause déjeuner (fenêtre 11h30-14h) + 30 min de pause dîner (fenêtre 18h30-21h) pour chacun·e, au moins 3 personnes en pause en même temps (affichées en Off). Exception : le samedi, les 2 Standiers fixes des Awards.</t>
         </is>
       </c>
     </row>
@@ -2599,9 +2599,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="G7" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="G7" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="H7" s="8" t="inlineStr">
@@ -2661,24 +2661,24 @@
           <t>Standiers</t>
         </is>
       </c>
-      <c r="G8" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="H8" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="I8" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="J8" s="10" t="inlineStr">
+      <c r="G8" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
+        </is>
+      </c>
+      <c r="H8" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="I8" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="J8" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="K8" s="4" t="inlineStr">
@@ -2733,19 +2733,19 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="I9" s="10" t="inlineStr">
+      <c r="I9" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="J9" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="J9" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="K9" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="K9" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="L9" s="4" t="inlineStr">
@@ -2775,24 +2775,24 @@
           <t>Standiers</t>
         </is>
       </c>
-      <c r="E10" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="F10" s="10" t="inlineStr">
+      <c r="E10" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
           <t>Run</t>
         </is>
       </c>
-      <c r="H10" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="H10" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="I10" s="8" t="inlineStr">
@@ -2800,9 +2800,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="J10" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="J10" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
       <c r="K10" s="8" t="inlineStr">
@@ -2810,9 +2810,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="L10" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="L10" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
     </row>
@@ -2822,9 +2822,9 @@
           <t>13h00</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
@@ -2832,49 +2832,49 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D11" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="E11" s="10" t="inlineStr">
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="I11" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="J11" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="K11" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="L11" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="F11" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="G11" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="H11" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="I11" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="J11" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="K11" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="L11" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
         </is>
       </c>
     </row>
@@ -2884,9 +2884,9 @@
           <t>13h30</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
@@ -2894,29 +2894,29 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D12" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="E12" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="F12" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="G12" s="10" t="inlineStr">
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="F12" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="H12" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="G12" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="H12" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="I12" s="8" t="inlineStr">
@@ -2934,9 +2934,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="L12" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="L12" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
     </row>
@@ -2956,14 +2956,14 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="E13" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="F13" s="8" t="inlineStr">
@@ -2971,34 +2971,34 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="G13" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="H13" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="I13" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="J13" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="K13" s="10" t="inlineStr">
+      <c r="G13" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="I13" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="L13" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="J13" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="K13" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="L13" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
     </row>
@@ -3018,9 +3018,9 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D14" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="E14" s="8" t="inlineStr">
@@ -3033,9 +3033,9 @@
           <t>Run</t>
         </is>
       </c>
-      <c r="G14" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="G14" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="H14" s="8" t="inlineStr">
@@ -3043,24 +3043,24 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="I14" s="10" t="inlineStr">
+      <c r="I14" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="J14" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="K14" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="J14" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="K14" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="L14" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="L14" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
     </row>
@@ -3070,34 +3070,34 @@
           <t>15h00</t>
         </is>
       </c>
-      <c r="B15" s="10" t="inlineStr">
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="E15" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="D15" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="E15" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
       <c r="F15" s="8" t="inlineStr">
         <is>
           <t>Off</t>
         </is>
       </c>
-      <c r="G15" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="H15" s="8" t="inlineStr">
@@ -3105,9 +3105,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="I15" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="I15" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="J15" s="8" t="inlineStr">
@@ -3115,14 +3115,14 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="K15" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="L15" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="K15" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="L15" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
     </row>
@@ -3152,34 +3152,34 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="F16" s="10" t="inlineStr">
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="G16" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="H16" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="I16" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="J16" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="G16" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="H16" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="I16" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="J16" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="K16" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="K16" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="L16" s="4" t="inlineStr">
@@ -3194,9 +3194,9 @@
           <t>16h00</t>
         </is>
       </c>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="B17" s="10" t="inlineStr">
+        <is>
+          <t>Stand IC</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
@@ -3204,14 +3204,14 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D17" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="E17" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="E17" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
@@ -3234,19 +3234,19 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="J17" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="K17" s="10" t="inlineStr">
-        <is>
-          <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="L17" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="J17" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="K17" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="L17" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
     </row>
@@ -3266,29 +3266,29 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D18" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="E18" s="10" t="inlineStr">
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="F18" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="G18" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="F18" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="G18" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="H18" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="H18" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
@@ -3296,9 +3296,9 @@
           <t>Run</t>
         </is>
       </c>
-      <c r="J18" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="J18" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
       <c r="K18" s="8" t="inlineStr">
@@ -3306,9 +3306,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="L18" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="L18" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
     </row>
@@ -3333,9 +3333,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="E19" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="F19" s="8" t="inlineStr">
@@ -3343,34 +3343,34 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="G19" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="H19" s="10" t="inlineStr">
+      <c r="G19" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="H19" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="I19" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="J19" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="K19" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="L19" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="I19" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="J19" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="K19" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="L19" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
         </is>
       </c>
     </row>
@@ -3390,21 +3390,21 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D20" s="10" t="inlineStr">
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="F20" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="E20" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="F20" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
           <t>Run</t>
@@ -3420,9 +3420,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="J20" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="J20" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="K20" s="8" t="inlineStr">
@@ -3430,9 +3430,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="L20" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="L20" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
     </row>
@@ -3477,14 +3477,14 @@
           <t>Standiers</t>
         </is>
       </c>
-      <c r="I21" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="J21" s="10" t="inlineStr">
+      <c r="I21" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
+        </is>
+      </c>
+      <c r="J21" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="K21" s="4" t="inlineStr">
@@ -3678,9 +3678,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="L24" s="22" t="inlineStr">
-        <is>
-          <t>Awards</t>
+      <c r="L24" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
     </row>
@@ -4020,7 +4020,7 @@
     <row r="43">
       <c r="A43" s="21" t="inlineStr">
         <is>
-          <t>Robin : présent uniquement samedi et dimanche. Jeff : présent les 3 jours de 11h à 22h, en Run continu. Chris : captation Média en continu.</t>
+          <t>Robin : présent uniquement samedi et dimanche. Jeff : présent les 3 jours de 11h à 22h, dans la rotation (seul en Run après 19h30). Chris : captation Média en continu.</t>
         </is>
       </c>
     </row>
@@ -4034,7 +4034,7 @@
     <row r="45">
       <c r="A45" s="21" t="inlineStr">
         <is>
-          <t>Règles : max 2h consécutives sur un même poste (hors Run de préparation du vendredi matin et Standiers fixes pendant les Awards, demandés explicitement) · 30 min de pause déjeuner (fenêtre 11h30-14h) + 30 min de pause dîner (fenêtre 18h30-21h) pour chacun·e, au moins 3 personnes en pause en même temps (affichées en Off). Exceptions : Jeff (Run continu) et, le samedi, les 2 Standiers fixes des Awards.</t>
+          <t>Règles : max 2h consécutives sur un même poste (hors Run de préparation du vendredi matin et Standiers fixes pendant les Awards, demandés explicitement) · 30 min de pause déjeuner (fenêtre 11h30-14h) + 30 min de pause dîner (fenêtre 18h30-21h) pour chacun·e, au moins 3 personnes en pause en même temps (affichées en Off). Exception : le samedi, les 2 Standiers fixes des Awards.</t>
         </is>
       </c>
     </row>
@@ -4417,9 +4417,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="G7" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="G7" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="H7" s="8" t="inlineStr">
@@ -4479,24 +4479,24 @@
           <t>Standiers</t>
         </is>
       </c>
-      <c r="G8" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="H8" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="I8" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="J8" s="10" t="inlineStr">
+      <c r="G8" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
+        </is>
+      </c>
+      <c r="H8" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="I8" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="J8" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="K8" s="4" t="inlineStr">
@@ -4551,19 +4551,19 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="I9" s="10" t="inlineStr">
+      <c r="I9" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="J9" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="J9" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="K9" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="K9" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="L9" s="4" t="inlineStr">
@@ -4593,24 +4593,24 @@
           <t>Standiers</t>
         </is>
       </c>
-      <c r="E10" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="F10" s="10" t="inlineStr">
+      <c r="E10" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
           <t>Run</t>
         </is>
       </c>
-      <c r="H10" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="H10" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="I10" s="8" t="inlineStr">
@@ -4618,9 +4618,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="J10" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="J10" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
       <c r="K10" s="8" t="inlineStr">
@@ -4628,9 +4628,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="L10" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="L10" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
     </row>
@@ -4640,9 +4640,9 @@
           <t>13h00</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
@@ -4650,49 +4650,49 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D11" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="E11" s="10" t="inlineStr">
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="I11" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="J11" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="K11" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="L11" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="F11" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="G11" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="H11" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="I11" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="J11" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="K11" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="L11" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
         </is>
       </c>
     </row>
@@ -4702,9 +4702,9 @@
           <t>13h30</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
@@ -4712,29 +4712,29 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D12" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="E12" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="F12" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="G12" s="10" t="inlineStr">
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="F12" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="H12" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="G12" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="H12" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="I12" s="8" t="inlineStr">
@@ -4752,9 +4752,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="L12" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="L12" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
     </row>
@@ -4774,14 +4774,14 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="E13" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="F13" s="8" t="inlineStr">
@@ -4789,34 +4789,34 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="G13" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="H13" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="I13" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="J13" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="K13" s="10" t="inlineStr">
+      <c r="G13" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="I13" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="L13" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="J13" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="K13" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="L13" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
     </row>
@@ -4836,9 +4836,9 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D14" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="E14" s="8" t="inlineStr">
@@ -4851,9 +4851,9 @@
           <t>Run</t>
         </is>
       </c>
-      <c r="G14" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="G14" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="H14" s="8" t="inlineStr">
@@ -4861,24 +4861,24 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="I14" s="10" t="inlineStr">
+      <c r="I14" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="J14" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="K14" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="J14" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="K14" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="L14" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="L14" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
     </row>
@@ -4888,34 +4888,34 @@
           <t>15h00</t>
         </is>
       </c>
-      <c r="B15" s="10" t="inlineStr">
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="E15" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="D15" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="E15" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
       <c r="F15" s="8" t="inlineStr">
         <is>
           <t>Off</t>
         </is>
       </c>
-      <c r="G15" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="H15" s="8" t="inlineStr">
@@ -4923,9 +4923,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="I15" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="I15" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="J15" s="8" t="inlineStr">
@@ -4933,14 +4933,14 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="K15" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="L15" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="K15" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="L15" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
     </row>
@@ -4970,34 +4970,34 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="F16" s="10" t="inlineStr">
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="G16" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="H16" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="I16" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="J16" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="G16" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="H16" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="I16" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="J16" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="K16" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="K16" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="L16" s="4" t="inlineStr">
@@ -5012,9 +5012,9 @@
           <t>16h00</t>
         </is>
       </c>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="B17" s="10" t="inlineStr">
+        <is>
+          <t>Stand IC</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
@@ -5022,14 +5022,14 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D17" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="E17" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="E17" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
@@ -5052,19 +5052,19 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="J17" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="K17" s="10" t="inlineStr">
-        <is>
-          <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="L17" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="J17" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="K17" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="L17" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
     </row>
@@ -5084,29 +5084,29 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D18" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="E18" s="10" t="inlineStr">
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="F18" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="G18" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="F18" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="G18" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="H18" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="H18" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
@@ -5114,9 +5114,9 @@
           <t>Run</t>
         </is>
       </c>
-      <c r="J18" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="J18" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
       <c r="K18" s="8" t="inlineStr">
@@ -5124,9 +5124,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="L18" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="L18" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
     </row>
@@ -5151,9 +5151,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="E19" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="F19" s="8" t="inlineStr">
@@ -5161,34 +5161,34 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="G19" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="H19" s="10" t="inlineStr">
+      <c r="G19" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="H19" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="I19" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="J19" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="K19" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="L19" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="I19" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="J19" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="K19" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="L19" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
         </is>
       </c>
     </row>
@@ -5208,21 +5208,21 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D20" s="10" t="inlineStr">
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="F20" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="E20" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="F20" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
           <t>Run</t>
@@ -5238,9 +5238,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="J20" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="J20" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="K20" s="8" t="inlineStr">
@@ -5248,9 +5248,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="L20" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="L20" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
     </row>
@@ -5295,14 +5295,14 @@
           <t>Standiers</t>
         </is>
       </c>
-      <c r="I21" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="J21" s="10" t="inlineStr">
+      <c r="I21" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
+        </is>
+      </c>
+      <c r="J21" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="K21" s="4" t="inlineStr">
@@ -5357,14 +5357,14 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="I22" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="J22" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="I22" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="J22" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
       <c r="K22" s="10" t="inlineStr">
@@ -5394,14 +5394,14 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="D23" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="E23" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="D23" s="10" t="inlineStr">
+        <is>
+          <t>Stand IC</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="F23" s="8" t="inlineStr">
@@ -5409,9 +5409,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="G23" s="10" t="inlineStr">
-        <is>
-          <t>Stand IC</t>
+      <c r="G23" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="H23" s="8" t="inlineStr">
@@ -5434,9 +5434,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="L23" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="L23" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
     </row>
@@ -5838,14 +5838,14 @@
     <row r="43">
       <c r="A43" s="21" t="inlineStr">
         <is>
-          <t>Robin : présent uniquement samedi et dimanche. Jeff : présent les 3 jours de 11h à 22h, en Run continu. Chris : captation Média en continu.</t>
+          <t>Robin : présent uniquement samedi et dimanche. Jeff : présent les 3 jours de 11h à 22h, dans la rotation (seul en Run après 19h30). Chris : captation Média en continu.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="21" t="inlineStr">
         <is>
-          <t>Règles : max 2h consécutives sur un même poste (hors Run de préparation du vendredi matin et Standiers fixes pendant les Awards, demandés explicitement) · 30 min de pause déjeuner (fenêtre 11h30-14h) + 30 min de pause dîner (fenêtre 18h30-21h) pour chacun·e, au moins 3 personnes en pause en même temps (affichées en Off). Exceptions : Jeff (Run continu) et, le samedi, les 2 Standiers fixes des Awards.</t>
+          <t>Règles : max 2h consécutives sur un même poste (hors Run de préparation du vendredi matin et Standiers fixes pendant les Awards, demandés explicitement) · 30 min de pause déjeuner (fenêtre 11h30-14h) + 30 min de pause dîner (fenêtre 18h30-21h) pour chacun·e, au moins 3 personnes en pause en même temps (affichées en Off). Exception : le samedi, les 2 Standiers fixes des Awards.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Pause fusionnée dans Off ; repas étalés sur les fenêtres 11h30-14h et 18h30-21h
</commit_message>
<xml_diff>
--- a/Planning_Stunfest2026_Indie.xlsx
+++ b/Planning_Stunfest2026_Indie.xlsx
@@ -923,9 +923,9 @@
           <t>11h30</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -933,14 +933,14 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
@@ -980,9 +980,9 @@
           <t>12h00</t>
         </is>
       </c>
-      <c r="B9" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="C9" s="8" t="inlineStr">
@@ -990,29 +990,29 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="D9" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="E9" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="F9" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="G9" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="H9" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -1057,19 +1057,19 @@
           <t>Run</t>
         </is>
       </c>
-      <c r="F10" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="G10" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="H10" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="H10" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
@@ -1751,19 +1751,19 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="H22" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="I22" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="J22" s="10" t="inlineStr">
+      <c r="H22" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="I22" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
+        </is>
+      </c>
+      <c r="J22" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="K22" s="4" t="inlineStr">
@@ -1788,24 +1788,24 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="D23" s="10" t="inlineStr">
+      <c r="D23" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="E23" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="E23" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="F23" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="G23" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="H23" s="8" t="inlineStr">
@@ -2173,7 +2173,7 @@
       <c r="A38" s="19" t="inlineStr"/>
       <c r="B38" s="13" t="inlineStr">
         <is>
-          <t>Off (inclut les 30 min de pause déjeuner + 30 min de pause dîner)</t>
+          <t>Off (inclut les repas : 30 min le midi, 30 min le soir, répartis sur les fenêtres 11h30-14h et 18h30-21h)</t>
         </is>
       </c>
     </row>
@@ -2651,14 +2651,14 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="E8" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="F8" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="G8" s="10" t="inlineStr">
@@ -2671,14 +2671,14 @@
           <t>Standiers</t>
         </is>
       </c>
-      <c r="I8" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="J8" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="I8" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="J8" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
       <c r="K8" s="4" t="inlineStr">
@@ -2698,9 +2698,9 @@
           <t>12h00</t>
         </is>
       </c>
-      <c r="B9" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="C9" s="8" t="inlineStr">
@@ -2713,19 +2713,19 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="E9" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="F9" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="G9" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="E9" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="F9" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="H9" s="8" t="inlineStr">
@@ -2733,24 +2733,24 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="I9" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="J9" s="10" t="inlineStr">
+      <c r="I9" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
+      <c r="J9" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
       <c r="K9" s="8" t="inlineStr">
         <is>
           <t>Off</t>
         </is>
       </c>
-      <c r="L9" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="L9" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
     </row>
@@ -2760,9 +2760,9 @@
           <t>12h30</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
@@ -2775,44 +2775,44 @@
           <t>Standiers</t>
         </is>
       </c>
-      <c r="E10" s="10" t="inlineStr">
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="F10" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="H10" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="J10" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="F10" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="G10" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="H10" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="I10" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="J10" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="K10" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="L10" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="K10" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="L10" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
     </row>
@@ -2822,9 +2822,9 @@
           <t>13h00</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
@@ -2832,19 +2832,19 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D11" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="E11" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="F11" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="E11" s="10" t="inlineStr">
+        <is>
+          <t>Stand IC</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="G11" s="8" t="inlineStr">
@@ -2857,9 +2857,9 @@
           <t>Run</t>
         </is>
       </c>
-      <c r="I11" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="J11" s="8" t="inlineStr">
@@ -2867,14 +2867,14 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="K11" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="L11" s="10" t="inlineStr">
-        <is>
-          <t>Stand IC</t>
+      <c r="K11" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="L11" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
     </row>
@@ -2884,9 +2884,9 @@
           <t>13h30</t>
         </is>
       </c>
-      <c r="B12" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
@@ -2894,14 +2894,14 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D12" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="E12" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="F12" s="10" t="inlineStr">
@@ -2909,19 +2909,19 @@
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="G12" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="H12" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="I12" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="G12" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="H12" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="I12" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
       <c r="J12" s="8" t="inlineStr">
@@ -2961,9 +2961,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="E13" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="F13" s="8" t="inlineStr">
@@ -2971,34 +2971,34 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="G13" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="H13" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="I13" s="10" t="inlineStr">
+      <c r="G13" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="H13" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="I13" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="J13" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="K13" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="J13" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="K13" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="L13" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="L13" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
     </row>
@@ -3018,9 +3018,9 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="E14" s="8" t="inlineStr">
@@ -3028,19 +3028,19 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="G14" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="H14" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="I14" s="8" t="inlineStr">
@@ -3053,14 +3053,14 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="K14" s="10" t="inlineStr">
+      <c r="K14" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="L14" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="L14" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
         </is>
       </c>
     </row>
@@ -3080,24 +3080,24 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D15" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="E15" s="10" t="inlineStr">
+      <c r="D15" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
       <c r="F15" s="8" t="inlineStr">
         <is>
           <t>Off</t>
         </is>
       </c>
-      <c r="G15" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="H15" s="8" t="inlineStr">
@@ -3110,9 +3110,9 @@
           <t>Run</t>
         </is>
       </c>
-      <c r="J15" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="J15" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="K15" s="8" t="inlineStr">
@@ -3147,24 +3147,24 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="E16" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="F16" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="G16" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="H16" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="E16" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="F16" s="10" t="inlineStr">
+        <is>
+          <t>Stand IC</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="I16" s="8" t="inlineStr">
@@ -3172,19 +3172,19 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="J16" s="10" t="inlineStr">
-        <is>
-          <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="K16" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="L16" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="J16" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="K16" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="L16" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
     </row>
@@ -3194,59 +3194,59 @@
           <t>16h00</t>
         </is>
       </c>
-      <c r="B17" s="10" t="inlineStr">
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="G17" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="H17" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="I17" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="J17" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="D17" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="E17" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="F17" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="G17" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="H17" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="I17" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="J17" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="K17" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="L17" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="K17" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="L17" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
     </row>
@@ -3256,9 +3256,9 @@
           <t>16h30</t>
         </is>
       </c>
-      <c r="B18" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>Stand IC</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
@@ -3266,39 +3266,39 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D18" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="E18" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="F18" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="G18" s="10" t="inlineStr">
-        <is>
-          <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="H18" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="I18" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="J18" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="G18" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="H18" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="J18" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="K18" s="8" t="inlineStr">
@@ -3318,9 +3318,9 @@
           <t>17h00</t>
         </is>
       </c>
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
@@ -3333,9 +3333,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="E19" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="F19" s="8" t="inlineStr">
@@ -3343,34 +3343,34 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="G19" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="H19" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="I19" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="J19" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="K19" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="L19" s="10" t="inlineStr">
+      <c r="G19" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="H19" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
+        </is>
+      </c>
+      <c r="I19" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="J19" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="K19" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="L19" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
     </row>
@@ -3380,9 +3380,9 @@
           <t>17h30</t>
         </is>
       </c>
-      <c r="B20" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
@@ -3390,9 +3390,9 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D20" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="E20" s="8" t="inlineStr">
@@ -3400,39 +3400,39 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="F20" s="10" t="inlineStr">
+      <c r="F20" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="G20" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="H20" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="I20" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="J20" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="K20" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="L20" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="G20" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="H20" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="I20" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="J20" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="K20" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="L20" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
         </is>
       </c>
     </row>
@@ -3457,44 +3457,44 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="E21" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="F21" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="G21" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="H21" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="I21" s="10" t="inlineStr">
+      <c r="E21" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
+      <c r="F21" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="I21" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
       <c r="J21" s="8" t="inlineStr">
         <is>
           <t>Off</t>
         </is>
       </c>
-      <c r="K21" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="L21" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="K21" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="L21" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
     </row>
@@ -3504,9 +3504,9 @@
           <t>18h30</t>
         </is>
       </c>
-      <c r="B22" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="B22" s="22" t="inlineStr">
+        <is>
+          <t>Awards</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
@@ -3514,9 +3514,9 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D22" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="D22" s="22" t="inlineStr">
+        <is>
+          <t>Awards</t>
         </is>
       </c>
       <c r="E22" s="22" t="inlineStr">
@@ -3539,14 +3539,14 @@
           <t>Awards</t>
         </is>
       </c>
-      <c r="I22" s="22" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="J22" s="22" t="inlineStr">
-        <is>
-          <t>Awards</t>
+      <c r="I22" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="J22" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
       <c r="K22" s="22" t="inlineStr">
@@ -3566,9 +3566,9 @@
           <t>19h00</t>
         </is>
       </c>
-      <c r="B23" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="B23" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="C23" s="8" t="inlineStr">
@@ -3576,9 +3576,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="D23" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="E23" s="8" t="inlineStr">
@@ -3591,24 +3591,24 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="G23" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="H23" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="I23" s="22" t="inlineStr">
+      <c r="G23" s="22" t="inlineStr">
         <is>
           <t>Awards</t>
         </is>
       </c>
-      <c r="J23" s="22" t="inlineStr">
+      <c r="H23" s="22" t="inlineStr">
         <is>
           <t>Awards</t>
+        </is>
+      </c>
+      <c r="I23" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="J23" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
       <c r="K23" s="22" t="inlineStr">
@@ -3628,9 +3628,9 @@
           <t>19h30</t>
         </is>
       </c>
-      <c r="B24" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="B24" s="22" t="inlineStr">
+        <is>
+          <t>Awards</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
@@ -3638,9 +3638,9 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D24" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="D24" s="22" t="inlineStr">
+        <is>
+          <t>Awards</t>
         </is>
       </c>
       <c r="E24" s="22" t="inlineStr">
@@ -3663,24 +3663,24 @@
           <t>Awards</t>
         </is>
       </c>
-      <c r="I24" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="J24" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="K24" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="L24" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="I24" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="J24" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="K24" s="22" t="inlineStr">
+        <is>
+          <t>Awards</t>
+        </is>
+      </c>
+      <c r="L24" s="22" t="inlineStr">
+        <is>
+          <t>Awards</t>
         </is>
       </c>
     </row>
@@ -3690,9 +3690,9 @@
           <t>20h00</t>
         </is>
       </c>
-      <c r="B25" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="B25" s="22" t="inlineStr">
+        <is>
+          <t>Awards</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
@@ -3700,9 +3700,9 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D25" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="D25" s="22" t="inlineStr">
+        <is>
+          <t>Awards</t>
         </is>
       </c>
       <c r="E25" s="22" t="inlineStr">
@@ -3715,34 +3715,34 @@
           <t>Awards</t>
         </is>
       </c>
-      <c r="G25" s="22" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="H25" s="22" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="I25" s="22" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="J25" s="22" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="K25" s="22" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="L25" s="22" t="inlineStr">
-        <is>
-          <t>Awards</t>
+      <c r="G25" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="H25" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="I25" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="J25" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="K25" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="L25" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
     </row>
@@ -3752,9 +3752,9 @@
           <t>20h30</t>
         </is>
       </c>
-      <c r="B26" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="B26" s="22" t="inlineStr">
+        <is>
+          <t>Awards</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
@@ -3762,9 +3762,9 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D26" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="D26" s="22" t="inlineStr">
+        <is>
+          <t>Awards</t>
         </is>
       </c>
       <c r="E26" s="22" t="inlineStr">
@@ -3787,14 +3787,14 @@
           <t>Awards</t>
         </is>
       </c>
-      <c r="I26" s="22" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="J26" s="22" t="inlineStr">
-        <is>
-          <t>Awards</t>
+      <c r="I26" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="J26" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
       <c r="K26" s="22" t="inlineStr">
@@ -3991,7 +3991,7 @@
       <c r="A38" s="19" t="inlineStr"/>
       <c r="B38" s="13" t="inlineStr">
         <is>
-          <t>Off (inclut les 30 min de pause déjeuner + 30 min de pause dîner)</t>
+          <t>Off (inclut les repas : 30 min le midi, 30 min le soir, répartis sur les fenêtres 11h30-14h et 18h30-21h)</t>
         </is>
       </c>
     </row>
@@ -4469,14 +4469,14 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="E8" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="F8" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="G8" s="10" t="inlineStr">
@@ -4489,14 +4489,14 @@
           <t>Standiers</t>
         </is>
       </c>
-      <c r="I8" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="J8" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="I8" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="J8" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
       <c r="K8" s="4" t="inlineStr">
@@ -4516,9 +4516,9 @@
           <t>12h00</t>
         </is>
       </c>
-      <c r="B9" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="C9" s="8" t="inlineStr">
@@ -4531,19 +4531,19 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="E9" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="F9" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="G9" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="E9" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="F9" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="H9" s="8" t="inlineStr">
@@ -4551,24 +4551,24 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="I9" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="J9" s="10" t="inlineStr">
+      <c r="I9" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
+      <c r="J9" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
       <c r="K9" s="8" t="inlineStr">
         <is>
           <t>Off</t>
         </is>
       </c>
-      <c r="L9" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="L9" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
     </row>
@@ -4578,9 +4578,9 @@
           <t>12h30</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
@@ -4593,44 +4593,44 @@
           <t>Standiers</t>
         </is>
       </c>
-      <c r="E10" s="10" t="inlineStr">
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="F10" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="H10" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="J10" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="F10" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="G10" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="H10" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="I10" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="J10" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="K10" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="L10" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="K10" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="L10" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
     </row>
@@ -4640,9 +4640,9 @@
           <t>13h00</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
@@ -4650,19 +4650,19 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D11" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="E11" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="F11" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="E11" s="10" t="inlineStr">
+        <is>
+          <t>Stand IC</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="G11" s="8" t="inlineStr">
@@ -4675,9 +4675,9 @@
           <t>Run</t>
         </is>
       </c>
-      <c r="I11" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="J11" s="8" t="inlineStr">
@@ -4685,14 +4685,14 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="K11" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="L11" s="10" t="inlineStr">
-        <is>
-          <t>Stand IC</t>
+      <c r="K11" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="L11" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
     </row>
@@ -4702,9 +4702,9 @@
           <t>13h30</t>
         </is>
       </c>
-      <c r="B12" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
@@ -4712,14 +4712,14 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D12" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="E12" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="F12" s="10" t="inlineStr">
@@ -4727,19 +4727,19 @@
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="G12" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="H12" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="I12" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="G12" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="H12" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="I12" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
       <c r="J12" s="8" t="inlineStr">
@@ -4779,9 +4779,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="E13" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="F13" s="8" t="inlineStr">
@@ -4789,34 +4789,34 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="G13" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="H13" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="I13" s="10" t="inlineStr">
+      <c r="G13" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="H13" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="I13" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="J13" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="K13" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="J13" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="K13" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="L13" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="L13" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
     </row>
@@ -4836,9 +4836,9 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="E14" s="8" t="inlineStr">
@@ -4846,19 +4846,19 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="G14" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="H14" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="I14" s="8" t="inlineStr">
@@ -4871,14 +4871,14 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="K14" s="10" t="inlineStr">
+      <c r="K14" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="L14" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="L14" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
         </is>
       </c>
     </row>
@@ -4898,24 +4898,24 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D15" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="E15" s="10" t="inlineStr">
+      <c r="D15" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
       <c r="F15" s="8" t="inlineStr">
         <is>
           <t>Off</t>
         </is>
       </c>
-      <c r="G15" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="H15" s="8" t="inlineStr">
@@ -4928,9 +4928,9 @@
           <t>Run</t>
         </is>
       </c>
-      <c r="J15" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="J15" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="K15" s="8" t="inlineStr">
@@ -4965,24 +4965,24 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="E16" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="F16" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="G16" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="H16" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="E16" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="F16" s="10" t="inlineStr">
+        <is>
+          <t>Stand IC</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="I16" s="8" t="inlineStr">
@@ -4990,19 +4990,19 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="J16" s="10" t="inlineStr">
-        <is>
-          <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="K16" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="L16" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="J16" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="K16" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="L16" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
     </row>
@@ -5012,59 +5012,59 @@
           <t>16h00</t>
         </is>
       </c>
-      <c r="B17" s="10" t="inlineStr">
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="G17" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="H17" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="I17" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="J17" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="D17" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="E17" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="F17" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="G17" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="H17" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="I17" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="J17" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="K17" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="L17" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="K17" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="L17" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
     </row>
@@ -5074,9 +5074,9 @@
           <t>16h30</t>
         </is>
       </c>
-      <c r="B18" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>Stand IC</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
@@ -5084,39 +5084,39 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D18" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="E18" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="F18" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="G18" s="10" t="inlineStr">
-        <is>
-          <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="H18" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="I18" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="J18" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="G18" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="H18" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="J18" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="K18" s="8" t="inlineStr">
@@ -5136,9 +5136,9 @@
           <t>17h00</t>
         </is>
       </c>
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
@@ -5151,9 +5151,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="E19" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="F19" s="8" t="inlineStr">
@@ -5161,34 +5161,34 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="G19" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="H19" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="I19" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="J19" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="K19" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="L19" s="10" t="inlineStr">
+      <c r="G19" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="H19" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
+        </is>
+      </c>
+      <c r="I19" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="J19" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="K19" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="L19" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
     </row>
@@ -5198,9 +5198,9 @@
           <t>17h30</t>
         </is>
       </c>
-      <c r="B20" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
@@ -5208,9 +5208,9 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D20" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="E20" s="8" t="inlineStr">
@@ -5218,39 +5218,39 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="F20" s="10" t="inlineStr">
+      <c r="F20" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="G20" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="H20" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="I20" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="J20" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="K20" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="L20" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="G20" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="H20" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="I20" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="J20" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="K20" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="L20" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
         </is>
       </c>
     </row>
@@ -5275,44 +5275,44 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="E21" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="F21" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="G21" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="H21" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="I21" s="10" t="inlineStr">
+      <c r="E21" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
+      <c r="F21" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="I21" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
       <c r="J21" s="8" t="inlineStr">
         <is>
           <t>Off</t>
         </is>
       </c>
-      <c r="K21" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="L21" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="K21" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="L21" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
     </row>
@@ -5352,14 +5352,14 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="H22" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="I22" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="H22" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="I22" s="10" t="inlineStr">
+        <is>
+          <t>Stand IC</t>
         </is>
       </c>
       <c r="J22" s="9" t="inlineStr">
@@ -5367,9 +5367,9 @@
           <t>Standiers</t>
         </is>
       </c>
-      <c r="K22" s="10" t="inlineStr">
-        <is>
-          <t>Stand IC</t>
+      <c r="K22" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="L22" s="4" t="inlineStr">
@@ -5394,24 +5394,24 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="D23" s="10" t="inlineStr">
+      <c r="D23" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="G23" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="E23" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="F23" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="G23" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
         </is>
       </c>
       <c r="H23" s="8" t="inlineStr">
@@ -5809,7 +5809,7 @@
       <c r="A38" s="19" t="inlineStr"/>
       <c r="B38" s="13" t="inlineStr">
         <is>
-          <t>Off (inclut les 30 min de pause déjeuner + 30 min de pause dîner)</t>
+          <t>Off (inclut les repas : 30 min le midi, 30 min le soir, répartis sur les fenêtres 11h30-14h et 18h30-21h)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tout le monde mange midi et soir, Standiers fixes des Awards compris
</commit_message>
<xml_diff>
--- a/Planning_Stunfest2026_Indie.xlsx
+++ b/Planning_Stunfest2026_Indie.xlsx
@@ -2216,7 +2216,7 @@
     <row r="45">
       <c r="A45" s="21" t="inlineStr">
         <is>
-          <t>Règles : max 2h consécutives sur un même poste (hors Run de préparation du vendredi matin et Standiers fixes pendant les Awards, demandés explicitement) · 30 min de pause déjeuner (fenêtre 11h30-14h) + 30 min de pause dîner (fenêtre 18h30-21h) pour chacun·e, au moins 3 personnes en pause en même temps (affichées en Off). Exception : le samedi, les 2 Standiers fixes des Awards.</t>
+          <t>Règles : max 2h consécutives sur un même poste (hors Run de préparation du vendredi matin et Standiers fixes pendant les Awards, demandés explicitement) · un repas de 30 min le midi (fenêtre 11h30-14h) et le soir (fenêtre 18h30-21h) pour chacun·e, y compris Chris et Jeff, au moins 3 personnes en Off en même temps. Le samedi, les 2 Standiers fixes des Awards mangent ensemble à 19h30, remplacés par 2 personnes des Awards.</t>
         </is>
       </c>
     </row>
@@ -3504,9 +3504,9 @@
           <t>18h30</t>
         </is>
       </c>
-      <c r="B22" s="22" t="inlineStr">
-        <is>
-          <t>Awards</t>
+      <c r="B22" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
@@ -3514,19 +3514,19 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D22" s="22" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="E22" s="22" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="F22" s="22" t="inlineStr">
-        <is>
-          <t>Awards</t>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="F22" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="G22" s="22" t="inlineStr">
@@ -3566,9 +3566,9 @@
           <t>19h00</t>
         </is>
       </c>
-      <c r="B23" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="B23" s="22" t="inlineStr">
+        <is>
+          <t>Awards</t>
         </is>
       </c>
       <c r="C23" s="8" t="inlineStr">
@@ -3576,19 +3576,19 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="D23" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="E23" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="F23" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="D23" s="22" t="inlineStr">
+        <is>
+          <t>Awards</t>
+        </is>
+      </c>
+      <c r="E23" s="22" t="inlineStr">
+        <is>
+          <t>Awards</t>
+        </is>
+      </c>
+      <c r="F23" s="22" t="inlineStr">
+        <is>
+          <t>Awards</t>
         </is>
       </c>
       <c r="G23" s="22" t="inlineStr">
@@ -3653,34 +3653,34 @@
           <t>Awards</t>
         </is>
       </c>
-      <c r="G24" s="22" t="inlineStr">
+      <c r="G24" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="H24" s="22" t="inlineStr">
         <is>
           <t>Awards</t>
         </is>
       </c>
-      <c r="H24" s="22" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="I24" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="J24" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="K24" s="22" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="L24" s="22" t="inlineStr">
-        <is>
-          <t>Awards</t>
+      <c r="I24" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="J24" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="K24" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="L24" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
     </row>
@@ -3715,14 +3715,14 @@
           <t>Awards</t>
         </is>
       </c>
-      <c r="G25" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="H25" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="G25" s="22" t="inlineStr">
+        <is>
+          <t>Awards</t>
+        </is>
+      </c>
+      <c r="H25" s="22" t="inlineStr">
+        <is>
+          <t>Awards</t>
         </is>
       </c>
       <c r="I25" s="9" t="inlineStr">
@@ -3735,14 +3735,14 @@
           <t>Standiers</t>
         </is>
       </c>
-      <c r="K25" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="L25" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="K25" s="22" t="inlineStr">
+        <is>
+          <t>Awards</t>
+        </is>
+      </c>
+      <c r="L25" s="22" t="inlineStr">
+        <is>
+          <t>Awards</t>
         </is>
       </c>
     </row>
@@ -3782,9 +3782,9 @@
           <t>Awards</t>
         </is>
       </c>
-      <c r="H26" s="22" t="inlineStr">
-        <is>
-          <t>Awards</t>
+      <c r="H26" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="I26" s="9" t="inlineStr">
@@ -3797,14 +3797,14 @@
           <t>Standiers</t>
         </is>
       </c>
-      <c r="K26" s="22" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="L26" s="22" t="inlineStr">
-        <is>
-          <t>Awards</t>
+      <c r="K26" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="L26" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
     </row>
@@ -4034,7 +4034,7 @@
     <row r="45">
       <c r="A45" s="21" t="inlineStr">
         <is>
-          <t>Règles : max 2h consécutives sur un même poste (hors Run de préparation du vendredi matin et Standiers fixes pendant les Awards, demandés explicitement) · 30 min de pause déjeuner (fenêtre 11h30-14h) + 30 min de pause dîner (fenêtre 18h30-21h) pour chacun·e, au moins 3 personnes en pause en même temps (affichées en Off). Exception : le samedi, les 2 Standiers fixes des Awards.</t>
+          <t>Règles : max 2h consécutives sur un même poste (hors Run de préparation du vendredi matin et Standiers fixes pendant les Awards, demandés explicitement) · un repas de 30 min le midi (fenêtre 11h30-14h) et le soir (fenêtre 18h30-21h) pour chacun·e, y compris Chris et Jeff, au moins 3 personnes en Off en même temps. Le samedi, les 2 Standiers fixes des Awards mangent ensemble à 19h30, remplacés par 2 personnes des Awards.</t>
         </is>
       </c>
     </row>
@@ -5845,7 +5845,7 @@
     <row r="44">
       <c r="A44" s="21" t="inlineStr">
         <is>
-          <t>Règles : max 2h consécutives sur un même poste (hors Run de préparation du vendredi matin et Standiers fixes pendant les Awards, demandés explicitement) · 30 min de pause déjeuner (fenêtre 11h30-14h) + 30 min de pause dîner (fenêtre 18h30-21h) pour chacun·e, au moins 3 personnes en pause en même temps (affichées en Off). Exception : le samedi, les 2 Standiers fixes des Awards.</t>
+          <t>Règles : max 2h consécutives sur un même poste (hors Run de préparation du vendredi matin et Standiers fixes pendant les Awards, demandés explicitement) · un repas de 30 min le midi (fenêtre 11h30-14h) et le soir (fenêtre 18h30-21h) pour chacun·e, y compris Chris et Jeff, au moins 3 personnes en Off en même temps. Le samedi, les 2 Standiers fixes des Awards mangent ensemble à 19h30, remplacés par 2 personnes des Awards.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Chris mange en groupe avec les autres, Média le reste du temps
</commit_message>
<xml_diff>
--- a/Planning_Stunfest2026_Indie.xlsx
+++ b/Planning_Stunfest2026_Indie.xlsx
@@ -943,9 +943,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="F8" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
@@ -985,9 +985,9 @@
           <t>Run</t>
         </is>
       </c>
-      <c r="C9" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Média</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
@@ -1057,9 +1057,9 @@
           <t>Run</t>
         </is>
       </c>
-      <c r="F10" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="G10" s="8" t="inlineStr">
@@ -1072,9 +1072,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="I10" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
@@ -1156,9 +1156,9 @@
           <t>Run</t>
         </is>
       </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>Média</t>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
@@ -1186,9 +1186,9 @@
           <t>Run</t>
         </is>
       </c>
-      <c r="I12" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="I12" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="J12" s="8" t="inlineStr">
@@ -2216,7 +2216,7 @@
     <row r="45">
       <c r="A45" s="21" t="inlineStr">
         <is>
-          <t>Règles : max 2h consécutives sur un même poste (hors Run de préparation du vendredi matin et Standiers fixes pendant les Awards, demandés explicitement) · un repas de 30 min le midi (fenêtre 11h30-14h) et le soir (fenêtre 18h30-21h) pour chacun·e, y compris Chris et Jeff, au moins 3 personnes en Off en même temps. Le samedi, les 2 Standiers fixes des Awards mangent ensemble à 19h30, remplacés par 2 personnes des Awards.</t>
+          <t>Règles : max 2h consécutives sur un même poste (hors Run de préparation du vendredi matin et Standiers fixes pendant les Awards, demandés explicitement) · un repas de 30 min le midi (fenêtre 11h30-14h) et le soir (fenêtre 18h30-21h) pour chacun·e, y compris Chris (Média le reste du temps) et Jeff, jamais seul : au moins 3 personnes en Off en même temps. Le samedi, les 2 Standiers fixes des Awards mangent ensemble à 19h30, remplacés par 2 personnes des Awards.</t>
         </is>
       </c>
     </row>
@@ -2703,9 +2703,9 @@
           <t>Run</t>
         </is>
       </c>
-      <c r="C9" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Média</t>
         </is>
       </c>
       <c r="D9" s="8" t="inlineStr">
@@ -2760,9 +2760,9 @@
           <t>12h30</t>
         </is>
       </c>
-      <c r="B10" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
@@ -2800,14 +2800,14 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="J10" s="10" t="inlineStr">
+      <c r="J10" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="K10" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="K10" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
         </is>
       </c>
       <c r="L10" s="4" t="inlineStr">
@@ -2822,9 +2822,9 @@
           <t>13h00</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
@@ -2862,9 +2862,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="J11" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="J11" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
       <c r="K11" s="8" t="inlineStr">
@@ -2884,14 +2884,14 @@
           <t>13h30</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>Média</t>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
@@ -2899,34 +2899,34 @@
           <t>Run</t>
         </is>
       </c>
-      <c r="E12" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="F12" s="10" t="inlineStr">
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="G12" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="H12" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="I12" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="J12" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="G12" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="H12" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="I12" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="J12" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
         </is>
       </c>
       <c r="K12" s="8" t="inlineStr">
@@ -2961,9 +2961,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="E13" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="F13" s="8" t="inlineStr">
@@ -2971,14 +2971,14 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="G13" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="H13" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="I13" s="8" t="inlineStr">
@@ -2986,19 +2986,19 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="J13" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="K13" s="10" t="inlineStr">
+      <c r="J13" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="K13" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="L13" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="L13" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
         </is>
       </c>
     </row>
@@ -3008,9 +3008,9 @@
           <t>14h30</t>
         </is>
       </c>
-      <c r="B14" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
@@ -3028,39 +3028,39 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="F14" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="G14" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="H14" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="I14" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="J14" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="K14" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="L14" s="10" t="inlineStr">
+      <c r="F14" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
+        </is>
+      </c>
+      <c r="G14" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="H14" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="I14" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="J14" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="K14" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="L14" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
     </row>
@@ -3105,24 +3105,24 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="I15" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="J15" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="K15" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="L15" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="I15" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="J15" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="K15" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="L15" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
     </row>
@@ -3571,9 +3571,9 @@
           <t>Awards</t>
         </is>
       </c>
-      <c r="C23" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>Média</t>
         </is>
       </c>
       <c r="D23" s="22" t="inlineStr">
@@ -3658,9 +3658,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="H24" s="22" t="inlineStr">
-        <is>
-          <t>Awards</t>
+      <c r="H24" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="I24" s="8" t="inlineStr">
@@ -3757,9 +3757,9 @@
           <t>Awards</t>
         </is>
       </c>
-      <c r="C26" s="5" t="inlineStr">
-        <is>
-          <t>Média</t>
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="D26" s="22" t="inlineStr">
@@ -3782,9 +3782,9 @@
           <t>Awards</t>
         </is>
       </c>
-      <c r="H26" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="H26" s="22" t="inlineStr">
+        <is>
+          <t>Awards</t>
         </is>
       </c>
       <c r="I26" s="9" t="inlineStr">
@@ -4034,7 +4034,7 @@
     <row r="45">
       <c r="A45" s="21" t="inlineStr">
         <is>
-          <t>Règles : max 2h consécutives sur un même poste (hors Run de préparation du vendredi matin et Standiers fixes pendant les Awards, demandés explicitement) · un repas de 30 min le midi (fenêtre 11h30-14h) et le soir (fenêtre 18h30-21h) pour chacun·e, y compris Chris et Jeff, au moins 3 personnes en Off en même temps. Le samedi, les 2 Standiers fixes des Awards mangent ensemble à 19h30, remplacés par 2 personnes des Awards.</t>
+          <t>Règles : max 2h consécutives sur un même poste (hors Run de préparation du vendredi matin et Standiers fixes pendant les Awards, demandés explicitement) · un repas de 30 min le midi (fenêtre 11h30-14h) et le soir (fenêtre 18h30-21h) pour chacun·e, y compris Chris (Média le reste du temps) et Jeff, jamais seul : au moins 3 personnes en Off en même temps. Le samedi, les 2 Standiers fixes des Awards mangent ensemble à 19h30, remplacés par 2 personnes des Awards.</t>
         </is>
       </c>
     </row>
@@ -4521,9 +4521,9 @@
           <t>Run</t>
         </is>
       </c>
-      <c r="C9" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Média</t>
         </is>
       </c>
       <c r="D9" s="8" t="inlineStr">
@@ -4578,9 +4578,9 @@
           <t>12h30</t>
         </is>
       </c>
-      <c r="B10" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
@@ -4618,14 +4618,14 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="J10" s="10" t="inlineStr">
+      <c r="J10" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="K10" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="K10" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
         </is>
       </c>
       <c r="L10" s="4" t="inlineStr">
@@ -4640,9 +4640,9 @@
           <t>13h00</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
@@ -4680,9 +4680,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="J11" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="J11" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
       <c r="K11" s="8" t="inlineStr">
@@ -4702,14 +4702,14 @@
           <t>13h30</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>Média</t>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
@@ -4717,34 +4717,34 @@
           <t>Run</t>
         </is>
       </c>
-      <c r="E12" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="F12" s="10" t="inlineStr">
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="G12" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="H12" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="I12" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="J12" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="G12" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="H12" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="I12" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="J12" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
         </is>
       </c>
       <c r="K12" s="8" t="inlineStr">
@@ -4779,9 +4779,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="E13" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="F13" s="8" t="inlineStr">
@@ -4789,14 +4789,14 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="G13" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="H13" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="I13" s="8" t="inlineStr">
@@ -4804,19 +4804,19 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="J13" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="K13" s="10" t="inlineStr">
+      <c r="J13" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="K13" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="L13" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="L13" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
         </is>
       </c>
     </row>
@@ -4826,9 +4826,9 @@
           <t>14h30</t>
         </is>
       </c>
-      <c r="B14" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
@@ -4846,39 +4846,39 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="F14" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="G14" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="H14" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="I14" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="J14" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="K14" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="L14" s="10" t="inlineStr">
+      <c r="F14" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
+        </is>
+      </c>
+      <c r="G14" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="H14" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="I14" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="J14" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="K14" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="L14" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
     </row>
@@ -4923,24 +4923,24 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="I15" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="J15" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="K15" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="L15" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="I15" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="J15" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="K15" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="L15" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
     </row>
@@ -5352,9 +5352,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="H22" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="H22" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="I22" s="10" t="inlineStr">
@@ -5414,9 +5414,9 @@
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="H23" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="H23" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
       <c r="I23" s="8" t="inlineStr">
@@ -5845,7 +5845,7 @@
     <row r="44">
       <c r="A44" s="21" t="inlineStr">
         <is>
-          <t>Règles : max 2h consécutives sur un même poste (hors Run de préparation du vendredi matin et Standiers fixes pendant les Awards, demandés explicitement) · un repas de 30 min le midi (fenêtre 11h30-14h) et le soir (fenêtre 18h30-21h) pour chacun·e, y compris Chris et Jeff, au moins 3 personnes en Off en même temps. Le samedi, les 2 Standiers fixes des Awards mangent ensemble à 19h30, remplacés par 2 personnes des Awards.</t>
+          <t>Règles : max 2h consécutives sur un même poste (hors Run de préparation du vendredi matin et Standiers fixes pendant les Awards, demandés explicitement) · un repas de 30 min le midi (fenêtre 11h30-14h) et le soir (fenêtre 18h30-21h) pour chacun·e, y compris Chris (Média le reste du temps) et Jeff, jamais seul : au moins 3 personnes en Off en même temps. Le samedi, les 2 Standiers fixes des Awards mangent ensemble à 19h30, remplacés par 2 personnes des Awards.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tout le monde finit à 20h tous les jours (clôture 19h30-20h, Awards tronqués à 20h)
</commit_message>
<xml_diff>
--- a/Planning_Stunfest2026_Indie.xlsx
+++ b/Planning_Stunfest2026_Indie.xlsx
@@ -552,7 +552,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K45"/>
+  <dimension ref="A1:K41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1835,49 +1835,49 @@
           <t>19h30</t>
         </is>
       </c>
-      <c r="B24" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C24" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D24" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E24" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F24" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G24" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H24" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I24" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J24" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="H24" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="I24" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="J24" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="K24" s="4" t="inlineStr">
@@ -1886,337 +1886,109 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="14" customHeight="1">
-      <c r="A25" s="3" t="inlineStr">
-        <is>
-          <t>20h00</t>
-        </is>
-      </c>
-      <c r="B25" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C25" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D25" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E25" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F25" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G25" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H25" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I25" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J25" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K25" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="14" customHeight="1">
-      <c r="A26" s="3" t="inlineStr">
-        <is>
-          <t>20h30</t>
-        </is>
-      </c>
-      <c r="B26" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C26" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D26" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E26" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F26" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G26" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H26" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I26" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J26" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K26" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="14" customHeight="1">
-      <c r="A27" s="3" t="inlineStr">
-        <is>
-          <t>21h00</t>
-        </is>
-      </c>
-      <c r="B27" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C27" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D27" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E27" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F27" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G27" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H27" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I27" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J27" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K27" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="14" customHeight="1">
-      <c r="A28" s="3" t="inlineStr">
-        <is>
-          <t>21h30</t>
-        </is>
-      </c>
-      <c r="B28" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C28" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D28" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E28" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F28" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G28" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H28" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I28" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J28" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K28" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+    <row r="27">
+      <c r="A27" s="11" t="inlineStr">
+        <is>
+          <t>Légende</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="12" t="inlineStr"/>
+      <c r="B28" s="13" t="inlineStr">
+        <is>
+          <t>Standiers = Back-up standiers Indie</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="14" t="inlineStr"/>
+      <c r="B29" s="13" t="inlineStr">
+        <is>
+          <t>Run = IC volant / Run (inclut le vote du public et le check des stands)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="15" t="inlineStr"/>
+      <c r="B30" s="13" t="inlineStr">
+        <is>
+          <t>Stand IC = Stand IC / Stunjam</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="11" t="inlineStr">
-        <is>
-          <t>Légende</t>
+      <c r="A31" s="16" t="inlineStr"/>
+      <c r="B31" s="13" t="inlineStr">
+        <is>
+          <t>Awards = Indie Awards (18h30-20h, samedi) ; 2 personnes fixes restent en Standiers</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="12" t="inlineStr"/>
+      <c r="A32" s="17" t="inlineStr"/>
       <c r="B32" s="13" t="inlineStr">
         <is>
-          <t>Standiers = Back-up standiers Indie</t>
+          <t>Média = Captation média (Chris, en continu les 3 jours)</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="14" t="inlineStr"/>
+      <c r="A33" s="18" t="inlineStr"/>
       <c r="B33" s="13" t="inlineStr">
         <is>
-          <t>Run = IC volant / Run (inclut le vote du public et le check des stands)</t>
+          <t>Briefing = Briefing d'équipe (vendredi 10h00-10h30)</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="15" t="inlineStr"/>
+      <c r="A34" s="19" t="inlineStr"/>
       <c r="B34" s="13" t="inlineStr">
         <is>
-          <t>Stand IC = Stand IC / Stunjam</t>
+          <t>Off (inclut les repas : 30 min le midi, 30 min le soir, répartis sur les fenêtres 11h30-14h et 18h30-20h)</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="16" t="inlineStr"/>
+      <c r="A35" s="20" t="inlineStr"/>
       <c r="B35" s="13" t="inlineStr">
         <is>
-          <t>Awards = Indie Awards (18h30-20h30, samedi) ; 2 personnes fixes restent en Standiers</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="17" t="inlineStr"/>
-      <c r="B36" s="13" t="inlineStr">
-        <is>
-          <t>Média = Captation média (Chris, en continu les 3 jours)</t>
+          <t>— = pas encore arrivé / absent ce jour-là</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="18" t="inlineStr"/>
-      <c r="B37" s="13" t="inlineStr">
-        <is>
-          <t>Briefing = Briefing d'équipe (vendredi 10h00-10h30)</t>
+      <c r="A37" s="21" t="inlineStr">
+        <is>
+          <t>FERMETURE DE LA ZONE INDÉ À 19h30 TOUS LES SOIRS (hors Awards du samedi). TOUT LE MONDE FINIT À 20h : rangement de 19h30 à 20h, tout le monde en Run.</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="19" t="inlineStr"/>
-      <c r="B38" s="13" t="inlineStr">
-        <is>
-          <t>Off (inclut les repas : 30 min le midi, 30 min le soir, répartis sur les fenêtres 11h30-14h et 18h30-21h)</t>
+      <c r="A38" s="21" t="inlineStr">
+        <is>
+          <t>Ouverture au public à 14h. Bénévoles présents dès 9h pour la préparation : tout le monde en Run de 9h à 14h.</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="20" t="inlineStr"/>
-      <c r="B39" s="13" t="inlineStr">
-        <is>
-          <t>— = pas encore arrivé / absent ce jour-là</t>
+      <c r="A39" s="21" t="inlineStr">
+        <is>
+          <t>Briefing d'équipe 10h00-10h30 (Jeff arrive à 11h).</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="21" t="inlineStr">
+        <is>
+          <t>Robin : présent uniquement samedi et dimanche. Jeff : présent les 3 jours de 11h à 20h, dans la rotation. Chris : captation Média en continu.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="21" t="inlineStr">
         <is>
-          <t>FERMETURE DE LA ZONE INDÉ À 19h30 TOUS LES SOIRS.</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="21" t="inlineStr">
-        <is>
-          <t>Ouverture au public à 14h. Bénévoles présents dès 9h pour la préparation : tout le monde en Run de 9h à 14h.</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="21" t="inlineStr">
-        <is>
-          <t>Briefing d'équipe 10h00-10h30 (Jeff arrive à 11h).</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="21" t="inlineStr">
-        <is>
-          <t>Robin : présent uniquement samedi et dimanche. Jeff : présent les 3 jours de 11h à 22h, dans la rotation (seul en Run après 19h30). Chris : captation Média en continu.</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="21" t="inlineStr">
-        <is>
-          <t>Règles : max 2h consécutives sur un même poste (hors Run de préparation du vendredi matin et Standiers fixes pendant les Awards, demandés explicitement) · un repas de 30 min le midi (fenêtre 11h30-14h) et le soir (fenêtre 18h30-21h) pour chacun·e, y compris Chris (Média le reste du temps) et Jeff, jamais seul : au moins 3 personnes en Off en même temps. Le samedi, les 2 Standiers fixes des Awards mangent ensemble à 19h30, remplacés par 2 personnes des Awards.</t>
+          <t>Règles : max 2h consécutives sur un même poste (hors Run de préparation du vendredi matin et Standiers fixes pendant les Awards, demandés explicitement) · un repas de 30 min le midi (fenêtre 11h30-14h) et le soir (fenêtre 18h30-20h) pour chacun·e, y compris Chris (Média le reste du temps) et Jeff, jamais seul : au moins 3 personnes en Off en même temps. Le samedi, les 2 Standiers fixes des Awards mangent ensemble à 19h30, remplacés par 2 personnes des Awards.</t>
         </is>
       </c>
     </row>
@@ -2234,7 +2006,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L45"/>
+  <dimension ref="A1:L41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -3591,34 +3363,34 @@
           <t>Awards</t>
         </is>
       </c>
-      <c r="G23" s="22" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="H23" s="22" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="I23" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="J23" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="K23" s="22" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="L23" s="22" t="inlineStr">
-        <is>
-          <t>Awards</t>
+      <c r="G23" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="H23" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="I23" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="J23" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="K23" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="L23" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
     </row>
@@ -3633,9 +3405,9 @@
           <t>Awards</t>
         </is>
       </c>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <t>Média</t>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="D24" s="22" t="inlineStr">
@@ -3653,388 +3425,140 @@
           <t>Awards</t>
         </is>
       </c>
-      <c r="G24" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="H24" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="I24" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="J24" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="K24" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="L24" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="14" customHeight="1">
-      <c r="A25" s="3" t="inlineStr">
-        <is>
-          <t>20h00</t>
-        </is>
-      </c>
-      <c r="B25" s="22" t="inlineStr">
+      <c r="G24" s="22" t="inlineStr">
         <is>
           <t>Awards</t>
         </is>
       </c>
-      <c r="C25" s="5" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="D25" s="22" t="inlineStr">
+      <c r="H24" s="22" t="inlineStr">
         <is>
           <t>Awards</t>
         </is>
       </c>
-      <c r="E25" s="22" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="F25" s="22" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="G25" s="22" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="H25" s="22" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="I25" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="J25" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="K25" s="22" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="L25" s="22" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="14" customHeight="1">
-      <c r="A26" s="3" t="inlineStr">
-        <is>
-          <t>20h30</t>
-        </is>
-      </c>
-      <c r="B26" s="22" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="C26" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="D26" s="22" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="E26" s="22" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="F26" s="22" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="G26" s="22" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="H26" s="22" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="I26" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="J26" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="K26" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="L26" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="14" customHeight="1">
-      <c r="A27" s="3" t="inlineStr">
-        <is>
-          <t>21h00</t>
-        </is>
-      </c>
-      <c r="B27" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C27" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D27" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E27" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F27" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G27" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H27" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I27" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J27" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K27" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L27" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="14" customHeight="1">
-      <c r="A28" s="3" t="inlineStr">
-        <is>
-          <t>21h30</t>
-        </is>
-      </c>
-      <c r="B28" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C28" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D28" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E28" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F28" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G28" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H28" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I28" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J28" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K28" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L28" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="I24" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="J24" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="K24" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="L24" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="11" t="inlineStr">
+        <is>
+          <t>Légende</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="12" t="inlineStr"/>
+      <c r="B28" s="13" t="inlineStr">
+        <is>
+          <t>Standiers = Back-up standiers Indie</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="14" t="inlineStr"/>
+      <c r="B29" s="13" t="inlineStr">
+        <is>
+          <t>Run = IC volant / Run (inclut le vote du public et le check des stands)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="15" t="inlineStr"/>
+      <c r="B30" s="13" t="inlineStr">
+        <is>
+          <t>Stand IC = Stand IC / Stunjam</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="11" t="inlineStr">
-        <is>
-          <t>Légende</t>
+      <c r="A31" s="16" t="inlineStr"/>
+      <c r="B31" s="13" t="inlineStr">
+        <is>
+          <t>Awards = Indie Awards (18h30-20h, samedi) ; 2 personnes fixes restent en Standiers</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="12" t="inlineStr"/>
+      <c r="A32" s="17" t="inlineStr"/>
       <c r="B32" s="13" t="inlineStr">
         <is>
-          <t>Standiers = Back-up standiers Indie</t>
+          <t>Média = Captation média (Chris, en continu les 3 jours)</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="14" t="inlineStr"/>
+      <c r="A33" s="18" t="inlineStr"/>
       <c r="B33" s="13" t="inlineStr">
         <is>
-          <t>Run = IC volant / Run (inclut le vote du public et le check des stands)</t>
+          <t>Briefing = Briefing d'équipe (vendredi 10h00-10h30)</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="15" t="inlineStr"/>
+      <c r="A34" s="19" t="inlineStr"/>
       <c r="B34" s="13" t="inlineStr">
         <is>
-          <t>Stand IC = Stand IC / Stunjam</t>
+          <t>Off (inclut les repas : 30 min le midi, 30 min le soir, répartis sur les fenêtres 11h30-14h et 18h30-20h)</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="16" t="inlineStr"/>
+      <c r="A35" s="20" t="inlineStr"/>
       <c r="B35" s="13" t="inlineStr">
         <is>
-          <t>Awards = Indie Awards (18h30-20h30, samedi) ; 2 personnes fixes restent en Standiers</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="17" t="inlineStr"/>
-      <c r="B36" s="13" t="inlineStr">
-        <is>
-          <t>Média = Captation média (Chris, en continu les 3 jours)</t>
+          <t>— = pas encore arrivé / absent ce jour-là</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="18" t="inlineStr"/>
-      <c r="B37" s="13" t="inlineStr">
-        <is>
-          <t>Briefing = Briefing d'équipe (vendredi 10h00-10h30)</t>
+      <c r="A37" s="21" t="inlineStr">
+        <is>
+          <t>FERMETURE DE LA ZONE INDÉ À 19h30 TOUS LES SOIRS (hors Awards du samedi). TOUT LE MONDE FINIT À 20h : rangement de 19h30 à 20h, tout le monde en Run.</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="19" t="inlineStr"/>
-      <c r="B38" s="13" t="inlineStr">
-        <is>
-          <t>Off (inclut les repas : 30 min le midi, 30 min le soir, répartis sur les fenêtres 11h30-14h et 18h30-21h)</t>
+      <c r="A38" s="21" t="inlineStr">
+        <is>
+          <t>Ouverture au public à 10h. Bénévoles présents dès 9h pour la préparation : tout le monde en Run de 9h à 10h.</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="20" t="inlineStr"/>
-      <c r="B39" s="13" t="inlineStr">
-        <is>
-          <t>— = pas encore arrivé / absent ce jour-là</t>
+      <c r="A39" s="21" t="inlineStr">
+        <is>
+          <t>Robin : présent uniquement samedi et dimanche. Jeff : présent les 3 jours de 11h à 20h, dans la rotation. Chris : captation Média en continu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="21" t="inlineStr">
+        <is>
+          <t>Indie Awards 18h30-20h : 2 personnes restent fixes sur l'accueil Standiers (sans rotation), le reste de l'équipe (y compris Jeff dès 18h30) est sur Awards ; Chris reste en Média. Tout le monde finit à 20h.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="21" t="inlineStr">
         <is>
-          <t>FERMETURE DE LA ZONE INDÉ À 19h30 TOUS LES SOIRS.</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="21" t="inlineStr">
-        <is>
-          <t>Ouverture au public à 10h. Bénévoles présents dès 9h pour la préparation : tout le monde en Run de 9h à 10h.</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="21" t="inlineStr">
-        <is>
-          <t>Robin : présent uniquement samedi et dimanche. Jeff : présent les 3 jours de 11h à 22h, dans la rotation (seul en Run après 19h30). Chris : captation Média en continu.</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="21" t="inlineStr">
-        <is>
-          <t>Indie Awards 18h30-20h30 : 2 personnes restent fixes sur l'accueil Standiers (sans rotation), le reste de l'équipe (y compris Jeff dès 18h30) est sur Awards ; Chris reste en Média. Le planning de l'équipe va jusqu'à 21h le samedi pour afficher les Awards en entier (Jeff jusqu'à 22h).</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="21" t="inlineStr">
-        <is>
-          <t>Règles : max 2h consécutives sur un même poste (hors Run de préparation du vendredi matin et Standiers fixes pendant les Awards, demandés explicitement) · un repas de 30 min le midi (fenêtre 11h30-14h) et le soir (fenêtre 18h30-21h) pour chacun·e, y compris Chris (Média le reste du temps) et Jeff, jamais seul : au moins 3 personnes en Off en même temps. Le samedi, les 2 Standiers fixes des Awards mangent ensemble à 19h30, remplacés par 2 personnes des Awards.</t>
+          <t>Règles : max 2h consécutives sur un même poste (hors Run de préparation du vendredi matin et Standiers fixes pendant les Awards, demandés explicitement) · un repas de 30 min le midi (fenêtre 11h30-14h) et le soir (fenêtre 18h30-20h) pour chacun·e, y compris Chris (Média le reste du temps) et Jeff, jamais seul : au moins 3 personnes en Off en même temps. Le samedi, les 2 Standiers fixes des Awards mangent ensemble à 19h30, remplacés par 2 personnes des Awards.</t>
         </is>
       </c>
     </row>
@@ -4052,7 +3576,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L44"/>
+  <dimension ref="A1:L40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -5446,54 +4970,54 @@
           <t>19h30</t>
         </is>
       </c>
-      <c r="B24" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C24" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D24" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E24" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F24" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G24" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H24" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I24" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J24" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K24" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="H24" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="I24" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="J24" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="K24" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="L24" s="4" t="inlineStr">
@@ -5502,350 +5026,102 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="14" customHeight="1">
-      <c r="A25" s="3" t="inlineStr">
-        <is>
-          <t>20h00</t>
-        </is>
-      </c>
-      <c r="B25" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C25" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D25" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E25" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F25" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G25" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H25" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I25" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J25" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K25" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L25" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="14" customHeight="1">
-      <c r="A26" s="3" t="inlineStr">
-        <is>
-          <t>20h30</t>
-        </is>
-      </c>
-      <c r="B26" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C26" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D26" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E26" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F26" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G26" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H26" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I26" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J26" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K26" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L26" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="14" customHeight="1">
-      <c r="A27" s="3" t="inlineStr">
-        <is>
-          <t>21h00</t>
-        </is>
-      </c>
-      <c r="B27" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C27" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D27" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E27" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F27" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G27" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H27" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I27" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J27" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K27" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L27" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="14" customHeight="1">
-      <c r="A28" s="3" t="inlineStr">
-        <is>
-          <t>21h30</t>
-        </is>
-      </c>
-      <c r="B28" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C28" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D28" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E28" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F28" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G28" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H28" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I28" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J28" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K28" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L28" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+    <row r="27">
+      <c r="A27" s="11" t="inlineStr">
+        <is>
+          <t>Légende</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="12" t="inlineStr"/>
+      <c r="B28" s="13" t="inlineStr">
+        <is>
+          <t>Standiers = Back-up standiers Indie</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="14" t="inlineStr"/>
+      <c r="B29" s="13" t="inlineStr">
+        <is>
+          <t>Run = IC volant / Run (inclut le vote du public et le check des stands)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="15" t="inlineStr"/>
+      <c r="B30" s="13" t="inlineStr">
+        <is>
+          <t>Stand IC = Stand IC / Stunjam</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="11" t="inlineStr">
-        <is>
-          <t>Légende</t>
+      <c r="A31" s="16" t="inlineStr"/>
+      <c r="B31" s="13" t="inlineStr">
+        <is>
+          <t>Awards = Indie Awards (18h30-20h, samedi) ; 2 personnes fixes restent en Standiers</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="12" t="inlineStr"/>
+      <c r="A32" s="17" t="inlineStr"/>
       <c r="B32" s="13" t="inlineStr">
         <is>
-          <t>Standiers = Back-up standiers Indie</t>
+          <t>Média = Captation média (Chris, en continu les 3 jours)</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="14" t="inlineStr"/>
+      <c r="A33" s="18" t="inlineStr"/>
       <c r="B33" s="13" t="inlineStr">
         <is>
-          <t>Run = IC volant / Run (inclut le vote du public et le check des stands)</t>
+          <t>Briefing = Briefing d'équipe (vendredi 10h00-10h30)</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="15" t="inlineStr"/>
+      <c r="A34" s="19" t="inlineStr"/>
       <c r="B34" s="13" t="inlineStr">
         <is>
-          <t>Stand IC = Stand IC / Stunjam</t>
+          <t>Off (inclut les repas : 30 min le midi, 30 min le soir, répartis sur les fenêtres 11h30-14h et 18h30-20h)</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="16" t="inlineStr"/>
+      <c r="A35" s="20" t="inlineStr"/>
       <c r="B35" s="13" t="inlineStr">
         <is>
-          <t>Awards = Indie Awards (18h30-20h30, samedi) ; 2 personnes fixes restent en Standiers</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="17" t="inlineStr"/>
-      <c r="B36" s="13" t="inlineStr">
-        <is>
-          <t>Média = Captation média (Chris, en continu les 3 jours)</t>
+          <t>— = pas encore arrivé / absent ce jour-là</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="18" t="inlineStr"/>
-      <c r="B37" s="13" t="inlineStr">
-        <is>
-          <t>Briefing = Briefing d'équipe (vendredi 10h00-10h30)</t>
+      <c r="A37" s="21" t="inlineStr">
+        <is>
+          <t>FERMETURE DE LA ZONE INDÉ À 19h30 TOUS LES SOIRS (hors Awards du samedi). TOUT LE MONDE FINIT À 20h : rangement de 19h30 à 20h, tout le monde en Run.</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="19" t="inlineStr"/>
-      <c r="B38" s="13" t="inlineStr">
-        <is>
-          <t>Off (inclut les repas : 30 min le midi, 30 min le soir, répartis sur les fenêtres 11h30-14h et 18h30-21h)</t>
+      <c r="A38" s="21" t="inlineStr">
+        <is>
+          <t>Ouverture au public à 10h. Bénévoles présents dès 9h pour la préparation : tout le monde en Run de 9h à 10h.</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="20" t="inlineStr"/>
-      <c r="B39" s="13" t="inlineStr">
-        <is>
-          <t>— = pas encore arrivé / absent ce jour-là</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="21" t="inlineStr">
-        <is>
-          <t>FERMETURE DE LA ZONE INDÉ À 19h30 TOUS LES SOIRS.</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="21" t="inlineStr">
-        <is>
-          <t>Ouverture au public à 10h. Bénévoles présents dès 9h pour la préparation : tout le monde en Run de 9h à 10h.</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="21" t="inlineStr">
-        <is>
-          <t>Robin : présent uniquement samedi et dimanche. Jeff : présent les 3 jours de 11h à 22h, dans la rotation (seul en Run après 19h30). Chris : captation Média en continu.</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="21" t="inlineStr">
-        <is>
-          <t>Règles : max 2h consécutives sur un même poste (hors Run de préparation du vendredi matin et Standiers fixes pendant les Awards, demandés explicitement) · un repas de 30 min le midi (fenêtre 11h30-14h) et le soir (fenêtre 18h30-21h) pour chacun·e, y compris Chris (Média le reste du temps) et Jeff, jamais seul : au moins 3 personnes en Off en même temps. Le samedi, les 2 Standiers fixes des Awards mangent ensemble à 19h30, remplacés par 2 personnes des Awards.</t>
+      <c r="A39" s="21" t="inlineStr">
+        <is>
+          <t>Robin : présent uniquement samedi et dimanche. Jeff : présent les 3 jours de 11h à 20h, dans la rotation. Chris : captation Média en continu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="21" t="inlineStr">
+        <is>
+          <t>Règles : max 2h consécutives sur un même poste (hors Run de préparation du vendredi matin et Standiers fixes pendant les Awards, demandés explicitement) · un repas de 30 min le midi (fenêtre 11h30-14h) et le soir (fenêtre 18h30-20h) pour chacun·e, y compris Chris (Média le reste du temps) et Jeff, jamais seul : au moins 3 personnes en Off en même temps. Le samedi, les 2 Standiers fixes des Awards mangent ensemble à 19h30, remplacés par 2 personnes des Awards.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Run: check des stands 1 jour
</commit_message>
<xml_diff>
--- a/Planning_Stunfest2026_Indie.xlsx
+++ b/Planning_Stunfest2026_Indie.xlsx
@@ -1905,7 +1905,7 @@
       <c r="A29" s="14" t="inlineStr"/>
       <c r="B29" s="13" t="inlineStr">
         <is>
-          <t>Run = IC volant / Run (inclut le vote du public et le check des stands)</t>
+          <t>Run = IC volant / Run (inclut le vote du public et le check des stands 1 jour)</t>
         </is>
       </c>
     </row>
@@ -3475,7 +3475,7 @@
       <c r="A29" s="14" t="inlineStr"/>
       <c r="B29" s="13" t="inlineStr">
         <is>
-          <t>Run = IC volant / Run (inclut le vote du public et le check des stands)</t>
+          <t>Run = IC volant / Run (inclut le vote du public et le check des stands 1 jour)</t>
         </is>
       </c>
     </row>
@@ -5045,7 +5045,7 @@
       <c r="A29" s="14" t="inlineStr"/>
       <c r="B29" s="13" t="inlineStr">
         <is>
-          <t>Run = IC volant / Run (inclut le vote du public et le check des stands)</t>
+          <t>Run = IC volant / Run (inclut le vote du public et le check des stands 1 jour)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Horaires de repas: le Run bascule en Standiers
</commit_message>
<xml_diff>
--- a/Planning_Stunfest2026_Indie.xlsx
+++ b/Planning_Stunfest2026_Indie.xlsx
@@ -1756,19 +1756,19 @@
           <t>Standiers</t>
         </is>
       </c>
-      <c r="I22" s="10" t="inlineStr">
+      <c r="I22" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="J22" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="K22" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="J22" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="K22" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
         </is>
       </c>
     </row>
@@ -1793,19 +1793,19 @@
           <t>Standiers</t>
         </is>
       </c>
-      <c r="E23" s="10" t="inlineStr">
+      <c r="E23" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="F23" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="G23" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="F23" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="G23" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
         </is>
       </c>
       <c r="H23" s="8" t="inlineStr">
@@ -2433,34 +2433,34 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="G8" s="10" t="inlineStr">
+      <c r="G8" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="H8" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="I8" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="J8" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="K8" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="H8" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="I8" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="J8" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="K8" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="L8" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="L8" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
     </row>
@@ -2470,9 +2470,9 @@
           <t>12h00</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
@@ -2480,9 +2480,9 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D9" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
       <c r="E9" s="9" t="inlineStr">
@@ -2495,9 +2495,9 @@
           <t>Standiers</t>
         </is>
       </c>
-      <c r="G9" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="G9" s="10" t="inlineStr">
+        <is>
+          <t>Stand IC</t>
         </is>
       </c>
       <c r="H9" s="8" t="inlineStr">
@@ -2505,9 +2505,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="I9" s="10" t="inlineStr">
-        <is>
-          <t>Stand IC</t>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="J9" s="8" t="inlineStr">
@@ -2532,9 +2532,9 @@
           <t>12h30</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
@@ -2577,14 +2577,14 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="K10" s="10" t="inlineStr">
+      <c r="K10" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="L10" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="L10" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
         </is>
       </c>
     </row>
@@ -2604,34 +2604,34 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D11" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="E11" s="10" t="inlineStr">
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="F11" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="F11" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
       <c r="G11" s="8" t="inlineStr">
         <is>
           <t>Off</t>
         </is>
       </c>
-      <c r="H11" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="I11" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="H11" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="I11" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
       <c r="J11" s="9" t="inlineStr">
@@ -2666,14 +2666,14 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="E12" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="E12" s="10" t="inlineStr">
+        <is>
+          <t>Stand IC</t>
         </is>
       </c>
       <c r="F12" s="8" t="inlineStr">
@@ -2696,9 +2696,9 @@
           <t>Standiers</t>
         </is>
       </c>
-      <c r="J12" s="10" t="inlineStr">
-        <is>
-          <t>Stand IC</t>
+      <c r="J12" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
       <c r="K12" s="8" t="inlineStr">
@@ -2718,9 +2718,9 @@
           <t>14h00</t>
         </is>
       </c>
-      <c r="B13" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>Stand IC</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
@@ -2748,9 +2748,9 @@
           <t>Run</t>
         </is>
       </c>
-      <c r="H13" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="H13" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="I13" s="8" t="inlineStr">
@@ -2768,9 +2768,9 @@
           <t>Standiers</t>
         </is>
       </c>
-      <c r="L13" s="10" t="inlineStr">
-        <is>
-          <t>Stand IC</t>
+      <c r="L13" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
     </row>
@@ -2780,9 +2780,9 @@
           <t>14h30</t>
         </is>
       </c>
-      <c r="B14" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
@@ -2800,34 +2800,34 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="F14" s="10" t="inlineStr">
+      <c r="F14" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="G14" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="I14" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="G14" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="H14" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="I14" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="J14" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="K14" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="J14" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="K14" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="L14" s="8" t="inlineStr">
@@ -2842,9 +2842,9 @@
           <t>15h00</t>
         </is>
       </c>
-      <c r="B15" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
@@ -2852,44 +2852,44 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D15" s="10" t="inlineStr">
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="H15" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="I15" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="J15" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="E15" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="F15" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="G15" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="H15" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="I15" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="J15" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="K15" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="K15" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="L15" s="4" t="inlineStr">
@@ -3028,19 +3028,19 @@
           <t>16h30</t>
         </is>
       </c>
-      <c r="B18" s="10" t="inlineStr">
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="D18" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="D18" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
@@ -4003,34 +4003,34 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="G8" s="10" t="inlineStr">
+      <c r="G8" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="H8" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="I8" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="J8" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="K8" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="H8" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="I8" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="J8" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="K8" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="L8" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="L8" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
     </row>
@@ -4040,9 +4040,9 @@
           <t>12h00</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
@@ -4050,9 +4050,9 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D9" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
       <c r="E9" s="9" t="inlineStr">
@@ -4065,9 +4065,9 @@
           <t>Standiers</t>
         </is>
       </c>
-      <c r="G9" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="G9" s="10" t="inlineStr">
+        <is>
+          <t>Stand IC</t>
         </is>
       </c>
       <c r="H9" s="8" t="inlineStr">
@@ -4075,9 +4075,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="I9" s="10" t="inlineStr">
-        <is>
-          <t>Stand IC</t>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="J9" s="8" t="inlineStr">
@@ -4102,9 +4102,9 @@
           <t>12h30</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
@@ -4147,14 +4147,14 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="K10" s="10" t="inlineStr">
+      <c r="K10" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="L10" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="L10" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
         </is>
       </c>
     </row>
@@ -4174,34 +4174,34 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D11" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="E11" s="10" t="inlineStr">
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="F11" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="F11" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
       <c r="G11" s="8" t="inlineStr">
         <is>
           <t>Off</t>
         </is>
       </c>
-      <c r="H11" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="I11" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="H11" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="I11" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
       <c r="J11" s="9" t="inlineStr">
@@ -4236,14 +4236,14 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="E12" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="E12" s="10" t="inlineStr">
+        <is>
+          <t>Stand IC</t>
         </is>
       </c>
       <c r="F12" s="8" t="inlineStr">
@@ -4266,9 +4266,9 @@
           <t>Standiers</t>
         </is>
       </c>
-      <c r="J12" s="10" t="inlineStr">
-        <is>
-          <t>Stand IC</t>
+      <c r="J12" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
       <c r="K12" s="8" t="inlineStr">
@@ -4288,9 +4288,9 @@
           <t>14h00</t>
         </is>
       </c>
-      <c r="B13" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>Stand IC</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
@@ -4318,9 +4318,9 @@
           <t>Run</t>
         </is>
       </c>
-      <c r="H13" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="H13" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="I13" s="8" t="inlineStr">
@@ -4338,9 +4338,9 @@
           <t>Standiers</t>
         </is>
       </c>
-      <c r="L13" s="10" t="inlineStr">
-        <is>
-          <t>Stand IC</t>
+      <c r="L13" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
     </row>
@@ -4350,9 +4350,9 @@
           <t>14h30</t>
         </is>
       </c>
-      <c r="B14" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
@@ -4370,34 +4370,34 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="F14" s="10" t="inlineStr">
+      <c r="F14" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="G14" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="I14" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="G14" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="H14" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="I14" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="J14" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="K14" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="J14" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="K14" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="L14" s="8" t="inlineStr">
@@ -4412,9 +4412,9 @@
           <t>15h00</t>
         </is>
       </c>
-      <c r="B15" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
@@ -4422,44 +4422,44 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D15" s="10" t="inlineStr">
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="H15" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="I15" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="J15" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="E15" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="F15" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="G15" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="H15" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="I15" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="J15" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="K15" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="K15" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="L15" s="4" t="inlineStr">
@@ -4598,19 +4598,19 @@
           <t>16h30</t>
         </is>
       </c>
-      <c r="B18" s="10" t="inlineStr">
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="D18" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="D18" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
@@ -4881,24 +4881,24 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="I22" s="10" t="inlineStr">
+      <c r="I22" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="J22" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="K22" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="J22" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="K22" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="L22" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="L22" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
     </row>
@@ -4923,14 +4923,14 @@
           <t>Standiers</t>
         </is>
       </c>
-      <c r="E23" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="F23" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="E23" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="F23" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
       <c r="G23" s="10" t="inlineStr">

</xml_diff>

<commit_message>
Installation (vendredi avant 14h) ; easter egg Chapeau pour Florent
</commit_message>
<xml_diff>
--- a/Planning_Stunfest2026_Indie.xlsx
+++ b/Planning_Stunfest2026_Indie.xlsx
@@ -64,7 +64,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -76,7 +76,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001565C0"/>
+        <fgColor rgb="006D4C41"/>
       </patternFill>
     </fill>
     <fill>
@@ -111,6 +111,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="001565C0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00B71C1C"/>
       </patternFill>
     </fill>
@@ -141,7 +146,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -173,18 +178,22 @@
     <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -552,7 +561,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K41"/>
+  <dimension ref="A1:K42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -640,7 +649,7 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>Run</t>
+          <t>Installation</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
@@ -650,37 +659,37 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>Run</t>
+          <t>Installation</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>Run</t>
+          <t>Installation</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>Run</t>
+          <t>Installation</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>Run</t>
+          <t>Installation</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>Run</t>
+          <t>Installation</t>
         </is>
       </c>
       <c r="I3" s="4" t="inlineStr">
         <is>
-          <t>Run</t>
+          <t>Installation</t>
         </is>
       </c>
       <c r="J3" s="4" t="inlineStr">
         <is>
-          <t>Run</t>
+          <t>Installation</t>
         </is>
       </c>
       <c r="K3" s="6" t="inlineStr">
@@ -697,7 +706,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Run</t>
+          <t>Installation</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
@@ -707,37 +716,37 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Run</t>
+          <t>Installation</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Run</t>
+          <t>Installation</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>Run</t>
+          <t>Installation</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>Run</t>
+          <t>Installation</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>Run</t>
+          <t>Installation</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>Run</t>
+          <t>Installation</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr">
         <is>
-          <t>Run</t>
+          <t>Installation</t>
         </is>
       </c>
       <c r="K4" s="6" t="inlineStr">
@@ -811,7 +820,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Run</t>
+          <t>Installation</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
@@ -821,37 +830,37 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Run</t>
+          <t>Installation</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Run</t>
+          <t>Installation</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>Run</t>
+          <t>Installation</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>Run</t>
+          <t>Installation</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>Run</t>
+          <t>Installation</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>Run</t>
+          <t>Installation</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
         <is>
-          <t>Run</t>
+          <t>Installation</t>
         </is>
       </c>
       <c r="K6" s="6" t="inlineStr">
@@ -868,7 +877,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Run</t>
+          <t>Installation</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
@@ -878,42 +887,42 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Run</t>
+          <t>Installation</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Run</t>
+          <t>Installation</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>Run</t>
+          <t>Installation</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>Run</t>
+          <t>Installation</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>Run</t>
+          <t>Installation</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>Run</t>
+          <t>Installation</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>Run</t>
+          <t>Installation</t>
         </is>
       </c>
       <c r="K7" s="4" t="inlineStr">
         <is>
-          <t>Run</t>
+          <t>Installation</t>
         </is>
       </c>
     </row>
@@ -950,27 +959,27 @@
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>Run</t>
+          <t>Installation</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>Run</t>
+          <t>Installation</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>Run</t>
+          <t>Installation</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
         <is>
-          <t>Run</t>
+          <t>Installation</t>
         </is>
       </c>
       <c r="K8" s="4" t="inlineStr">
         <is>
-          <t>Run</t>
+          <t>Installation</t>
         </is>
       </c>
     </row>
@@ -982,7 +991,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Run</t>
+          <t>Installation</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
@@ -992,42 +1001,42 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Run</t>
+          <t>Installation</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Run</t>
+          <t>Installation</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>Run</t>
+          <t>Installation</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>Run</t>
+          <t>Installation</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>Run</t>
+          <t>Installation</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>Run</t>
+          <t>Installation</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
         <is>
-          <t>Run</t>
+          <t>Installation</t>
         </is>
       </c>
       <c r="K9" s="4" t="inlineStr">
         <is>
-          <t>Run</t>
+          <t>Installation</t>
         </is>
       </c>
     </row>
@@ -1039,7 +1048,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Run</t>
+          <t>Installation</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
@@ -1049,17 +1058,17 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Run</t>
+          <t>Installation</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>Run</t>
+          <t>Installation</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>Run</t>
+          <t>Installation</t>
         </is>
       </c>
       <c r="G10" s="8" t="inlineStr">
@@ -1079,12 +1088,12 @@
       </c>
       <c r="J10" s="4" t="inlineStr">
         <is>
-          <t>Run</t>
+          <t>Installation</t>
         </is>
       </c>
       <c r="K10" s="4" t="inlineStr">
         <is>
-          <t>Run</t>
+          <t>Installation</t>
         </is>
       </c>
     </row>
@@ -1096,7 +1105,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Run</t>
+          <t>Installation</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
@@ -1106,42 +1115,42 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Run</t>
+          <t>Installation</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Run</t>
+          <t>Installation</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>Run</t>
+          <t>Installation</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>Run</t>
+          <t>Installation</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>Run</t>
+          <t>Installation</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>Run</t>
+          <t>Installation</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr">
         <is>
-          <t>Run</t>
+          <t>Installation</t>
         </is>
       </c>
       <c r="K11" s="4" t="inlineStr">
         <is>
-          <t>Run</t>
+          <t>Installation</t>
         </is>
       </c>
     </row>
@@ -1153,7 +1162,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Run</t>
+          <t>Installation</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
@@ -1163,32 +1172,32 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Run</t>
+          <t>Installation</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Run</t>
+          <t>Installation</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>Run</t>
+          <t>Installation</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>Run</t>
+          <t>Installation</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>Run</t>
+          <t>Installation</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>Run</t>
+          <t>Installation</t>
         </is>
       </c>
       <c r="J12" s="8" t="inlineStr">
@@ -1223,12 +1232,12 @@
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="E13" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="F13" s="4" t="inlineStr">
+      <c r="E13" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="F13" s="11" t="inlineStr">
         <is>
           <t>Run</t>
         </is>
@@ -1300,12 +1309,12 @@
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="I14" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="J14" s="4" t="inlineStr">
+      <c r="I14" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="J14" s="11" t="inlineStr">
         <is>
           <t>Run</t>
         </is>
@@ -1332,7 +1341,7 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="D15" s="11" t="inlineStr">
         <is>
           <t>Run</t>
         </is>
@@ -1347,7 +1356,7 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="G15" s="4" t="inlineStr">
+      <c r="G15" s="11" t="inlineStr">
         <is>
           <t>Run</t>
         </is>
@@ -1409,7 +1418,7 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="H16" s="4" t="inlineStr">
+      <c r="H16" s="11" t="inlineStr">
         <is>
           <t>Run</t>
         </is>
@@ -1424,7 +1433,7 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="K16" s="4" t="inlineStr">
+      <c r="K16" s="11" t="inlineStr">
         <is>
           <t>Run</t>
         </is>
@@ -1436,7 +1445,7 @@
           <t>16h00</t>
         </is>
       </c>
-      <c r="B17" s="4" t="inlineStr">
+      <c r="B17" s="11" t="inlineStr">
         <is>
           <t>Run</t>
         </is>
@@ -1446,7 +1455,7 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr">
+      <c r="D17" s="11" t="inlineStr">
         <is>
           <t>Run</t>
         </is>
@@ -1518,12 +1527,12 @@
           <t>Standiers</t>
         </is>
       </c>
-      <c r="G18" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="H18" s="4" t="inlineStr">
+      <c r="G18" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="H18" s="11" t="inlineStr">
         <is>
           <t>Run</t>
         </is>
@@ -1550,7 +1559,7 @@
           <t>17h00</t>
         </is>
       </c>
-      <c r="B19" s="4" t="inlineStr">
+      <c r="B19" s="11" t="inlineStr">
         <is>
           <t>Run</t>
         </is>
@@ -1595,7 +1604,7 @@
           <t>Standiers</t>
         </is>
       </c>
-      <c r="K19" s="4" t="inlineStr">
+      <c r="K19" s="11" t="inlineStr">
         <is>
           <t>Run</t>
         </is>
@@ -1622,12 +1631,12 @@
           <t>Standiers</t>
         </is>
       </c>
-      <c r="E20" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="F20" s="4" t="inlineStr">
+      <c r="E20" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="F20" s="11" t="inlineStr">
         <is>
           <t>Run</t>
         </is>
@@ -1699,12 +1708,12 @@
           <t>Standiers</t>
         </is>
       </c>
-      <c r="I21" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="J21" s="4" t="inlineStr">
+      <c r="I21" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="J21" s="11" t="inlineStr">
         <is>
           <t>Run</t>
         </is>
@@ -1835,7 +1844,7 @@
           <t>19h30</t>
         </is>
       </c>
-      <c r="B24" s="4" t="inlineStr">
+      <c r="B24" s="11" t="inlineStr">
         <is>
           <t>Run</t>
         </is>
@@ -1845,148 +1854,156 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D24" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="E24" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="F24" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="G24" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="H24" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="I24" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="J24" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="K24" s="4" t="inlineStr">
+      <c r="D24" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="E24" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="F24" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="G24" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="H24" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="I24" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="J24" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="K24" s="11" t="inlineStr">
         <is>
           <t>Run</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="11" t="inlineStr">
+      <c r="A27" s="12" t="inlineStr">
         <is>
           <t>Légende</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="12" t="inlineStr"/>
-      <c r="B28" s="13" t="inlineStr">
+      <c r="A28" s="13" t="inlineStr"/>
+      <c r="B28" s="14" t="inlineStr">
         <is>
           <t>Standiers = Back-up standiers Indie</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="14" t="inlineStr"/>
-      <c r="B29" s="13" t="inlineStr">
+      <c r="A29" s="15" t="inlineStr"/>
+      <c r="B29" s="14" t="inlineStr">
         <is>
           <t>Run = IC volant / Run (inclut le vote du public et le check des stands 1 jour)</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="15" t="inlineStr"/>
-      <c r="B30" s="13" t="inlineStr">
+      <c r="A30" s="16" t="inlineStr"/>
+      <c r="B30" s="14" t="inlineStr">
+        <is>
+          <t>Installation = montage du pôle avant l'ouverture du vendredi (9h-14h)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="17" t="inlineStr"/>
+      <c r="B31" s="14" t="inlineStr">
         <is>
           <t>Stand IC = Stand IC / Stunjam</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="16" t="inlineStr"/>
-      <c r="B31" s="13" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="18" t="inlineStr"/>
+      <c r="B32" s="14" t="inlineStr">
         <is>
           <t>Awards = Indie Awards (18h30-20h, samedi) ; 2 personnes fixes restent en Standiers</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="17" t="inlineStr"/>
-      <c r="B32" s="13" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="19" t="inlineStr"/>
+      <c r="B33" s="14" t="inlineStr">
         <is>
           <t>Média = Captation média (Chris, en continu les 3 jours)</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="18" t="inlineStr"/>
-      <c r="B33" s="13" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="20" t="inlineStr"/>
+      <c r="B34" s="14" t="inlineStr">
         <is>
           <t>Briefing = Briefing d'équipe (vendredi 10h00-10h30)</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="19" t="inlineStr"/>
-      <c r="B34" s="13" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="21" t="inlineStr"/>
+      <c r="B35" s="14" t="inlineStr">
         <is>
           <t>Off (inclut les repas : 30 min le midi, 30 min le soir, répartis sur les fenêtres 11h30-14h et 18h30-20h)</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="20" t="inlineStr"/>
-      <c r="B35" s="13" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="22" t="inlineStr"/>
+      <c r="B36" s="14" t="inlineStr">
         <is>
           <t>— = pas encore arrivé / absent ce jour-là</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="21" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="23" t="inlineStr">
         <is>
           <t>FERMETURE DE LA ZONE INDÉ À 19h30 TOUS LES SOIRS (hors Awards du samedi). TOUT LE MONDE FINIT À 20h : rangement de 19h30 à 20h, tout le monde en Run.</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="21" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="23" t="inlineStr">
         <is>
           <t>Ouverture au public à 14h. Bénévoles présents dès 9h pour la préparation : tout le monde en Run de 9h à 14h.</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="21" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="23" t="inlineStr">
         <is>
           <t>Briefing d'équipe 10h00-10h30 (Jeff arrive à 11h).</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="21" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="23" t="inlineStr">
         <is>
           <t>Robin : présent uniquement samedi et dimanche. Jeff : présent les 3 jours de 11h à 20h, dans la rotation. Chris : captation Média en continu.</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="21" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="23" t="inlineStr">
         <is>
           <t>Règles : max 2h consécutives sur un même poste (hors Run de préparation du vendredi matin et Standiers fixes pendant les Awards, demandés explicitement) · un repas de 30 min le midi (fenêtre 11h30-14h) et le soir (fenêtre 18h30-20h) pour chacun·e, y compris Chris (Média le reste du temps) et Jeff, jamais seul : au moins 3 personnes en Off en même temps. Le samedi, les 2 Standiers fixes des Awards mangent ensemble à 19h30, remplacés par 2 personnes des Awards.</t>
         </is>
@@ -2001,6 +2018,1584 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L42"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>STUNFEST 2026 — Planning bénévolat Indé — Samedi 24 octobre</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Horaire</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>François</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Chris</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Étienne</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Florent</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Arthur</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Mael</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Gabriel</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Lylou</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Suliac</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Robin</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>Jeff</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="14" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>9h00</t>
+        </is>
+      </c>
+      <c r="B3" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="D3" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="E3" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="F3" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="G3" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="H3" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="I3" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="J3" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="K3" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="L3" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="14" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>9h30</t>
+        </is>
+      </c>
+      <c r="B4" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="D4" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="E4" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="F4" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="G4" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="H4" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="I4" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="J4" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="K4" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="L4" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="14" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>10h00</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>Stand IC</t>
+        </is>
+      </c>
+      <c r="E5" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="F5" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="G5" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="H5" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="I5" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="J5" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="K5" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="L5" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="14" customHeight="1">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>10h30</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="G6" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="H6" s="10" t="inlineStr">
+        <is>
+          <t>Stand IC</t>
+        </is>
+      </c>
+      <c r="I6" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="J6" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="K6" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="L6" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="14" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>11h00</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>Stand IC</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="D7" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="G7" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="H7" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="I7" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="J7" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="K7" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="L7" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="14" customHeight="1">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>11h30</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="G8" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="H8" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="I8" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="J8" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="K8" s="10" t="inlineStr">
+        <is>
+          <t>Stand IC</t>
+        </is>
+      </c>
+      <c r="L8" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="14" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>12h00</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="E9" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="F9" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="G9" s="10" t="inlineStr">
+        <is>
+          <t>Stand IC</t>
+        </is>
+      </c>
+      <c r="H9" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="J9" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="K9" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="L9" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="14" customHeight="1">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>12h30</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="F10" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="H10" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="J10" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="K10" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="L10" s="10" t="inlineStr">
+        <is>
+          <t>Stand IC</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="14" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>13h00</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="F11" s="10" t="inlineStr">
+        <is>
+          <t>Stand IC</t>
+        </is>
+      </c>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="H11" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="I11" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="J11" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="K11" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="L11" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="14" customHeight="1">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>13h30</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="E12" s="10" t="inlineStr">
+        <is>
+          <t>Stand IC</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="G12" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="H12" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="I12" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="J12" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="K12" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="L12" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="14" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>14h00</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>Stand IC</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="G13" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="H13" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="I13" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="J13" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="K13" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="L13" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="14" customHeight="1">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>14h30</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="G14" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="H14" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="I14" s="10" t="inlineStr">
+        <is>
+          <t>Stand IC</t>
+        </is>
+      </c>
+      <c r="J14" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="K14" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="L14" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="14" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>15h00</t>
+        </is>
+      </c>
+      <c r="B15" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="H15" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="I15" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="J15" s="10" t="inlineStr">
+        <is>
+          <t>Stand IC</t>
+        </is>
+      </c>
+      <c r="K15" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="L15" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="14" customHeight="1">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>15h30</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="E16" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="F16" s="10" t="inlineStr">
+        <is>
+          <t>Stand IC</t>
+        </is>
+      </c>
+      <c r="G16" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="H16" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="I16" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="J16" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="K16" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="L16" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="14" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>16h00</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="G17" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="H17" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="I17" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="J17" s="10" t="inlineStr">
+        <is>
+          <t>Stand IC</t>
+        </is>
+      </c>
+      <c r="K17" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="L17" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="14" customHeight="1">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>16h30</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="D18" s="10" t="inlineStr">
+        <is>
+          <t>Stand IC</t>
+        </is>
+      </c>
+      <c r="E18" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="F18" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="G18" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="H18" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="J18" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="K18" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="L18" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="14" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>17h00</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="F19" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="G19" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="H19" s="10" t="inlineStr">
+        <is>
+          <t>Stand IC</t>
+        </is>
+      </c>
+      <c r="I19" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="J19" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="K19" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="L19" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="14" customHeight="1">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>17h30</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="D20" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="F20" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="G20" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="H20" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="I20" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="J20" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="K20" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="L20" s="10" t="inlineStr">
+        <is>
+          <t>Stand IC</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="14" customHeight="1">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>18h00</t>
+        </is>
+      </c>
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="E21" s="10" t="inlineStr">
+        <is>
+          <t>Stand IC</t>
+        </is>
+      </c>
+      <c r="F21" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="G21" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="H21" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="I21" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="J21" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="K21" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="L21" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="14" customHeight="1">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>18h30</t>
+        </is>
+      </c>
+      <c r="B22" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="F22" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="G22" s="24" t="inlineStr">
+        <is>
+          <t>Awards</t>
+        </is>
+      </c>
+      <c r="H22" s="24" t="inlineStr">
+        <is>
+          <t>Awards</t>
+        </is>
+      </c>
+      <c r="I22" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="J22" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="K22" s="24" t="inlineStr">
+        <is>
+          <t>Awards</t>
+        </is>
+      </c>
+      <c r="L22" s="24" t="inlineStr">
+        <is>
+          <t>Awards</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="14" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>19h00</t>
+        </is>
+      </c>
+      <c r="B23" s="24" t="inlineStr">
+        <is>
+          <t>Awards</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="D23" s="24" t="inlineStr">
+        <is>
+          <t>Awards</t>
+        </is>
+      </c>
+      <c r="E23" s="24" t="inlineStr">
+        <is>
+          <t>Awards</t>
+        </is>
+      </c>
+      <c r="F23" s="24" t="inlineStr">
+        <is>
+          <t>Awards</t>
+        </is>
+      </c>
+      <c r="G23" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="H23" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="I23" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="J23" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="K23" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="L23" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="14" customHeight="1">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>19h30</t>
+        </is>
+      </c>
+      <c r="B24" s="24" t="inlineStr">
+        <is>
+          <t>Awards</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="D24" s="24" t="inlineStr">
+        <is>
+          <t>Awards</t>
+        </is>
+      </c>
+      <c r="E24" s="24" t="inlineStr">
+        <is>
+          <t>Awards</t>
+        </is>
+      </c>
+      <c r="F24" s="24" t="inlineStr">
+        <is>
+          <t>Awards</t>
+        </is>
+      </c>
+      <c r="G24" s="24" t="inlineStr">
+        <is>
+          <t>Awards</t>
+        </is>
+      </c>
+      <c r="H24" s="24" t="inlineStr">
+        <is>
+          <t>Awards</t>
+        </is>
+      </c>
+      <c r="I24" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="J24" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="K24" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="L24" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="12" t="inlineStr">
+        <is>
+          <t>Légende</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="13" t="inlineStr"/>
+      <c r="B28" s="14" t="inlineStr">
+        <is>
+          <t>Standiers = Back-up standiers Indie</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="15" t="inlineStr"/>
+      <c r="B29" s="14" t="inlineStr">
+        <is>
+          <t>Run = IC volant / Run (inclut le vote du public et le check des stands 1 jour)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="16" t="inlineStr"/>
+      <c r="B30" s="14" t="inlineStr">
+        <is>
+          <t>Installation = montage du pôle avant l'ouverture du vendredi (9h-14h)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="17" t="inlineStr"/>
+      <c r="B31" s="14" t="inlineStr">
+        <is>
+          <t>Stand IC = Stand IC / Stunjam</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="18" t="inlineStr"/>
+      <c r="B32" s="14" t="inlineStr">
+        <is>
+          <t>Awards = Indie Awards (18h30-20h, samedi) ; 2 personnes fixes restent en Standiers</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="19" t="inlineStr"/>
+      <c r="B33" s="14" t="inlineStr">
+        <is>
+          <t>Média = Captation média (Chris, en continu les 3 jours)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="20" t="inlineStr"/>
+      <c r="B34" s="14" t="inlineStr">
+        <is>
+          <t>Briefing = Briefing d'équipe (vendredi 10h00-10h30)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="21" t="inlineStr"/>
+      <c r="B35" s="14" t="inlineStr">
+        <is>
+          <t>Off (inclut les repas : 30 min le midi, 30 min le soir, répartis sur les fenêtres 11h30-14h et 18h30-20h)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="22" t="inlineStr"/>
+      <c r="B36" s="14" t="inlineStr">
+        <is>
+          <t>— = pas encore arrivé / absent ce jour-là</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="23" t="inlineStr">
+        <is>
+          <t>FERMETURE DE LA ZONE INDÉ À 19h30 TOUS LES SOIRS (hors Awards du samedi). TOUT LE MONDE FINIT À 20h : rangement de 19h30 à 20h, tout le monde en Run.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="23" t="inlineStr">
+        <is>
+          <t>Ouverture au public à 10h. Bénévoles présents dès 9h pour la préparation : tout le monde en Run de 9h à 10h.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="23" t="inlineStr">
+        <is>
+          <t>Robin : présent uniquement samedi et dimanche. Jeff : présent les 3 jours de 11h à 20h, dans la rotation. Chris : captation Média en continu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="23" t="inlineStr">
+        <is>
+          <t>Indie Awards 18h30-20h : 2 personnes restent fixes sur l'accueil Standiers (sans rotation), le reste de l'équipe (y compris Jeff dès 18h30) est sur Awards ; Chris reste en Média. Tout le monde finit à 20h.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="23" t="inlineStr">
+        <is>
+          <t>Règles : max 2h consécutives sur un même poste (hors Run de préparation du vendredi matin et Standiers fixes pendant les Awards, demandés explicitement) · un repas de 30 min le midi (fenêtre 11h30-14h) et le soir (fenêtre 18h30-20h) pour chacun·e, y compris Chris (Média le reste du temps) et Jeff, jamais seul : au moins 3 personnes en Off en même temps. Le samedi, les 2 Standiers fixes des Awards mangent ensemble à 19h30, remplacés par 2 personnes des Awards.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:L1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2026,7 +3621,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>STUNFEST 2026 — Planning bénévolat Indé — Samedi 24 octobre</t>
+          <t>STUNFEST 2026 — Planning bénévolat Indé — Dimanche 25 octobre</t>
         </is>
       </c>
     </row>
@@ -2098,7 +3693,7 @@
           <t>9h00</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B3" s="11" t="inlineStr">
         <is>
           <t>Run</t>
         </is>
@@ -2108,42 +3703,42 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="G3" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="H3" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="I3" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="J3" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="K3" s="4" t="inlineStr">
+      <c r="D3" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="E3" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="F3" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="G3" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="H3" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="I3" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="J3" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="K3" s="11" t="inlineStr">
         <is>
           <t>Run</t>
         </is>
@@ -2160,7 +3755,7 @@
           <t>9h30</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" s="11" t="inlineStr">
         <is>
           <t>Run</t>
         </is>
@@ -2170,42 +3765,42 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="G4" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="H4" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="I4" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="J4" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="K4" s="4" t="inlineStr">
+      <c r="D4" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="E4" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="F4" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="G4" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="H4" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="I4" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="J4" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="K4" s="11" t="inlineStr">
         <is>
           <t>Run</t>
         </is>
@@ -2237,12 +3832,12 @@
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="E5" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="F5" s="11" t="inlineStr">
         <is>
           <t>Run</t>
         </is>
@@ -2319,12 +3914,12 @@
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="I6" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="J6" s="4" t="inlineStr">
+      <c r="I6" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="J6" s="11" t="inlineStr">
         <is>
           <t>Run</t>
         </is>
@@ -2356,7 +3951,7 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="D7" s="11" t="inlineStr">
         <is>
           <t>Run</t>
         </is>
@@ -2396,7 +3991,7 @@
           <t>Standiers</t>
         </is>
       </c>
-      <c r="L7" s="4" t="inlineStr">
+      <c r="L7" s="11" t="inlineStr">
         <is>
           <t>Run</t>
         </is>
@@ -2743,7 +4338,7 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="G13" s="4" t="inlineStr">
+      <c r="G13" s="11" t="inlineStr">
         <is>
           <t>Run</t>
         </is>
@@ -2768,7 +4363,7 @@
           <t>Standiers</t>
         </is>
       </c>
-      <c r="L13" s="4" t="inlineStr">
+      <c r="L13" s="11" t="inlineStr">
         <is>
           <t>Run</t>
         </is>
@@ -2810,7 +4405,7 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="H14" s="11" t="inlineStr">
         <is>
           <t>Run</t>
         </is>
@@ -2825,7 +4420,7 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="K14" s="4" t="inlineStr">
+      <c r="K14" s="11" t="inlineStr">
         <is>
           <t>Run</t>
         </is>
@@ -2842,7 +4437,7 @@
           <t>15h00</t>
         </is>
       </c>
-      <c r="B15" s="4" t="inlineStr">
+      <c r="B15" s="11" t="inlineStr">
         <is>
           <t>Run</t>
         </is>
@@ -2892,7 +4487,7 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="L15" s="4" t="inlineStr">
+      <c r="L15" s="11" t="inlineStr">
         <is>
           <t>Run</t>
         </is>
@@ -2929,12 +4524,12 @@
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="G16" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="H16" s="4" t="inlineStr">
+      <c r="G16" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="H16" s="11" t="inlineStr">
         <is>
           <t>Run</t>
         </is>
@@ -3011,12 +4606,12 @@
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="K17" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="L17" s="4" t="inlineStr">
+      <c r="K17" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="L17" s="11" t="inlineStr">
         <is>
           <t>Run</t>
         </is>
@@ -3043,12 +4638,12 @@
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="E18" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="F18" s="4" t="inlineStr">
+      <c r="E18" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="F18" s="11" t="inlineStr">
         <is>
           <t>Run</t>
         </is>
@@ -3125,12 +4720,12 @@
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="I19" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="J19" s="4" t="inlineStr">
+      <c r="I19" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="J19" s="11" t="inlineStr">
         <is>
           <t>Run</t>
         </is>
@@ -3152,7 +4747,7 @@
           <t>17h30</t>
         </is>
       </c>
-      <c r="B20" s="4" t="inlineStr">
+      <c r="B20" s="11" t="inlineStr">
         <is>
           <t>Run</t>
         </is>
@@ -3162,7 +4757,7 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D20" s="4" t="inlineStr">
+      <c r="D20" s="11" t="inlineStr">
         <is>
           <t>Run</t>
         </is>
@@ -3239,12 +4834,12 @@
           <t>Standiers</t>
         </is>
       </c>
-      <c r="G21" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="H21" s="4" t="inlineStr">
+      <c r="G21" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="H21" s="11" t="inlineStr">
         <is>
           <t>Run</t>
         </is>
@@ -3301,14 +4896,14 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="G22" s="22" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="H22" s="22" t="inlineStr">
-        <is>
-          <t>Awards</t>
+      <c r="G22" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="H22" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="I22" s="9" t="inlineStr">
@@ -3321,14 +4916,14 @@
           <t>Standiers</t>
         </is>
       </c>
-      <c r="K22" s="22" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="L22" s="22" t="inlineStr">
-        <is>
-          <t>Awards</t>
+      <c r="K22" s="10" t="inlineStr">
+        <is>
+          <t>Stand IC</t>
+        </is>
+      </c>
+      <c r="L22" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
     </row>
@@ -3338,39 +4933,39 @@
           <t>19h00</t>
         </is>
       </c>
-      <c r="B23" s="22" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="C23" s="5" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="D23" s="22" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="E23" s="22" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="F23" s="22" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="G23" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="H23" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="D23" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="E23" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="F23" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="G23" s="10" t="inlineStr">
+        <is>
+          <t>Stand IC</t>
+        </is>
+      </c>
+      <c r="H23" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
       <c r="I23" s="8" t="inlineStr">
@@ -3383,14 +4978,14 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="K23" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="L23" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="K23" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="L23" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
     </row>
@@ -3400,1726 +4995,164 @@
           <t>19h30</t>
         </is>
       </c>
-      <c r="B24" s="22" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="C24" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="D24" s="22" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="E24" s="22" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="F24" s="22" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="G24" s="22" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="H24" s="22" t="inlineStr">
-        <is>
-          <t>Awards</t>
-        </is>
-      </c>
-      <c r="I24" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="J24" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="K24" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="L24" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="B24" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="D24" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="E24" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="F24" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="G24" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="H24" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="I24" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="J24" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="K24" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="L24" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="11" t="inlineStr">
+      <c r="A27" s="12" t="inlineStr">
         <is>
           <t>Légende</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="12" t="inlineStr"/>
-      <c r="B28" s="13" t="inlineStr">
+      <c r="A28" s="13" t="inlineStr"/>
+      <c r="B28" s="14" t="inlineStr">
         <is>
           <t>Standiers = Back-up standiers Indie</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="14" t="inlineStr"/>
-      <c r="B29" s="13" t="inlineStr">
+      <c r="A29" s="15" t="inlineStr"/>
+      <c r="B29" s="14" t="inlineStr">
         <is>
           <t>Run = IC volant / Run (inclut le vote du public et le check des stands 1 jour)</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="15" t="inlineStr"/>
-      <c r="B30" s="13" t="inlineStr">
+      <c r="A30" s="16" t="inlineStr"/>
+      <c r="B30" s="14" t="inlineStr">
+        <is>
+          <t>Installation = montage du pôle avant l'ouverture du vendredi (9h-14h)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="17" t="inlineStr"/>
+      <c r="B31" s="14" t="inlineStr">
         <is>
           <t>Stand IC = Stand IC / Stunjam</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="16" t="inlineStr"/>
-      <c r="B31" s="13" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="18" t="inlineStr"/>
+      <c r="B32" s="14" t="inlineStr">
         <is>
           <t>Awards = Indie Awards (18h30-20h, samedi) ; 2 personnes fixes restent en Standiers</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="17" t="inlineStr"/>
-      <c r="B32" s="13" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="19" t="inlineStr"/>
+      <c r="B33" s="14" t="inlineStr">
         <is>
           <t>Média = Captation média (Chris, en continu les 3 jours)</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="18" t="inlineStr"/>
-      <c r="B33" s="13" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="20" t="inlineStr"/>
+      <c r="B34" s="14" t="inlineStr">
         <is>
           <t>Briefing = Briefing d'équipe (vendredi 10h00-10h30)</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="19" t="inlineStr"/>
-      <c r="B34" s="13" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="21" t="inlineStr"/>
+      <c r="B35" s="14" t="inlineStr">
         <is>
           <t>Off (inclut les repas : 30 min le midi, 30 min le soir, répartis sur les fenêtres 11h30-14h et 18h30-20h)</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="20" t="inlineStr"/>
-      <c r="B35" s="13" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="22" t="inlineStr"/>
+      <c r="B36" s="14" t="inlineStr">
         <is>
           <t>— = pas encore arrivé / absent ce jour-là</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="21" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="23" t="inlineStr">
         <is>
           <t>FERMETURE DE LA ZONE INDÉ À 19h30 TOUS LES SOIRS (hors Awards du samedi). TOUT LE MONDE FINIT À 20h : rangement de 19h30 à 20h, tout le monde en Run.</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="21" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="23" t="inlineStr">
         <is>
           <t>Ouverture au public à 10h. Bénévoles présents dès 9h pour la préparation : tout le monde en Run de 9h à 10h.</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="21" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="23" t="inlineStr">
         <is>
           <t>Robin : présent uniquement samedi et dimanche. Jeff : présent les 3 jours de 11h à 20h, dans la rotation. Chris : captation Média en continu.</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="21" t="inlineStr">
-        <is>
-          <t>Indie Awards 18h30-20h : 2 personnes restent fixes sur l'accueil Standiers (sans rotation), le reste de l'équipe (y compris Jeff dès 18h30) est sur Awards ; Chris reste en Média. Tout le monde finit à 20h.</t>
-        </is>
-      </c>
-    </row>
     <row r="41">
-      <c r="A41" s="21" t="inlineStr">
-        <is>
-          <t>Règles : max 2h consécutives sur un même poste (hors Run de préparation du vendredi matin et Standiers fixes pendant les Awards, demandés explicitement) · un repas de 30 min le midi (fenêtre 11h30-14h) et le soir (fenêtre 18h30-20h) pour chacun·e, y compris Chris (Média le reste du temps) et Jeff, jamais seul : au moins 3 personnes en Off en même temps. Le samedi, les 2 Standiers fixes des Awards mangent ensemble à 19h30, remplacés par 2 personnes des Awards.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:L1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:L40"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
-    <col width="11" customWidth="1" min="10" max="10"/>
-    <col width="11" customWidth="1" min="11" max="11"/>
-    <col width="11" customWidth="1" min="12" max="12"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>STUNFEST 2026 — Planning bénévolat Indé — Dimanche 25 octobre</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Horaire</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>François</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Chris</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Étienne</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Florent</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Arthur</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>Mael</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>Gabriel</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>Lylou</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>Suliac</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>Robin</t>
-        </is>
-      </c>
-      <c r="L2" s="2" t="inlineStr">
-        <is>
-          <t>Jeff</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="14" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>9h00</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="G3" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="H3" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="I3" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="J3" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="K3" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="L3" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="14" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>9h30</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="G4" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="H4" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="I4" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="J4" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="K4" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="L4" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="14" customHeight="1">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>10h00</t>
-        </is>
-      </c>
-      <c r="B5" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="D5" s="10" t="inlineStr">
-        <is>
-          <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="G5" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="H5" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="I5" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="J5" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="K5" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="L5" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="14" customHeight="1">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>10h30</t>
-        </is>
-      </c>
-      <c r="B6" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="D6" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="E6" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="F6" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="G6" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="H6" s="10" t="inlineStr">
-        <is>
-          <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="I6" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="J6" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="K6" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="L6" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="14" customHeight="1">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>11h00</t>
-        </is>
-      </c>
-      <c r="B7" s="10" t="inlineStr">
-        <is>
-          <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="E7" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="F7" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="G7" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="H7" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="I7" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="J7" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="K7" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="L7" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="14" customHeight="1">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>11h30</t>
-        </is>
-      </c>
-      <c r="B8" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="D8" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="E8" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="F8" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="G8" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="H8" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="I8" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="J8" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="K8" s="10" t="inlineStr">
-        <is>
-          <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="L8" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="14" customHeight="1">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>12h00</t>
-        </is>
-      </c>
-      <c r="B9" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="D9" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="E9" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="F9" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="G9" s="10" t="inlineStr">
-        <is>
-          <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="H9" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="I9" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="J9" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="K9" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="L9" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="14" customHeight="1">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>12h30</t>
-        </is>
-      </c>
-      <c r="B10" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="D10" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="E10" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="F10" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="G10" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="H10" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="I10" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="J10" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="K10" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="L10" s="10" t="inlineStr">
-        <is>
-          <t>Stand IC</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="14" customHeight="1">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>13h00</t>
-        </is>
-      </c>
-      <c r="B11" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="D11" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="E11" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="F11" s="10" t="inlineStr">
-        <is>
-          <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="G11" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="H11" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="I11" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="J11" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="K11" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="L11" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="14" customHeight="1">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>13h30</t>
-        </is>
-      </c>
-      <c r="B12" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="C12" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="D12" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="E12" s="10" t="inlineStr">
-        <is>
-          <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="F12" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="G12" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="H12" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="I12" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="J12" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="K12" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="L12" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="14" customHeight="1">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>14h00</t>
-        </is>
-      </c>
-      <c r="B13" s="10" t="inlineStr">
-        <is>
-          <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="D13" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="E13" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="F13" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="G13" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="H13" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="I13" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="J13" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="K13" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="L13" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="14" customHeight="1">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>14h30</t>
-        </is>
-      </c>
-      <c r="B14" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="D14" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="E14" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="F14" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="G14" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="H14" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="I14" s="10" t="inlineStr">
-        <is>
-          <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="J14" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="K14" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="L14" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="14" customHeight="1">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>15h00</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="D15" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="E15" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="F15" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="G15" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="H15" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="I15" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="J15" s="10" t="inlineStr">
-        <is>
-          <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="K15" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="L15" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="14" customHeight="1">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>15h30</t>
-        </is>
-      </c>
-      <c r="B16" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="D16" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="E16" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="F16" s="10" t="inlineStr">
-        <is>
-          <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="G16" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="H16" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="I16" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="J16" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="K16" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="L16" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="14" customHeight="1">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>16h00</t>
-        </is>
-      </c>
-      <c r="B17" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="D17" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="E17" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="F17" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="G17" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="H17" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="I17" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="J17" s="10" t="inlineStr">
-        <is>
-          <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="K17" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="L17" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="14" customHeight="1">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>16h30</t>
-        </is>
-      </c>
-      <c r="B18" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="D18" s="10" t="inlineStr">
-        <is>
-          <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="E18" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="F18" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="G18" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="H18" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="I18" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="J18" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="K18" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="L18" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="14" customHeight="1">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>17h00</t>
-        </is>
-      </c>
-      <c r="B19" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="D19" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="E19" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="F19" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="G19" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="H19" s="10" t="inlineStr">
-        <is>
-          <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="I19" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="J19" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="K19" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="L19" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="14" customHeight="1">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t>17h30</t>
-        </is>
-      </c>
-      <c r="B20" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="C20" s="5" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="D20" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="E20" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="F20" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="G20" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="H20" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="I20" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="J20" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="K20" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="L20" s="10" t="inlineStr">
-        <is>
-          <t>Stand IC</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="14" customHeight="1">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>18h00</t>
-        </is>
-      </c>
-      <c r="B21" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="C21" s="5" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="D21" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="E21" s="10" t="inlineStr">
-        <is>
-          <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="F21" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="G21" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="H21" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="I21" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="J21" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="K21" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="L21" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="14" customHeight="1">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t>18h30</t>
-        </is>
-      </c>
-      <c r="B22" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="D22" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="E22" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="F22" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="G22" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="H22" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="I22" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="J22" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="K22" s="10" t="inlineStr">
-        <is>
-          <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="L22" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="14" customHeight="1">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t>19h00</t>
-        </is>
-      </c>
-      <c r="B23" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="C23" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="D23" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="E23" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="F23" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="G23" s="10" t="inlineStr">
-        <is>
-          <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="H23" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="I23" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="J23" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="K23" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="L23" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="14" customHeight="1">
-      <c r="A24" s="3" t="inlineStr">
-        <is>
-          <t>19h30</t>
-        </is>
-      </c>
-      <c r="B24" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="D24" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="E24" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="F24" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="G24" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="H24" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="I24" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="J24" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="K24" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="L24" s="4" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="11" t="inlineStr">
-        <is>
-          <t>Légende</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="12" t="inlineStr"/>
-      <c r="B28" s="13" t="inlineStr">
-        <is>
-          <t>Standiers = Back-up standiers Indie</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="14" t="inlineStr"/>
-      <c r="B29" s="13" t="inlineStr">
-        <is>
-          <t>Run = IC volant / Run (inclut le vote du public et le check des stands 1 jour)</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="15" t="inlineStr"/>
-      <c r="B30" s="13" t="inlineStr">
-        <is>
-          <t>Stand IC = Stand IC / Stunjam</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="16" t="inlineStr"/>
-      <c r="B31" s="13" t="inlineStr">
-        <is>
-          <t>Awards = Indie Awards (18h30-20h, samedi) ; 2 personnes fixes restent en Standiers</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="17" t="inlineStr"/>
-      <c r="B32" s="13" t="inlineStr">
-        <is>
-          <t>Média = Captation média (Chris, en continu les 3 jours)</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="18" t="inlineStr"/>
-      <c r="B33" s="13" t="inlineStr">
-        <is>
-          <t>Briefing = Briefing d'équipe (vendredi 10h00-10h30)</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="19" t="inlineStr"/>
-      <c r="B34" s="13" t="inlineStr">
-        <is>
-          <t>Off (inclut les repas : 30 min le midi, 30 min le soir, répartis sur les fenêtres 11h30-14h et 18h30-20h)</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="20" t="inlineStr"/>
-      <c r="B35" s="13" t="inlineStr">
-        <is>
-          <t>— = pas encore arrivé / absent ce jour-là</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="21" t="inlineStr">
-        <is>
-          <t>FERMETURE DE LA ZONE INDÉ À 19h30 TOUS LES SOIRS (hors Awards du samedi). TOUT LE MONDE FINIT À 20h : rangement de 19h30 à 20h, tout le monde en Run.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="21" t="inlineStr">
-        <is>
-          <t>Ouverture au public à 10h. Bénévoles présents dès 9h pour la préparation : tout le monde en Run de 9h à 10h.</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="21" t="inlineStr">
-        <is>
-          <t>Robin : présent uniquement samedi et dimanche. Jeff : présent les 3 jours de 11h à 20h, dans la rotation. Chris : captation Média en continu.</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="21" t="inlineStr">
+      <c r="A41" s="23" t="inlineStr">
         <is>
           <t>Règles : max 2h consécutives sur un même poste (hors Run de préparation du vendredi matin et Standiers fixes pendant les Awards, demandés explicitement) · un repas de 30 min le midi (fenêtre 11h30-14h) et le soir (fenêtre 18h30-20h) pour chacun·e, y compris Chris (Média le reste du temps) et Jeff, jamais seul : au moins 3 personnes en Off en même temps. Le samedi, les 2 Standiers fixes des Awards mangent ensemble à 19h30, remplacés par 2 personnes des Awards.</t>
         </is>

</xml_diff>

<commit_message>
Planning: mission du Run (espaces indés, renfort freeplay), passages d'1h sur un poste, absences d'Arthur
</commit_message>
<xml_diff>
--- a/Planning_Stunfest2026_Indie.xlsx
+++ b/Planning_Stunfest2026_Indie.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vendredi 23 oct" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Samedi 24 oct" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dimanche 25 oct" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Vendredi 23 oct" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Samedi 24 oct" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Dimanche 25 oct" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1274,9 +1274,9 @@
           <t>14h30</t>
         </is>
       </c>
-      <c r="B14" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
@@ -1284,39 +1284,39 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D14" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="E14" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="F14" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="G14" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="H14" s="10" t="inlineStr">
+      <c r="D14" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="I14" s="11" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="J14" s="11" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="E14" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="F14" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="G14" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="H14" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="I14" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="J14" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="K14" s="8" t="inlineStr">
@@ -1331,54 +1331,54 @@
           <t>15h00</t>
         </is>
       </c>
-      <c r="B15" s="10" t="inlineStr">
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="G15" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="H15" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="D15" s="11" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="E15" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="F15" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="G15" s="11" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="H15" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="I15" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="J15" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="K15" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="I15" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="J15" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="K15" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
     </row>
@@ -1403,39 +1403,39 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="E16" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="F16" s="10" t="inlineStr">
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="G16" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="H16" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="G16" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="H16" s="11" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="I16" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="J16" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="K16" s="11" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="I16" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="J16" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="K16" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
     </row>
@@ -1445,9 +1445,9 @@
           <t>16h00</t>
         </is>
       </c>
-      <c r="B17" s="11" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="B17" s="10" t="inlineStr">
+        <is>
+          <t>Stand IC</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
@@ -1470,9 +1470,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="G17" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="G17" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="H17" s="8" t="inlineStr">
@@ -1480,19 +1480,19 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="I17" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="J17" s="10" t="inlineStr">
-        <is>
-          <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="K17" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="I17" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="J17" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="K17" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
     </row>
@@ -1502,9 +1502,9 @@
           <t>16h30</t>
         </is>
       </c>
-      <c r="B18" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>Stand IC</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
@@ -1512,19 +1512,19 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D18" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="E18" s="10" t="inlineStr">
-        <is>
-          <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="F18" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="D18" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="F18" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="G18" s="11" t="inlineStr">
@@ -1532,9 +1532,9 @@
           <t>Run</t>
         </is>
       </c>
-      <c r="H18" s="11" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="H18" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="I18" s="8" t="inlineStr">
@@ -1547,9 +1547,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="K18" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="K18" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
     </row>
@@ -1559,9 +1559,9 @@
           <t>17h00</t>
         </is>
       </c>
-      <c r="B19" s="11" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
@@ -1574,14 +1574,14 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="E19" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="F19" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="E19" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="F19" s="10" t="inlineStr">
+        <is>
+          <t>Stand IC</t>
         </is>
       </c>
       <c r="G19" s="8" t="inlineStr">
@@ -1589,19 +1589,19 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="H19" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="I19" s="10" t="inlineStr">
-        <is>
-          <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="J19" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="H19" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="I19" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="J19" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="K19" s="11" t="inlineStr">
@@ -1626,29 +1626,29 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D20" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="E20" s="11" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="F20" s="11" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="G20" s="10" t="inlineStr">
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="E20" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="F20" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="H20" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="G20" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="H20" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="I20" s="8" t="inlineStr">
@@ -1661,9 +1661,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="K20" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="K20" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
     </row>
@@ -1673,9 +1673,9 @@
           <t>18h00</t>
         </is>
       </c>
-      <c r="B21" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="B21" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
@@ -1688,9 +1688,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="E21" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="E21" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="F21" s="8" t="inlineStr">
@@ -1703,24 +1703,24 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="H21" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="I21" s="11" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="J21" s="11" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="K21" s="10" t="inlineStr">
+      <c r="H21" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="I21" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="J21" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
+        </is>
+      </c>
+      <c r="K21" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
     </row>
@@ -1770,14 +1770,14 @@
           <t>Standiers</t>
         </is>
       </c>
-      <c r="J22" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="K22" s="10" t="inlineStr">
+      <c r="J22" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
+        </is>
+      </c>
+      <c r="K22" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
     </row>
@@ -1802,9 +1802,9 @@
           <t>Standiers</t>
         </is>
       </c>
-      <c r="E23" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="E23" s="10" t="inlineStr">
+        <is>
+          <t>Stand IC</t>
         </is>
       </c>
       <c r="F23" s="9" t="inlineStr">
@@ -1812,9 +1812,9 @@
           <t>Standiers</t>
         </is>
       </c>
-      <c r="G23" s="10" t="inlineStr">
-        <is>
-          <t>Stand IC</t>
+      <c r="G23" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
       <c r="H23" s="8" t="inlineStr">
@@ -1914,7 +1914,7 @@
       <c r="A29" s="15" t="inlineStr"/>
       <c r="B29" s="14" t="inlineStr">
         <is>
-          <t>Run = IC volant / Run (inclut le vote du public et le check des stands 1 jour)</t>
+          <t>Run = IC volant / Run (espaces indés + renfort freeplay ; vérifie les postes de vote du public et l'installation des stands 1 jour)</t>
         </is>
       </c>
     </row>
@@ -2301,9 +2301,9 @@
           <t>10h30</t>
         </is>
       </c>
-      <c r="B6" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
@@ -2311,39 +2311,39 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="E6" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="F6" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="G6" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="H6" s="10" t="inlineStr">
+      <c r="D6" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="I6" s="11" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="J6" s="11" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="E6" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="F6" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="G6" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="H6" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="I6" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="J6" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="K6" s="8" t="inlineStr">
@@ -2363,44 +2363,44 @@
           <t>11h00</t>
         </is>
       </c>
-      <c r="B7" s="10" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="G7" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="H7" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="D7" s="11" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="E7" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="F7" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="G7" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="H7" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="I7" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="I7" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="J7" s="8" t="inlineStr">
@@ -2408,9 +2408,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="K7" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="K7" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="L7" s="11" t="inlineStr">
@@ -2455,9 +2455,9 @@
           <t>Standiers</t>
         </is>
       </c>
-      <c r="H8" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="H8" s="10" t="inlineStr">
+        <is>
+          <t>Stand IC</t>
         </is>
       </c>
       <c r="I8" s="9" t="inlineStr">
@@ -2470,9 +2470,9 @@
           <t>Standiers</t>
         </is>
       </c>
-      <c r="K8" s="10" t="inlineStr">
-        <is>
-          <t>Stand IC</t>
+      <c r="K8" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
       <c r="L8" s="9" t="inlineStr">
@@ -2487,9 +2487,9 @@
           <t>12h00</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>Stand IC</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
@@ -2502,19 +2502,19 @@
           <t>Standiers</t>
         </is>
       </c>
-      <c r="E9" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="F9" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="G9" s="10" t="inlineStr">
-        <is>
-          <t>Stand IC</t>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="H9" s="8" t="inlineStr">
@@ -2522,19 +2522,19 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="I9" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="J9" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="K9" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="I9" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="J9" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="K9" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
       <c r="L9" s="9" t="inlineStr">
@@ -2549,9 +2549,9 @@
           <t>12h30</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>Stand IC</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
@@ -2599,9 +2599,9 @@
           <t>Standiers</t>
         </is>
       </c>
-      <c r="L10" s="10" t="inlineStr">
-        <is>
-          <t>Stand IC</t>
+      <c r="L10" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
     </row>
@@ -2631,34 +2631,34 @@
           <t>Standiers</t>
         </is>
       </c>
-      <c r="F11" s="10" t="inlineStr">
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="G11" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="G11" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
       <c r="H11" s="9" t="inlineStr">
         <is>
           <t>Standiers</t>
         </is>
       </c>
-      <c r="I11" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="J11" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="K11" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="J11" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="K11" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
       <c r="L11" s="9" t="inlineStr">
@@ -2673,9 +2673,9 @@
           <t>13h30</t>
         </is>
       </c>
-      <c r="B12" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
@@ -2683,34 +2683,34 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="D12" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="E12" s="10" t="inlineStr">
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="E12" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="G12" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="F12" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="G12" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
       <c r="H12" s="9" t="inlineStr">
         <is>
           <t>Standiers</t>
         </is>
       </c>
-      <c r="I12" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="J12" s="9" t="inlineStr">
@@ -2735,54 +2735,54 @@
           <t>14h00</t>
         </is>
       </c>
-      <c r="B13" s="10" t="inlineStr">
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="G13" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="H13" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="I13" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="D13" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="E13" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="F13" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="G13" s="11" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="H13" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="I13" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="J13" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="K13" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="J13" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="K13" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="L13" s="11" t="inlineStr">
@@ -2817,19 +2817,19 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="F14" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="G14" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="H14" s="11" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="G14" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="H14" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="I14" s="10" t="inlineStr">
@@ -2837,19 +2837,19 @@
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="J14" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="K14" s="11" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="L14" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="J14" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="K14" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="L14" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
     </row>
@@ -2859,9 +2859,9 @@
           <t>15h00</t>
         </is>
       </c>
-      <c r="B15" s="11" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
@@ -2869,9 +2869,9 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D15" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="D15" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="E15" s="8" t="inlineStr">
@@ -2884,14 +2884,14 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="G15" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="H15" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="G15" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="H15" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="I15" s="8" t="inlineStr">
@@ -2899,19 +2899,19 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="J15" s="10" t="inlineStr">
+      <c r="J15" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="K15" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="K15" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="L15" s="11" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="L15" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
     </row>
@@ -2931,44 +2931,44 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D16" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="E16" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="F16" s="10" t="inlineStr">
+      <c r="D16" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="G16" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="H16" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="I16" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="J16" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="K16" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="G16" s="11" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="H16" s="11" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="I16" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="J16" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="K16" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
         </is>
       </c>
       <c r="L16" s="8" t="inlineStr">
@@ -2983,9 +2983,9 @@
           <t>16h00</t>
         </is>
       </c>
-      <c r="B17" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="B17" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
@@ -2998,14 +2998,14 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="E17" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="F17" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="E17" s="10" t="inlineStr">
+        <is>
+          <t>Stand IC</t>
+        </is>
+      </c>
+      <c r="F17" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="G17" s="8" t="inlineStr">
@@ -3023,19 +3023,19 @@
           <t>Standiers</t>
         </is>
       </c>
-      <c r="J17" s="10" t="inlineStr">
-        <is>
-          <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="K17" s="11" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="L17" s="11" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="J17" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="K17" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="L17" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
     </row>
@@ -3045,9 +3045,9 @@
           <t>16h30</t>
         </is>
       </c>
-      <c r="B18" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
@@ -3055,14 +3055,14 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D18" s="10" t="inlineStr">
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="E18" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="E18" s="11" t="inlineStr">
-        <is>
-          <t>Run</t>
         </is>
       </c>
       <c r="F18" s="11" t="inlineStr">
@@ -3117,9 +3117,9 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D19" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
       <c r="E19" s="8" t="inlineStr">
@@ -3132,29 +3132,29 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="G19" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="H19" s="10" t="inlineStr">
+      <c r="G19" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="H19" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="I19" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="J19" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="I19" s="11" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="J19" s="11" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="K19" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="K19" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="L19" s="8" t="inlineStr">
@@ -3169,9 +3169,9 @@
           <t>17h30</t>
         </is>
       </c>
-      <c r="B20" s="11" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="B20" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
@@ -3179,9 +3179,9 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D20" s="11" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="E20" s="8" t="inlineStr">
@@ -3194,14 +3194,14 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="G20" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="H20" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="G20" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="H20" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
       <c r="I20" s="8" t="inlineStr">
@@ -3209,19 +3209,19 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="J20" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="K20" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="L20" s="10" t="inlineStr">
+      <c r="J20" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
+        </is>
+      </c>
+      <c r="K20" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="L20" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
     </row>
@@ -3246,44 +3246,44 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="E21" s="10" t="inlineStr">
+      <c r="E21" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="G21" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="H21" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="I21" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="J21" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="K21" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="L21" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="F21" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="G21" s="11" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="H21" s="11" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="I21" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="J21" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="K21" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="L21" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
         </is>
       </c>
     </row>
@@ -3313,29 +3313,29 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="F22" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="G22" s="24" t="inlineStr">
+      <c r="F22" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="G22" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="H22" s="24" t="inlineStr">
         <is>
           <t>Awards</t>
         </is>
       </c>
-      <c r="H22" s="24" t="inlineStr">
+      <c r="I22" s="24" t="inlineStr">
         <is>
           <t>Awards</t>
         </is>
       </c>
-      <c r="I22" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="J22" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="J22" s="24" t="inlineStr">
+        <is>
+          <t>Awards</t>
         </is>
       </c>
       <c r="K22" s="24" t="inlineStr">
@@ -3343,9 +3343,9 @@
           <t>Awards</t>
         </is>
       </c>
-      <c r="L22" s="24" t="inlineStr">
-        <is>
-          <t>Awards</t>
+      <c r="L22" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
     </row>
@@ -3355,59 +3355,59 @@
           <t>19h00</t>
         </is>
       </c>
-      <c r="B23" s="24" t="inlineStr">
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="D23" s="24" t="inlineStr">
         <is>
           <t>Awards</t>
         </is>
       </c>
-      <c r="C23" s="5" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="D23" s="24" t="inlineStr">
+      <c r="E23" s="24" t="inlineStr">
         <is>
           <t>Awards</t>
         </is>
       </c>
-      <c r="E23" s="24" t="inlineStr">
+      <c r="F23" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="G23" s="24" t="inlineStr">
         <is>
           <t>Awards</t>
         </is>
       </c>
-      <c r="F23" s="24" t="inlineStr">
+      <c r="H23" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="I23" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="J23" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="K23" s="24" t="inlineStr">
         <is>
           <t>Awards</t>
         </is>
       </c>
-      <c r="G23" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="H23" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="I23" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="J23" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="K23" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="L23" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="L23" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
     </row>
@@ -3437,29 +3437,29 @@
           <t>Awards</t>
         </is>
       </c>
-      <c r="F24" s="24" t="inlineStr">
+      <c r="F24" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="G24" s="24" t="inlineStr">
         <is>
           <t>Awards</t>
         </is>
       </c>
-      <c r="G24" s="24" t="inlineStr">
+      <c r="H24" s="24" t="inlineStr">
         <is>
           <t>Awards</t>
         </is>
       </c>
-      <c r="H24" s="24" t="inlineStr">
+      <c r="I24" s="24" t="inlineStr">
         <is>
           <t>Awards</t>
         </is>
       </c>
-      <c r="I24" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="J24" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="J24" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="K24" s="8" t="inlineStr">
@@ -3467,9 +3467,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="L24" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="L24" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
     </row>
@@ -3492,7 +3492,7 @@
       <c r="A29" s="15" t="inlineStr"/>
       <c r="B29" s="14" t="inlineStr">
         <is>
-          <t>Run = IC volant / Run (inclut le vote du public et le check des stands 1 jour)</t>
+          <t>Run = IC volant / Run (espaces indés + renfort freeplay ; vérifie les postes de vote du public et l'installation des stands 1 jour)</t>
         </is>
       </c>
     </row>
@@ -3879,9 +3879,9 @@
           <t>10h30</t>
         </is>
       </c>
-      <c r="B6" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
@@ -3889,39 +3889,39 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="E6" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="F6" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="G6" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="H6" s="10" t="inlineStr">
+      <c r="D6" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="I6" s="11" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="J6" s="11" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="E6" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="F6" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="G6" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="H6" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="I6" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="J6" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="K6" s="8" t="inlineStr">
@@ -3941,44 +3941,44 @@
           <t>11h00</t>
         </is>
       </c>
-      <c r="B7" s="10" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="G7" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="H7" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="D7" s="11" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="E7" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="F7" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="G7" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="H7" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="I7" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="I7" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="J7" s="8" t="inlineStr">
@@ -3986,9 +3986,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="K7" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="K7" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="L7" s="11" t="inlineStr">
@@ -4023,19 +4023,19 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="F8" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="G8" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="H8" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="F8" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="G8" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="H8" s="10" t="inlineStr">
+        <is>
+          <t>Stand IC</t>
         </is>
       </c>
       <c r="I8" s="9" t="inlineStr">
@@ -4048,9 +4048,9 @@
           <t>Standiers</t>
         </is>
       </c>
-      <c r="K8" s="10" t="inlineStr">
-        <is>
-          <t>Stand IC</t>
+      <c r="K8" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
       <c r="L8" s="9" t="inlineStr">
@@ -4065,9 +4065,9 @@
           <t>12h00</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
@@ -4080,14 +4080,14 @@
           <t>Standiers</t>
         </is>
       </c>
-      <c r="E9" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="F9" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="G9" s="10" t="inlineStr">
@@ -4100,19 +4100,19 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="I9" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="J9" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="K9" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="I9" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="J9" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="K9" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
       <c r="L9" s="9" t="inlineStr">
@@ -4147,14 +4147,14 @@
           <t>Standiers</t>
         </is>
       </c>
-      <c r="F10" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="G10" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="G10" s="10" t="inlineStr">
+        <is>
+          <t>Stand IC</t>
         </is>
       </c>
       <c r="H10" s="8" t="inlineStr">
@@ -4177,9 +4177,9 @@
           <t>Standiers</t>
         </is>
       </c>
-      <c r="L10" s="10" t="inlineStr">
-        <is>
-          <t>Stand IC</t>
+      <c r="L10" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
     </row>
@@ -4189,9 +4189,9 @@
           <t>13h00</t>
         </is>
       </c>
-      <c r="B11" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
@@ -4209,34 +4209,34 @@
           <t>Standiers</t>
         </is>
       </c>
-      <c r="F11" s="10" t="inlineStr">
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="H11" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="J11" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="G11" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="H11" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="I11" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="J11" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="K11" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="K11" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
       <c r="L11" s="9" t="inlineStr">
@@ -4251,9 +4251,9 @@
           <t>13h30</t>
         </is>
       </c>
-      <c r="B12" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
@@ -4261,39 +4261,39 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="D12" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="E12" s="10" t="inlineStr">
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="E12" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="G12" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="H12" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="J12" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="F12" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="G12" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="H12" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="I12" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="J12" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
         </is>
       </c>
       <c r="K12" s="8" t="inlineStr">
@@ -4313,54 +4313,54 @@
           <t>14h00</t>
         </is>
       </c>
-      <c r="B13" s="10" t="inlineStr">
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="F13" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="G13" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="H13" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="I13" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="D13" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="E13" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="F13" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="G13" s="11" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="H13" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="I13" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
       <c r="J13" s="8" t="inlineStr">
         <is>
           <t>Off</t>
         </is>
       </c>
-      <c r="K13" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="K13" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="L13" s="11" t="inlineStr">
@@ -4395,19 +4395,19 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="F14" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="G14" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="H14" s="11" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="G14" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="H14" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="I14" s="10" t="inlineStr">
@@ -4415,19 +4415,19 @@
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="J14" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="K14" s="11" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="L14" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="J14" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="K14" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="L14" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
     </row>
@@ -4437,9 +4437,9 @@
           <t>15h00</t>
         </is>
       </c>
-      <c r="B15" s="11" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
@@ -4447,9 +4447,9 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D15" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="D15" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="E15" s="8" t="inlineStr">
@@ -4467,9 +4467,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="H15" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="H15" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="I15" s="8" t="inlineStr">
@@ -4477,19 +4477,19 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="J15" s="10" t="inlineStr">
+      <c r="J15" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="K15" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="K15" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="L15" s="11" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="L15" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
     </row>
@@ -4509,9 +4509,9 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D16" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="D16" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -4519,34 +4519,34 @@
           <t>Standiers</t>
         </is>
       </c>
-      <c r="F16" s="10" t="inlineStr">
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="G16" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="H16" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="I16" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="J16" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="K16" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="G16" s="11" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="H16" s="11" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="I16" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="J16" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="K16" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
         </is>
       </c>
       <c r="L16" s="8" t="inlineStr">
@@ -4561,9 +4561,9 @@
           <t>16h00</t>
         </is>
       </c>
-      <c r="B17" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="B17" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
@@ -4576,14 +4576,14 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="E17" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="F17" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="E17" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="F17" s="10" t="inlineStr">
+        <is>
+          <t>Stand IC</t>
         </is>
       </c>
       <c r="G17" s="8" t="inlineStr">
@@ -4596,24 +4596,24 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="I17" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="J17" s="10" t="inlineStr">
-        <is>
-          <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="K17" s="11" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="L17" s="11" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="I17" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="J17" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="K17" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="L17" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
     </row>
@@ -4623,9 +4623,9 @@
           <t>16h30</t>
         </is>
       </c>
-      <c r="B18" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
@@ -4633,21 +4633,21 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D18" s="10" t="inlineStr">
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="F18" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="E18" s="11" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="F18" s="11" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
       <c r="G18" s="8" t="inlineStr">
         <is>
           <t>Off</t>
@@ -4658,9 +4658,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="I18" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="I18" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="J18" s="8" t="inlineStr">
@@ -4695,9 +4695,9 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D19" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
       <c r="E19" s="8" t="inlineStr">
@@ -4710,34 +4710,34 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="G19" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="H19" s="10" t="inlineStr">
+      <c r="G19" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="H19" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="I19" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="J19" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="K19" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="L19" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="I19" s="11" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="J19" s="11" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="K19" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="L19" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
         </is>
       </c>
     </row>
@@ -4747,9 +4747,9 @@
           <t>17h30</t>
         </is>
       </c>
-      <c r="B20" s="11" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="B20" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
@@ -4757,9 +4757,9 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D20" s="11" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="E20" s="8" t="inlineStr">
@@ -4772,9 +4772,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="G20" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="G20" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
       <c r="H20" s="8" t="inlineStr">
@@ -4787,14 +4787,14 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="J20" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="K20" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="J20" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="K20" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="L20" s="10" t="inlineStr">
@@ -4809,9 +4809,9 @@
           <t>18h00</t>
         </is>
       </c>
-      <c r="B21" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="B21" s="10" t="inlineStr">
+        <is>
+          <t>Stand IC</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
@@ -4824,24 +4824,24 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="E21" s="10" t="inlineStr">
-        <is>
-          <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="F21" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="G21" s="11" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="H21" s="11" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="E21" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="F21" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="G21" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="H21" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="I21" s="8" t="inlineStr">
@@ -4901,9 +4901,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="H22" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="H22" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
       <c r="I22" s="9" t="inlineStr">
@@ -4911,9 +4911,9 @@
           <t>Standiers</t>
         </is>
       </c>
-      <c r="J22" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="J22" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="K22" s="10" t="inlineStr">
@@ -4963,9 +4963,9 @@
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="H23" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="H23" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="I23" s="8" t="inlineStr">
@@ -4973,9 +4973,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="J23" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="J23" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
       <c r="K23" s="8" t="inlineStr">
@@ -5070,7 +5070,7 @@
       <c r="A29" s="15" t="inlineStr"/>
       <c r="B29" s="14" t="inlineStr">
         <is>
-          <t>Run = IC volant / Run (inclut le vote du public et le check des stands 1 jour)</t>
+          <t>Run = IC volant / Run (espaces indés + renfort freeplay ; vérifie les postes de vote du public et l'installation des stands 1 jour)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Planning: Lylou absente le vendredi, planning rééquilibré; colonnes des absents masquées dans le planning complet
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Y6c29rnu3MpJHzcwavvYNk
</commit_message>
<xml_diff>
--- a/Planning_Stunfest2026_Indie.xlsx
+++ b/Planning_Stunfest2026_Indie.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Vendredi 23 oct" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Samedi 24 oct" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Dimanche 25 oct" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vendredi 23 oct" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Samedi 24 oct" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dimanche 25 oct" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -561,7 +561,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K42"/>
+  <dimension ref="A1:J42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -574,7 +574,6 @@
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="11" customWidth="1" min="9" max="9"/>
     <col width="11" customWidth="1" min="10" max="10"/>
-    <col width="11" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -627,15 +626,10 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Lylou</t>
+          <t>Suliac</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>Suliac</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>Jeff</t>
         </is>
@@ -687,12 +681,7 @@
           <t>Installation</t>
         </is>
       </c>
-      <c r="J3" s="4" t="inlineStr">
-        <is>
-          <t>Installation</t>
-        </is>
-      </c>
-      <c r="K3" s="6" t="inlineStr">
+      <c r="J3" s="6" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -744,12 +733,7 @@
           <t>Installation</t>
         </is>
       </c>
-      <c r="J4" s="4" t="inlineStr">
-        <is>
-          <t>Installation</t>
-        </is>
-      </c>
-      <c r="K4" s="6" t="inlineStr">
+      <c r="J4" s="6" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -801,12 +785,7 @@
           <t>Briefing</t>
         </is>
       </c>
-      <c r="J5" s="7" t="inlineStr">
-        <is>
-          <t>Briefing</t>
-        </is>
-      </c>
-      <c r="K5" s="6" t="inlineStr">
+      <c r="J5" s="6" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -858,12 +837,7 @@
           <t>Installation</t>
         </is>
       </c>
-      <c r="J6" s="4" t="inlineStr">
-        <is>
-          <t>Installation</t>
-        </is>
-      </c>
-      <c r="K6" s="6" t="inlineStr">
+      <c r="J6" s="6" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -920,11 +894,6 @@
           <t>Installation</t>
         </is>
       </c>
-      <c r="K7" s="4" t="inlineStr">
-        <is>
-          <t>Installation</t>
-        </is>
-      </c>
     </row>
     <row r="8" ht="14" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
@@ -952,9 +921,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="F8" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>Installation</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
@@ -973,11 +942,6 @@
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
-        <is>
-          <t>Installation</t>
-        </is>
-      </c>
-      <c r="K8" s="4" t="inlineStr">
         <is>
           <t>Installation</t>
         </is>
@@ -1034,11 +998,6 @@
           <t>Installation</t>
         </is>
       </c>
-      <c r="K9" s="4" t="inlineStr">
-        <is>
-          <t>Installation</t>
-        </is>
-      </c>
     </row>
     <row r="10" ht="14" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
@@ -1066,9 +1025,9 @@
           <t>Installation</t>
         </is>
       </c>
-      <c r="F10" s="4" t="inlineStr">
-        <is>
-          <t>Installation</t>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="G10" s="8" t="inlineStr">
@@ -1081,17 +1040,12 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="I10" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="I10" s="4" t="inlineStr">
+        <is>
+          <t>Installation</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
-        <is>
-          <t>Installation</t>
-        </is>
-      </c>
-      <c r="K10" s="4" t="inlineStr">
         <is>
           <t>Installation</t>
         </is>
@@ -1148,11 +1102,6 @@
           <t>Installation</t>
         </is>
       </c>
-      <c r="K11" s="4" t="inlineStr">
-        <is>
-          <t>Installation</t>
-        </is>
-      </c>
     </row>
     <row r="12" ht="14" customHeight="1">
       <c r="A12" s="3" t="inlineStr">
@@ -1195,17 +1144,12 @@
           <t>Installation</t>
         </is>
       </c>
-      <c r="I12" s="4" t="inlineStr">
-        <is>
-          <t>Installation</t>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="J12" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="K12" s="8" t="inlineStr">
         <is>
           <t>Off</t>
         </is>
@@ -1262,11 +1206,6 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="K13" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
     </row>
     <row r="14" ht="14" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
@@ -1319,11 +1258,6 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="K14" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
     </row>
     <row r="15" ht="14" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
@@ -1376,11 +1310,6 @@
           <t>Run</t>
         </is>
       </c>
-      <c r="K15" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
     </row>
     <row r="16" ht="14" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
@@ -1433,11 +1362,6 @@
           <t>Run</t>
         </is>
       </c>
-      <c r="K16" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
     </row>
     <row r="17" ht="14" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
@@ -1455,9 +1379,9 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D17" s="11" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="D17" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
       <c r="E17" s="8" t="inlineStr">
@@ -1475,9 +1399,9 @@
           <t>Run</t>
         </is>
       </c>
-      <c r="H17" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="H17" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="I17" s="8" t="inlineStr">
@@ -1488,11 +1412,6 @@
       <c r="J17" s="8" t="inlineStr">
         <is>
           <t>Off</t>
-        </is>
-      </c>
-      <c r="K17" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
         </is>
       </c>
     </row>
@@ -1512,9 +1431,9 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D18" s="11" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
       <c r="E18" s="8" t="inlineStr">
@@ -1532,9 +1451,9 @@
           <t>Run</t>
         </is>
       </c>
-      <c r="H18" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="H18" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="I18" s="8" t="inlineStr">
@@ -1545,11 +1464,6 @@
       <c r="J18" s="8" t="inlineStr">
         <is>
           <t>Off</t>
-        </is>
-      </c>
-      <c r="K18" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
         </is>
       </c>
     </row>
@@ -1559,9 +1473,9 @@
           <t>17h00</t>
         </is>
       </c>
-      <c r="B19" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="B19" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
@@ -1569,9 +1483,9 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D19" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="D19" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="E19" s="9" t="inlineStr">
@@ -1589,9 +1503,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="H19" s="11" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="H19" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="I19" s="8" t="inlineStr">
@@ -1602,11 +1516,6 @@
       <c r="J19" s="8" t="inlineStr">
         <is>
           <t>Off</t>
-        </is>
-      </c>
-      <c r="K19" s="11" t="inlineStr">
-        <is>
-          <t>Run</t>
         </is>
       </c>
     </row>
@@ -1616,9 +1525,9 @@
           <t>17h30</t>
         </is>
       </c>
-      <c r="B20" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
@@ -1626,9 +1535,9 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D20" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="D20" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -1646,9 +1555,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="H20" s="11" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="H20" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="I20" s="8" t="inlineStr">
@@ -1659,11 +1568,6 @@
       <c r="J20" s="8" t="inlineStr">
         <is>
           <t>Off</t>
-        </is>
-      </c>
-      <c r="K20" s="11" t="inlineStr">
-        <is>
-          <t>Run</t>
         </is>
       </c>
     </row>
@@ -1673,9 +1577,9 @@
           <t>18h00</t>
         </is>
       </c>
-      <c r="B21" s="11" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
@@ -1693,9 +1597,9 @@
           <t>Run</t>
         </is>
       </c>
-      <c r="F21" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="F21" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="G21" s="8" t="inlineStr">
@@ -1716,11 +1620,6 @@
       <c r="J21" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="K21" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
         </is>
       </c>
     </row>
@@ -1770,12 +1669,7 @@
           <t>Standiers</t>
         </is>
       </c>
-      <c r="J22" s="10" t="inlineStr">
-        <is>
-          <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="K22" s="9" t="inlineStr">
+      <c r="J22" s="9" t="inlineStr">
         <is>
           <t>Standiers</t>
         </is>
@@ -1832,11 +1726,6 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="K23" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
     </row>
     <row r="24" ht="14" customHeight="1">
       <c r="A24" s="3" t="inlineStr">
@@ -1885,11 +1774,6 @@
         </is>
       </c>
       <c r="J24" s="11" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="K24" s="11" t="inlineStr">
         <is>
           <t>Run</t>
         </is>
@@ -2011,7 +1895,7 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A1:J1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Planning: Arthur Off vendredi 18h-19h
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Y6c29rnu3MpJHzcwavvYNk
</commit_message>
<xml_diff>
--- a/Planning_Stunfest2026_Indie.xlsx
+++ b/Planning_Stunfest2026_Indie.xlsx
@@ -1577,9 +1577,9 @@
           <t>18h00</t>
         </is>
       </c>
-      <c r="B21" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="B21" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
@@ -1597,9 +1597,9 @@
           <t>Run</t>
         </is>
       </c>
-      <c r="F21" s="11" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="G21" s="8" t="inlineStr">

</xml_diff>

<commit_message>
Planning: vendredi, dîners décalés à 19h30, Run à 2 de 18h30 à 19h30
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Y6c29rnu3MpJHzcwavvYNk
</commit_message>
<xml_diff>
--- a/Planning_Stunfest2026_Indie.xlsx
+++ b/Planning_Stunfest2026_Indie.xlsx
@@ -1629,9 +1629,9 @@
           <t>18h30</t>
         </is>
       </c>
-      <c r="B22" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="B22" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
@@ -1644,9 +1644,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="E22" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="E22" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
       <c r="F22" s="8" t="inlineStr">
@@ -1659,9 +1659,9 @@
           <t>Off</t>
         </is>
       </c>
-      <c r="H22" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="H22" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
       <c r="I22" s="9" t="inlineStr">
@@ -1669,9 +1669,9 @@
           <t>Standiers</t>
         </is>
       </c>
-      <c r="J22" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
+      <c r="J22" s="10" t="inlineStr">
+        <is>
+          <t>Stand IC</t>
         </is>
       </c>
     </row>
@@ -1681,49 +1681,49 @@
           <t>19h00</t>
         </is>
       </c>
-      <c r="B23" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="C23" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="D23" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="E23" s="10" t="inlineStr">
+      <c r="B23" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="F23" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
+        </is>
+      </c>
+      <c r="G23" s="10" t="inlineStr">
         <is>
           <t>Stand IC</t>
         </is>
       </c>
-      <c r="F23" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="G23" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
       <c r="H23" s="8" t="inlineStr">
         <is>
           <t>Off</t>
         </is>
       </c>
-      <c r="I23" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="J23" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="I23" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="J23" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
         </is>
       </c>
     </row>
@@ -1733,49 +1733,49 @@
           <t>19h30</t>
         </is>
       </c>
-      <c r="B24" s="11" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="D24" s="11" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="E24" s="11" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="F24" s="11" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="G24" s="11" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="H24" s="11" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="I24" s="11" t="inlineStr">
-        <is>
-          <t>Run</t>
-        </is>
-      </c>
-      <c r="J24" s="11" t="inlineStr">
-        <is>
-          <t>Run</t>
+      <c r="B24" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="F24" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="G24" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="H24" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="I24" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="J24" s="8" t="inlineStr">
+        <is>
+          <t>Off</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Planning: vendredi 19h, tous les Off en Run
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Y6c29rnu3MpJHzcwavvYNk
</commit_message>
<xml_diff>
--- a/Planning_Stunfest2026_Indie.xlsx
+++ b/Planning_Stunfest2026_Indie.xlsx
@@ -1681,9 +1681,9 @@
           <t>19h00</t>
         </is>
       </c>
-      <c r="B23" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="B23" s="10" t="inlineStr">
+        <is>
+          <t>Stand IC</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
@@ -1691,29 +1691,29 @@
           <t>Média</t>
         </is>
       </c>
-      <c r="D23" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="E23" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
-        </is>
-      </c>
-      <c r="F23" s="9" t="inlineStr">
-        <is>
-          <t>Standiers</t>
-        </is>
-      </c>
-      <c r="G23" s="10" t="inlineStr">
-        <is>
-          <t>Stand IC</t>
-        </is>
-      </c>
-      <c r="H23" s="8" t="inlineStr">
-        <is>
-          <t>Off</t>
+      <c r="D23" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="E23" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="F23" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="G23" s="11" t="inlineStr">
+        <is>
+          <t>Run</t>
+        </is>
+      </c>
+      <c r="H23" s="9" t="inlineStr">
+        <is>
+          <t>Standiers</t>
         </is>
       </c>
       <c r="I23" s="11" t="inlineStr">

</xml_diff>